<commit_message>
Add B section attendees to Excel sheet
Appends 54 attendees from the B section screenshots, bringing the
total to 107 entries.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1348,6 +1348,920 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Deepa B</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Senior Customer Onboarding Advisor</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>JP BHATT</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ImpactQA</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Jin Seon Baek</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ERP Manager</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>H Mart Companies, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Stefan Baeuerle</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SVP | Chief Product Officer, SAP HAN…</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Paul Baines</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Programme Direct…</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>YORK TELECOM LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Staci Baker</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Divya Balaji</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Value Advisor</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Alvar Baldarrama</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Procurement Consultant</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>State of Louisiana</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Christie Balestra</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Senior Ind…</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SAP America Inc. (Hudson Yards)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Mithun Bangad</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sr Manager Finance IT</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>NRG Energy, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sahil Bansal</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Senior Manager</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Tricopp LLC dba CloudPaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Paul Baraniuk</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Global Solution…</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Florida Crystals Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Horacio Barbosa</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Proce…</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Techint Cia Tecnica Internacional SACI</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Devraj Bardhan</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SAP AI Leader</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>IBM United Kingdom Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Paul Barrett</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Senior Manager, Channel Sa…</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SPS Commerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Pam Barrowcliffe</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Product Marketing,…</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SAP Canada - Waterloo</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Alejandro Basigalup</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Jefe de infraestructura corporativo</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Grupo HZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Martin Bava</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>IT Bus…</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Techint Cia Tecnica Internacional SACI</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Lynn Bayer</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Procurement…</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Securian Financial Group, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Justin Beachnau</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Senior Account Exe…</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Benjamin Beberness</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Business Architect</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Proquire LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Chris Becker</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Director, Finance Tr…</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Cintas Corporation No. 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Andy Bell</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Head of Consulting</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>RESULTING LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Carrie Bennett</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SVP, Technology Deli…</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Ascentium Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Marissa Bennett</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Director, Global People Solutio…</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>James Benson</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Solutions Sales Executiv…</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Dan Berard</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>International Business Machines Corporation…</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Ethan Berceli</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Director of Sales Engineer</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Mediafly, Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Frederic Berg</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>VP SAP UI Technologies &amp; Mobile</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Nick Berg</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SVP Digital Platforms</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Softserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Elliot Berger</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Managing Partner, bp</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SAP UK Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Kerry Jo Berger</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase Bank, NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Catalina Bernal</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Seller Partner Manager</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SAP CANADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Kori Betsalel</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Senior accountant executive</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SAP CANADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Pallav Bhatnagar</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Sr. Director</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Nitin Bhide</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Regional Sales lead</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Incture LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Raja Sekhar Bhomadi</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Verizon Sourcing LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Marco Bickel</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Vice President IT Program Manage…</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Bayer AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Amos Biegun</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Vistex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Alex Birle</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Senior Sales Development</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Confido</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Justin Bisesi</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Business A…</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>The Davey Tree Expert Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Ron Blackburn</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EVP of Sales and GTM</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CloudPaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Eric Blondin</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Head of Business Te…</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SimpleFi Solutions, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Matt Blyth</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Vice President, Global Pr…</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Sanjeev Bode</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>HCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Arndt-Alexander Boehnert</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Global VP CAS…</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Beverley Den Boestert</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Director - Technology…</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>EY Global Services Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Kate Bollard</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Consulting Manager</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Collective Insights</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Raju Bolledla</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SAP Strategic Advisor</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>SAP Australia Pty Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Jackson Borges</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>RVP Finance &amp; Spend</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>SAP International Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Patrick Boruta</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Partner - Business Consultin…</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Grant Thornton</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Babs Bouchillon</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>NA Tradeshows and Event Manager</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Serrala</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Megan Boulter</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Director of Strategic…</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>The Silicon Partners Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Kailen Boumal</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Sr. Channel Manger</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ADP, Inc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add remaining B and start of C section attendees
Appends 55 more entries (rest of B section through start of C) for a
total of 162 attendees.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2262,6 +2262,929 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Art Boyd</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SVP Growth Partnerships</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Mirakl</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Joanne Bradford</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Procurement Data &amp; Capability Manager</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>JLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Holger Brammer</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>VP AI Ecosystem</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Stephen Brandes</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Confido</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Chuck Bratton</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Vice President of Solutions</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>FPT USA CORP</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Gary Braunscheidel</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Chief Technology Offic…</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Baillie Lumber Co Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Adam Breiterman</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Maryland &amp; Virginia Milk Producers Cooperati…</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Oscar Brennan</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Global Head of Growth for Digital Appli…</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Atos</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Renee Brewer</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Dir Finc Trans.</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Carrier World Headquarters</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Tim Brewer</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Technology Solutions Manager</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Corevist, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Paul Britter</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SAP Program Mana…</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Caterpillar Logistics, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Drew Brooks</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Chief Development Officer</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Ergon</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Jean-F. Brossard</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Partner &amp; VP Business Development</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>DBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Ian Brown</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Field Risk Management</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Jay Brown</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>ConsultingNetwork Business Solutions, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Jesse Brown</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Sr Success Executive</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>PartnerTap</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Michelle Brown</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Director Supply Chain</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Raytheon</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Mitch Brown</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>VP, North America</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Acuiti Labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Holger Bruchelt</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Eduardo Brunetti</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Value Advisor</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Franklin Bruno</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Solution Advisor Manager -…</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Renee Bruno</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>IT Manager</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Prime Conduit, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Ann Bryant</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Director - Financi…</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Old Dominion Freight Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Patricia Buchholz</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Gl…</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>SUSE Software Solutions Germany GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Sneha Budhwani</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Senior Solution Archi…</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Tricentis Americas, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Phillip Budidharma</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>IS Mana…</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Charlotte Pipe &amp; Foundry Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Mitchell Burkart</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Globalsource, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Alice Burrell</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Data Analytics Senior Manager</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>JLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Eamonn Burton</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Erin Buss</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Globalsource Information Technology III, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Tara Butler-Krgovic</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>VP, NA Experience and E…</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Shawn Byers</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>VP, Digital Product Marketing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>SAPinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>YOUNA CHOI</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Assistant Manager</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>sunjin</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Juan Carlos Caballero</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>System Developer M…</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>PAN AMERICAN GRAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Lisa Cabarcos</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>America's SAP Allianc…</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Ernst &amp; Young U.S. LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Bobby Cain</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SVP &amp; CIO - North America</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Schneider Electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Elidan Calvo</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>SAP Manager</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Align Technology Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Phil Cameron</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Growth Officer,…</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>SAP NEW ZEALAND LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Stefan Camp Angell</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SAP P…</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Komatsu-Mitsui Maquinarias Perú S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Mariano Caniglia</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Industry Executive Advis…</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>SAP Chile Limitada</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Amanda Cantu</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Schneider Electric USA, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Seila Carcavilla</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Innovation Manager</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>JLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Pat Carmody</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Senior Manag…</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sharp Electronics Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Tyler Carr</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Sr. Capabilities Manag…</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Matias Romero Carranza</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Sales Solution Director</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Sergio Carriero</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Bell Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Chrissy Caruso</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Client Engagement Manag…</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Mariana Carvajal</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Mobile App Lead</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Gabriele Casalena</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Aubay Italia S.p.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Sumner Case</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Syntax Systems Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Margarita Castillo</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Marketing Director</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Sam Castro</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Global Product Marketin…</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Vy Cates</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Director, HR PM/Produ…</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Phillips 66 Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>William Cdebaca</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Group operations Control…</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Fluor Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Donatella Cechet</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Chief Product Expert — Cloud ERP Fi…</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add more C section attendees
Appends 55 more entries from the C section screenshots, bringing the
total to 217 attendees.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C163"/>
+  <dimension ref="A1:C218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3185,6 +3185,933 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Anirban Chatterjee Chatterjee</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>SAP SLED Leader</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>IBM Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Karan Chauhan</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Life Sciences Solutions</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Cognizant</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Sanjay Chavan</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Head Enterpri…</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Mahindra &amp; Mahindra Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Abraham Cherian</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Director Security Govern…</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Kontoor Brands Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Venu Cherupillil</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Systems Engineer Sr Princi…</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>The Home Depot</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Jeff Cheung</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>SAP Platform Ow…</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Ionis Pharmaceuticals, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Michelle Chew</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Sr. Project Coordinator</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Marine Atlantic Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Taiseer Chirakkal</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr"/>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>International Business Machines Corporation…</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Karen Chirico</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Executive Director Enterprise Services</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Will Chisholm</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Southwest Airlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Flora Choi</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Director, ERP…</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>BioMarin Pharmaceutical, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>JongYun Choi</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>BSG partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Parinda Choksi</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>CIO - Enablement</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Ball Horticultural Co.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Sanjay Choubey</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Global Chief Digital an…</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Sylvamo Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Nicolas Christiaen Christiaen</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Dealside</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Saurabh Chug</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Solution Advisor</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Yoon Chung</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Solution Engineer Manager</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Precisely</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Douglas Ciolli</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>IT Principal Mana…</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Southern California Edison</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Tania Cirone-Fenyes</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Sr. Director Alliances</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>GyanSys, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Odércio Claro</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Klabin SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Greg Clausing</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Director SAP COE</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>The Andersons, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Zach Clement</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr"/>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>American Equity Investment Li fe Insurance C…</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Michael Cobler</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Sr. Account Executive</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Cognitus Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Tim Coffey</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Sr. AE</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Alinne Cogrossi</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Product Manager, ERP Procure to P…</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Arc'teryx</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Chad Cohen</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Client Engagement Manger</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Allan Colaco</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>ERP Transfor…</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>HellermannTyton Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Colin Cole</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>IT Director</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>JBS USA Food Company Holdings</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Clay Coleman</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Global Service Director, BPO</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Andrew Collins</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>SVP ERP Transformation</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>BP</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Kelli Collins</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>BlackJet Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Oisin Collins</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Mark Colosimo</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Director of Strategic Acc…</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>The Silicon Partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Tom Coltrain</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Enterprise Architect</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Dominion Energy, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Sean Comer</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Senior Project…</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>TAMKO Building Products LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Meena Confait</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Global Business &amp; Engagem…</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Alex Connor</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Senior Develo…</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Lantech.com Coöperatie U.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Adam Conrad</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Bus Proc Architect</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>McKesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Eileen Conway</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Global Head Strategic Partnerships</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Qualitest</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Julie Cooper</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Client Relationship Executive</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>BravoTECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Michael Coppola</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>VP, Finance &amp; Treasury</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Ashland Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Juan Correa</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Sharp Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Manoel Costa</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Demo Solutions Expert</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Sophie-Anne Cote</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Finance Director</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Barrette-Chapais</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Maryanne Coughlin</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Robert Coutu</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Sr. Accoun…</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>System Design Analysis (SDA) inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Julie Craig</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Spon…</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>SPARKS MARKETING (EMEA) LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Bill Cranston</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>SAP Sales Director</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Techwave</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Keith Creech</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Director, Enterprise Sales</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>SPS Commerce, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Philippe Cretier</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Head Finance and Spend Manage…</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Chris Crosby</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Founder | Managing Partner</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Adoptlab</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Ademar Crotti Junior</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Principal Technical Cons…</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>metaphacts GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Ken Crovetti</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Business Development Manager-…</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Miguel Cruz</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Gerente de Calidad</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Punta Cana</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Michael Cugliari</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Senior Account Exec…</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>The Silicon Partners Inc</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 10 missing C section attendees
Inserts entries between Cechet and Chatterjee that were previously
obscured by a notification banner. Includes Alexandra Charris (the
Softtek Renovation SAS row). Total now 227.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C218"/>
+  <dimension ref="A1:C228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3188,925 +3188,1095 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Anirban Chatterjee Chatterjee</t>
+          <t>Ekta Chadha</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>SAP SLED Leader</t>
+          <t>Head of Cloud Delivery,…</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>IBM Corporation</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Karan Chauhan</t>
+          <t>Joydeep Chakraborty</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Life Sciences Solutions</t>
+          <t>Head of ECS CAA…</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Cognizant</t>
+          <t>SAP LABS INDIA PVT. LTD.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Sanjay Chavan</t>
+          <t>Arun Chakravarthi</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Head Enterpri…</t>
+          <t>Enterprise Account M…</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra Limited</t>
+          <t>Kaar Technologies Inc</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Abraham Cherian</t>
+          <t>Kamlesh Chalasani</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Director Security Govern…</t>
+          <t>Vice President, Manufacturing</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Kontoor Brands Inc</t>
+          <t>Tech Mahindra</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Venu Cherupillil</t>
+          <t>Greg Chamberland</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Systems Engineer Sr Princi…</t>
+          <t>IT, Enterprise…</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>The Home Depot</t>
+          <t>Ocean Spray Cranberries, Inc.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Jeff Cheung</t>
+          <t>Chris Chamberlin</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>SAP Platform Ow…</t>
+          <t>Relationship Manager</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Ionis Pharmaceuticals, Inc.</t>
+          <t>Moody's Corporation</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Michelle Chew</t>
+          <t>Prasanna Chand</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Sr. Project Coordinator</t>
+          <t>Director - Enterprise Tech</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Marine Atlantic Inc.</t>
+          <t>Wayfair</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Taiseer Chirakkal</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr"/>
+          <t>Srinivasan Chandramohan</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>International Business Machines Corporation…</t>
+          <t>Cardinal Health Inc.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Karen Chirico</t>
+          <t>Matt Charleston</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Executive Director Enterprise Services</t>
+          <t>Sr Manager Fi…</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>Performance Food Group, Inc.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Will Chisholm</t>
+          <t>Alexandra Charris</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Business Relationsh…</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Southwest Airlines</t>
+          <t>Softtek Renovation SAS</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Flora Choi</t>
+          <t>Anirban Chatterjee Chatterjee</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Director, ERP…</t>
+          <t>SAP SLED Leader</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>BioMarin Pharmaceutical, Inc.</t>
+          <t>IBM Corporation</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>JongYun Choi</t>
+          <t>Karan Chauhan</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Life Sciences Solutions</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>BSG partners</t>
+          <t>Cognizant</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Parinda Choksi</t>
+          <t>Sanjay Chavan</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CIO - Enablement</t>
+          <t>Head Enterpri…</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ball Horticultural Co.</t>
+          <t>Mahindra &amp; Mahindra Limited</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Sanjay Choubey</t>
+          <t>Abraham Cherian</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Global Chief Digital an…</t>
+          <t>Director Security Govern…</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Sylvamo Corporation</t>
+          <t>Kontoor Brands Inc</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Nicolas Christiaen Christiaen</t>
+          <t>Venu Cherupillil</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Systems Engineer Sr Princi…</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Dealside</t>
+          <t>The Home Depot</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Saurabh Chug</t>
+          <t>Jeff Cheung</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Solution Advisor</t>
+          <t>SAP Platform Ow…</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Ionis Pharmaceuticals, Inc.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Yoon Chung</t>
+          <t>Michelle Chew</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Solution Engineer Manager</t>
+          <t>Sr. Project Coordinator</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Precisely</t>
+          <t>Marine Atlantic Inc.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Douglas Ciolli</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>IT Principal Mana…</t>
-        </is>
-      </c>
+          <t>Taiseer Chirakkal</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr"/>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Southern California Edison</t>
+          <t>International Business Machines Corporation…</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Tania Cirone-Fenyes</t>
+          <t>Karen Chirico</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Sr. Director Alliances</t>
+          <t>Executive Director Enterprise Services</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>GyanSys, Inc.</t>
+          <t>RTX</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Odércio Claro</t>
+          <t>Will Chisholm</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CIO</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Klabin SA</t>
+          <t>Southwest Airlines</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Greg Clausing</t>
+          <t>Flora Choi</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Director SAP COE</t>
+          <t>Director, ERP…</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>The Andersons, Inc.</t>
+          <t>BioMarin Pharmaceutical, Inc.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Zach Clement</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr"/>
+          <t>JongYun Choi</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>American Equity Investment Li fe Insurance C…</t>
+          <t>BSG partners</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Michael Cobler</t>
+          <t>Parinda Choksi</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Sr. Account Executive</t>
+          <t>CIO - Enablement</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Cognitus Ltd</t>
+          <t>Ball Horticultural Co.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Tim Coffey</t>
+          <t>Sanjay Choubey</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Sr. AE</t>
+          <t>Global Chief Digital an…</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Sylvamo Corporation</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Alinne Cogrossi</t>
+          <t>Nicolas Christiaen Christiaen</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Product Manager, ERP Procure to P…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Arc'teryx</t>
+          <t>Dealside</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Chad Cohen</t>
+          <t>Saurabh Chug</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Client Engagement Manger</t>
+          <t>Solution Advisor</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Veritas Prime, LLC</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Allan Colaco</t>
+          <t>Yoon Chung</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>ERP Transfor…</t>
+          <t>Solution Engineer Manager</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>HellermannTyton Corporation</t>
+          <t>Precisely</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Colin Cole</t>
+          <t>Douglas Ciolli</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>IT Principal Mana…</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>JBS USA Food Company Holdings</t>
+          <t>Southern California Edison</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Clay Coleman</t>
+          <t>Tania Cirone-Fenyes</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Global Service Director, BPO</t>
+          <t>Sr. Director Alliances</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Wipro Limited</t>
+          <t>GyanSys, Inc.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Andrew Collins</t>
+          <t>Odércio Claro</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>SVP ERP Transformation</t>
+          <t>CIO</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>Klabin SA</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Kelli Collins</t>
+          <t>Greg Clausing</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Director SAP COE</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>BlackJet Marketing</t>
+          <t>The Andersons, Inc.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Oisin Collins</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
+          <t>Zach Clement</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr"/>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>American Equity Investment Li fe Insurance C…</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Mark Colosimo</t>
+          <t>Michael Cobler</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Director of Strategic Acc…</t>
+          <t>Sr. Account Executive</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>The Silicon Partners</t>
+          <t>Cognitus Ltd</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Tom Coltrain</t>
+          <t>Tim Coffey</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Enterprise Architect</t>
+          <t>Sr. AE</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Dominion Energy, Inc.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Sean Comer</t>
+          <t>Alinne Cogrossi</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Senior Project…</t>
+          <t>Product Manager, ERP Procure to P…</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>TAMKO Building Products LLC</t>
+          <t>Arc'teryx</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Meena Confait</t>
+          <t>Chad Cohen</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Global Business &amp; Engagem…</t>
+          <t>Client Engagement Manger</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>Veritas Prime, LLC</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Alex Connor</t>
+          <t>Allan Colaco</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Senior Develo…</t>
+          <t>ERP Transfor…</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Lantech.com Coöperatie U.A.</t>
+          <t>HellermannTyton Corporation</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Adam Conrad</t>
+          <t>Colin Cole</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Bus Proc Architect</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>McKesson</t>
+          <t>JBS USA Food Company Holdings</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Eileen Conway</t>
+          <t>Clay Coleman</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Global Head Strategic Partnerships</t>
+          <t>Global Service Director, BPO</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Qualitest</t>
+          <t>Wipro Limited</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Julie Cooper</t>
+          <t>Andrew Collins</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Client Relationship Executive</t>
+          <t>SVP ERP Transformation</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>BravoTECH</t>
+          <t>BP</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Michael Coppola</t>
+          <t>Kelli Collins</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>VP, Finance &amp; Treasury</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Ashland Inc.</t>
+          <t>BlackJet Marketing</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Juan Correa</t>
+          <t>Oisin Collins</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Employee</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Sharp Corporation</t>
+          <t>Deloitte</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Manoel Costa</t>
+          <t>Mark Colosimo</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Demo Solutions Expert</t>
+          <t>Director of Strategic Acc…</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>SAP Brasil Ltda.</t>
+          <t>The Silicon Partners</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Sophie-Anne Cote</t>
+          <t>Tom Coltrain</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Finance Director</t>
+          <t>Enterprise Architect</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Barrette-Chapais</t>
+          <t>Dominion Energy, Inc.</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Maryanne Coughlin</t>
+          <t>Sean Comer</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Senior Project…</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>TAMKO Building Products LLC</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Robert Coutu</t>
+          <t>Meena Confait</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Sr. Accoun…</t>
+          <t>Global Business &amp; Engagem…</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>System Design Analysis (SDA) inc.</t>
+          <t>SAP MENA LLC</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Julie Craig</t>
+          <t>Alex Connor</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Spon…</t>
+          <t>Senior Develo…</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>SPARKS MARKETING (EMEA) LIMITED</t>
+          <t>Lantech.com Coöperatie U.A.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Bill Cranston</t>
+          <t>Adam Conrad</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>SAP Sales Director</t>
+          <t>Bus Proc Architect</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Techwave</t>
+          <t>McKesson</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Keith Creech</t>
+          <t>Eileen Conway</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Director, Enterprise Sales</t>
+          <t>Global Head Strategic Partnerships</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>SPS Commerce, Inc.</t>
+          <t>Qualitest</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Philippe Cretier</t>
+          <t>Julie Cooper</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Head Finance and Spend Manage…</t>
+          <t>Client Relationship Executive</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>BravoTECH</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Chris Crosby</t>
+          <t>Michael Coppola</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Founder | Managing Partner</t>
+          <t>VP, Finance &amp; Treasury</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Adoptlab</t>
+          <t>Ashland Inc.</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Ademar Crotti Junior</t>
+          <t>Juan Correa</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Principal Technical Cons…</t>
+          <t>Employee</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>metaphacts GmbH</t>
+          <t>Sharp Corporation</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Ken Crovetti</t>
+          <t>Manoel Costa</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Business Development Manager-…</t>
+          <t>Demo Solutions Expert</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Vertex, Inc.</t>
+          <t>SAP Brasil Ltda.</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Miguel Cruz</t>
+          <t>Sophie-Anne Cote</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Gerente de Calidad</t>
+          <t>Finance Director</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Punta Cana</t>
+          <t>Barrette-Chapais</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
+          <t>Maryanne Coughlin</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Robert Coutu</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Sr. Accoun…</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>System Design Analysis (SDA) inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Julie Craig</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Spon…</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>SPARKS MARKETING (EMEA) LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Bill Cranston</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>SAP Sales Director</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Techwave</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Keith Creech</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Director, Enterprise Sales</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>SPS Commerce, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Philippe Cretier</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Head Finance and Spend Manage…</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Chris Crosby</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Founder | Managing Partner</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Adoptlab</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Ademar Crotti Junior</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Principal Technical Cons…</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>metaphacts GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Ken Crovetti</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Business Development Manager-…</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Miguel Cruz</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Gerente de Calidad</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Punta Cana</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
           <t>Michael Cugliari</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
+      <c r="B228" t="inlineStr">
         <is>
           <t>Senior Account Exec…</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr">
+      <c r="C228" t="inlineStr">
         <is>
           <t>The Silicon Partners Inc</t>
         </is>

</xml_diff>

<commit_message>
Add W, Y, Z and Asian-character section attendees
Appends 53 entries from the W (Christy Weaver onward), Y, Z, 縣, 阿,
and 青 sections. Note there is a gap from D through V that hasn't
been provided yet. Total now 280.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C228"/>
+  <dimension ref="A1:C281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4282,6 +4282,903 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Christy Weaver</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Global Demand Generation Man…</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Mike Weaver</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Senior I…</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>True Commerce Inc. TrueCommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Chris Webster</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>SVP IT Strategy &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Ahold Delhaize</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Matt Webster</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Director of…</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Gardner White Furniture Co., Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Patrick Weil</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>IT Director</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Metrie Canada Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Sarah Weiler</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Manager, Busine…</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Ball Horticultural Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Adam Werner</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>VP, Corporate Technology</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Crocs, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Maddie Werner</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Director of Delivery Solutions</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Robra IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Katherine West</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>CX Account Executive</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Anja Wettling</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>anuwo GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Charleen Wetzstein</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>SAP Principal Architect</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>PROSPECTOR, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Peter Wheatley</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Enterprise Architect…</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Robb White</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr"/>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Peter Widmer</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the Global Head of S…</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Chad Wiech</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Director of Solution…</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Chamnida Wijetilleke</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>The Ducats Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Pete Wilkins</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>NA Partner Manager</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>SAP America(Bellevue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Mark Willey</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Vice…</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Ed Williamson</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Client Services Lead</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>XMATERIA LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Monica Willis</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>HR Strategy and Value A…</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Plano- Legacy West</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Charlotte Wilson</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Senior Manager Strategic Cha…</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Direct Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Emily Wisemiller</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Sr. Data Analyst</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Molex</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Julia Wolfe</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Analyst Relations Manager</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Jennifer Workman</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Techn…</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Universal Destinations &amp; Experiences</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Steven Wright Wright</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>VP Sales</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Monty Wurth</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>VP of Operations</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Optima Consulting L.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Brad Wylie</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>KAORI YASHIKI</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Business Resear…</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Hitachi Digital Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>YOUNGHO YOO</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Team Leader</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>LG CNS Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Mohamed YUSUF</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Head of Integrated Toolchain</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Hikaru Yafuso</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Senior Alliance Director</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Sonoko Yamamoto</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Partner Business Manager</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Osamu Yamazaki</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Co…</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Kenji Yanagi</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Group Leader</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>ASAHI GROUP JAPAN, LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>EJ Yang</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>IT Deputy Director</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>MediaTek Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Kiran Yarlagadda Yarlagadda</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Managing…</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Adroix Corp DBA CodeForce 360</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Takayuki Yasuda</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>JFE Systems, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Tomoki Yasuda</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>AssistantMana…</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Kazuhiro Yonekawa</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Chief/Proj…</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CANON MARKETING JAPAN INC.,</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Sungeui Yoon</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Senior Specialist</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Christopher Yope</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>SAP Supply C…</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>DXC Technology Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Kohei Yoshimatsu</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>アズビル株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>taichi yoshida</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Senior Ma…</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>nakajima yuki</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Nitori Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Stefan Zach</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>VP Global IT</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Wieland Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Beau Zaremski</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Yuan Zhang</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Senior Project Manager, SAP AI RIG</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Cathy Zhou</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>IT Director, EBS</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Gustavo Zintak</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>SWISS MEDICAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Alina Zuberi</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Global Content Strategist</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Yoshiaki Agata 縣</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>consultant</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>AJS株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>裕紀 阿保</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>FORTIENCE CONSULTING INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>謙介 青木</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Manager, Uvance Market Developme…</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Fujitsu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add V section and start of W section attendees
Inserts 45 entries (V section + Wa- through Waxman) between Cugliari
and Christy Weaver in the alphabetical list. Total now 325.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C281"/>
+  <dimension ref="A1:C326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4285,895 +4285,1652 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Christy Weaver</t>
+          <t>Suman Varma</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Global Demand Generation Man…</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Vertex, Inc.</t>
+          <t>Cintas Corporation</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Mike Weaver</t>
+          <t>Chris Vassalotti</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Senior I…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>True Commerce Inc. TrueCommerce</t>
+          <t>Opentext</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Chris Webster</t>
+          <t>Raju Vedala</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>SVP IT Strategy &amp; Architecture</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Ahold Delhaize</t>
+          <t>CES Business Technologies, LLC</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Matt Webster</t>
+          <t>Asier Vega Sanchez</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Director of…</t>
+          <t>Implementation Consultant</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Gardner White Furniture Co., Inc.</t>
+          <t>Arkyn</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Patrick Weil</t>
+          <t>Jennifer Veillon</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Dir Project Controls</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metrie Canada Ltd</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Sarah Weiler</t>
+          <t>Ajay Reddy Velampudi</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Manager, Busine…</t>
+          <t>Senior VP - Sa…</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Ball Horticultural Company</t>
+          <t>Miracle Software Systems Inc.</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Adam Werner</t>
+          <t>William Velastegui</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>VP, Corporate Technology</t>
+          <t>JEFE DE TI Y PR…</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Crocs, Inc.</t>
+          <t>Plasticaucho Industrial S.A.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Maddie Werner</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>Director of Delivery Solutions</t>
-        </is>
-      </c>
+          <t>Rajiv Vemula</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr"/>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Robra IT</t>
+          <t>Cognizant Technology Solutions U.S. Corporat…</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Katherine West</t>
+          <t>Sundu Venkataramani</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CX Account Executive</t>
+          <t>Industry Val…</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>SAP Industries (Washington DC)</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Anja Wettling</t>
+          <t>Venkat Venkataramani</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>VP</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>anuwo GmbH</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Charleen Wetzstein</t>
+          <t>Tom Venner-Crysell</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>SAP Principal Architect</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>PROSPECTOR, LLC</t>
+          <t>ERPeople Solutions Ltd</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Peter Wheatley</t>
+          <t>Eduardo Vergara</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Enterprise Architect…</t>
+          <t>Manager/Head of Dept</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>SAP America (Houston)</t>
+          <t>Agrosuper S.A.</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Robb White</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr"/>
+          <t>Amit Verma</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>RVP, Head of CFO Advisory…</t>
+        </is>
+      </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Peter Widmer</t>
+          <t>Kumar Vidit</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Chief of Staff to the Global Head of S…</t>
+          <t>Product Marketing M…</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>SAP America(Bellevue)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Chad Wiech</t>
+          <t>Lakshmi Vidyashankar</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Director of Solution…</t>
+          <t>VP of IT</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>Marvin Engineering Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Chamnida Wijetilleke</t>
+          <t>Jayant Vikram</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Cloud Delivery Lead</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>The Ducats Group LLC</t>
+          <t>Accenture LLP</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Pete Wilkins</t>
+          <t>Yeni Villanueva</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>NA Partner Manager</t>
+          <t>Supervisora…</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>Compañia Minera Antamina S.A.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Mark Willey</t>
+          <t>Robert Vinyard</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Vice…</t>
+          <t>VP and Senior Partner</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+          <t>IBM</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Ed Williamson</t>
+          <t>Thomas Vioux</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Client Services Lead</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>XMATERIA LTD</t>
+          <t>PwC</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Monica Willis</t>
+          <t>Anil Visal</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>HR Strategy and Value A…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Plano- Legacy West</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Charlotte Wilson</t>
+          <t>Clara Viscido</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Senior Manager Strategic Cha…</t>
+          <t>Consulting Services Director</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Direct Energy</t>
+          <t>GEONOSIS</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Emily Wisemiller</t>
-        </is>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>Sr. Data Analyst</t>
-        </is>
-      </c>
+          <t>Paulo Vita Vita</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr"/>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Julia Wolfe</t>
+          <t>Ranjan Vitt</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Analyst Relations Manager</t>
+          <t>AI Compliance Governance Program…</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Jennifer Workman</t>
+          <t>Jose Voisin</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Techn…</t>
+          <t>Global CIO</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Universal Destinations &amp; Experiences</t>
+          <t>Carmeuse</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Steven Wright Wright</t>
+          <t>Christina Volk</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>VP Sales</t>
+          <t>Head of Strate…</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Acuiti Labs Limited</t>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Monty Wurth</t>
+          <t>Jessica Voyles</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>VP of Operations</t>
+          <t>Account Executive, South</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Optima Consulting L.L.C.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Brad Wylie</t>
+          <t>Sandeep Vyas</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Account Executive</t>
+          <t>Solutio…</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>Incture Technologies Private Limited</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>KAORI YASHIKI</t>
+          <t>Thomas von Alm</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Business Resear…</t>
+          <t>SVP Cross-Solution Services</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services LLC</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>YOUNGHO YOO</t>
+          <t>Markus von Quast</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Team Leader</t>
+          <t>Global Head Industry Ecosystem</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>LG CNS Co., Ltd.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Mohamed YUSUF</t>
+          <t>TATSUO WATANABE</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Head of Integrated Toolchain</t>
+          <t>Principal Cons…</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>D I SQUARE CORPORATION.</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Hikaru Yafuso</t>
+          <t>Masayuki Wada</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Senior Alliance Director</t>
+          <t>SVP, Head of Corporate Digit…</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Fujitsu Limited</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Sonoko Yamamoto</t>
+          <t>Stephen Wagenheim</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Partner Business Manager</t>
+          <t>Senior Sales Executive - Suppl…</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>Dallas (Allen)</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Osamu Yamazaki</t>
+          <t>Neha Wahi</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Co…</t>
+          <t>Global Alliance Lead</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+          <t>A.T. Kearney, Inc.</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Kenji Yanagi</t>
+          <t>Waka Wakabayashi</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Group Leader</t>
+          <t>Associate Partner</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ASAHI GROUP JAPAN, LTD.</t>
+          <t>KPMG Consulting Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>EJ Yang</t>
+          <t>Gustavo Waldfogiel</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>IT Deputy Director</t>
+          <t>LAC HCM Head</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>MediaTek Inc.</t>
+          <t>SAP Argentina - Buenos Aires</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Kiran Yarlagadda Yarlagadda</t>
+          <t>Shashikant Walimbe</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Managing…</t>
+          <t>Vice President &amp; Global Head -…</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Adroix Corp DBA CodeForce 360</t>
+          <t>LTM LIMITED</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Takayuki Yasuda</t>
+          <t>Julie Walker</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>Sr. Director, Enterprise Applicatio…</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>JFE Systems, Inc.</t>
+          <t>Armstrong</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Tomoki Yasuda</t>
+          <t>Rob Wallace</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>AssistantMana…</t>
+          <t>Senior Manager Digital &amp; In…</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>NTT DATA Japan Corporation</t>
+          <t>Jaguarlandrover</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Kazuhiro Yonekawa</t>
+          <t>Enzhou Wang</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Chief/Proj…</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>CANON MARKETING JAPAN INC.,</t>
+          <t>City of Tacoma</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Sungeui Yoon</t>
+          <t>May Wang</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Senior Specialist</t>
+          <t>Direc…</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Christopher Yope</t>
+          <t>Adam Warner</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>SAP Supply C…</t>
+          <t>Cost Analyst</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>DXC Technology Services LLC</t>
+          <t>Marathon Cheese Corporation</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Kohei Yoshimatsu</t>
+          <t>Kosuke Watanabe</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Senior Account Executive</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>アズビル株式会社</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>taichi yoshida</t>
+          <t>Takashi Watanabe</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Senior Ma…</t>
+          <t>執行役員</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>BENIC SOLUTION CORPORATION</t>
+          <t>JFE Systems,Inc.</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>nakajima yuki</t>
+          <t>Robert Watson</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Member</t>
+          <t>Sr Account Executive</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Nitori Co., Ltd.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Stefan Zach</t>
+          <t>Ashley Waxman</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>VP Global IT</t>
+          <t>Strategic Sales Executive</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Wieland Group</t>
+          <t>Aevitas IT LLC</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Beau Zaremski</t>
+          <t>Christy Weaver</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>VP of Sales</t>
+          <t>Global Demand Generation Man…</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Vertex, Inc.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Yuan Zhang</t>
+          <t>Mike Weaver</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Senior Project Manager, SAP AI RIG</t>
+          <t>Senior I…</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>True Commerce Inc. TrueCommerce</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Cathy Zhou</t>
+          <t>Chris Webster</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>IT Director, EBS</t>
+          <t>SVP IT Strategy &amp; Architecture</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Ecolab Inc.</t>
+          <t>Ahold Delhaize</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Gustavo Zintak</t>
+          <t>Matt Webster</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>Director of…</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>SWISS MEDICAL S.A.</t>
+          <t>Gardner White Furniture Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Alina Zuberi</t>
+          <t>Patrick Weil</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Global Content Strategist</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>Metrie Canada Ltd</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Yoshiaki Agata 縣</t>
+          <t>Sarah Weiler</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>consultant</t>
+          <t>Manager, Busine…</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>AJS株式会社</t>
+          <t>Ball Horticultural Company</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>裕紀 阿保</t>
+          <t>Adam Werner</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>VP, Corporate Technology</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>FORTIENCE CONSULTING INC.</t>
+          <t>Crocs, Inc.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
+          <t>Maddie Werner</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Director of Delivery Solutions</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Robra IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Katherine West</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>CX Account Executive</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Anja Wettling</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>anuwo GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Charleen Wetzstein</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>SAP Principal Architect</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>PROSPECTOR, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Peter Wheatley</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Enterprise Architect…</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Robb White</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr"/>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Peter Widmer</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the Global Head of S…</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Chad Wiech</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Director of Solution…</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Chamnida Wijetilleke</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>The Ducats Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Pete Wilkins</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>NA Partner Manager</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>SAP America(Bellevue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Mark Willey</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Vice…</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Ed Williamson</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Client Services Lead</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>XMATERIA LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Monica Willis</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>HR Strategy and Value A…</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Plano- Legacy West</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Charlotte Wilson</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Senior Manager Strategic Cha…</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Direct Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Emily Wisemiller</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Sr. Data Analyst</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Molex</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Julia Wolfe</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Analyst Relations Manager</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Jennifer Workman</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Techn…</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Universal Destinations &amp; Experiences</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Steven Wright Wright</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>VP Sales</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Monty Wurth</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>VP of Operations</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Optima Consulting L.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Brad Wylie</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>KAORI YASHIKI</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Business Resear…</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Hitachi Digital Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>YOUNGHO YOO</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Team Leader</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>LG CNS Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Mohamed YUSUF</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Head of Integrated Toolchain</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Hikaru Yafuso</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Senior Alliance Director</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Sonoko Yamamoto</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Partner Business Manager</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Osamu Yamazaki</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Co…</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Kenji Yanagi</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Group Leader</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ASAHI GROUP JAPAN, LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>EJ Yang</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>IT Deputy Director</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>MediaTek Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Kiran Yarlagadda Yarlagadda</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Managing…</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Adroix Corp DBA CodeForce 360</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Takayuki Yasuda</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>JFE Systems, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Tomoki Yasuda</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>AssistantMana…</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Kazuhiro Yonekawa</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Chief/Proj…</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>CANON MARKETING JAPAN INC.,</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Sungeui Yoon</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Senior Specialist</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Christopher Yope</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>SAP Supply C…</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>DXC Technology Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Kohei Yoshimatsu</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>アズビル株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>taichi yoshida</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Senior Ma…</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>nakajima yuki</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Nitori Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Stefan Zach</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>VP Global IT</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Wieland Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Beau Zaremski</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Yuan Zhang</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Senior Project Manager, SAP AI RIG</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Cathy Zhou</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>IT Director, EBS</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Gustavo Zintak</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>SWISS MEDICAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Alina Zuberi</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Global Content Strategist</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Yoshiaki Agata 縣</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>consultant</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>AJS株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>裕紀 阿保</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>FORTIENCE CONSULTING INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
           <t>謙介 青木</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr">
+      <c r="B326" t="inlineStr">
         <is>
           <t>Manager, Uvance Market Developme…</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
+      <c r="C326" t="inlineStr">
         <is>
           <t>Fujitsu</t>
         </is>

</xml_diff>

<commit_message>
Add T, U, and start of V section attendees
Inserts 54 entries (T section, U section, and SACHIN VAIDYA through
Vijay Varee) between Cugliari and Suman Varma. Total now 379.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C326"/>
+  <dimension ref="A1:C380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4285,7 +4285,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Suman Varma</t>
+          <t>Ahmed Taher</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -4295,1642 +4295,2556 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Cintas Corporation</t>
+          <t>Al Daajan Trading</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Chris Vassalotti</t>
+          <t>Chieko Takahata</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Chief</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Opentext</t>
+          <t>BROTHER INDUSTRIES,LTD.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Raju Vedala</t>
+          <t>Arai Takahiro</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Services Delivery Manag…</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>CES Business Technologies, LLC</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Asier Vega Sanchez</t>
+          <t>Eiji Takashina</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Implementation Consultant</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Arkyn</t>
+          <t>Kyndryl Japan KK</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Jennifer Veillon</t>
+          <t>Tetsushi Takino</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Dir Project Controls</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>大和ハウス工業株式会社</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Ajay Reddy Velampudi</t>
+          <t>Makoto Tamura</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Senior VP - Sa…</t>
+          <t>Alliance Group Director</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Miracle Software Systems Inc.</t>
+          <t>FUJITSU LIMITED</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>William Velastegui</t>
+          <t>Chiyuki Tanaka</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>JEFE DE TI Y PR…</t>
+          <t>Team leader</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Plasticaucho Industrial S.A.</t>
+          <t>Recruit Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Rajiv Vemula</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr"/>
+          <t>Steve Tanaka</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Sr Vice Presid…</t>
+        </is>
+      </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Cognizant Technology Solutions U.S. Corporat…</t>
+          <t>Blommer Chocolate Company</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Sundu Venkataramani</t>
+          <t>Yasuhiro Tanaka</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Industry Val…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>SAP Industries (Washington DC)</t>
+          <t>Recuruit Co.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Venkat Venkataramani</t>
+          <t>Kristin Taner</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>Chief Marke…</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Vortex Software Consulting, LLC</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Tom Venner-Crysell</t>
+          <t>Mitchell Tauer</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Services Account Execut…</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>ERPeople Solutions Ltd</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Eduardo Vergara</t>
+          <t>Roxanna Tavares</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>Director, Gl…</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Agrosuper S.A.</t>
+          <t>The Nielsen Company (US), LLC.</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Amit Verma</t>
+          <t>Theo Tavrides</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>RVP, Head of CFO Advisory…</t>
+          <t>Vice Presi…</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>SAP ASIA Pte Ltd</t>
+          <t>NTT Data Business Solutions, Inc.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Kumar Vidit</t>
+          <t>Jamie Taylor</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Product Marketing M…</t>
+          <t>Global VP, Strategic Partnerships</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Lakshmi Vidyashankar</t>
+          <t>Meghan Taylor</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>VP of IT</t>
+          <t>Industry Account Ex…</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Marvin Engineering Co., Inc.</t>
+          <t>Pittsburgh, SAP America</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Jayant Vikram</t>
+          <t>Samantha Taylor</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Cloud Delivery Lead</t>
+          <t>Senior Solutions Account Exec…</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Accenture LLP</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Yeni Villanueva</t>
+          <t>Sarah Taylor</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Supervisora…</t>
+          <t>Solution Advisor</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Compañia Minera Antamina S.A.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Robert Vinyard</t>
+          <t>Jorge Tercero</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>VP and Senior Partner</t>
+          <t>Manager/H…</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Asociacion Mutual Sancor Salud</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Thomas Vioux</t>
+          <t>Michael Teti</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Carlisle Construction Materials</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Anil Visal</t>
+          <t>Suji Thampi</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers LLP</t>
+          <t>MINDSPRINT PTE. LTD.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Clara Viscido</t>
+          <t>Le Thanh Phong</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Consulting Services Director</t>
+          <t>Managing Direc…</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>GEONOSIS</t>
+          <t>FPT Japan Holdings Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Paulo Vita Vita</t>
-        </is>
-      </c>
-      <c r="B250" t="inlineStr"/>
+          <t>Michael Theis</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Senior Director, Healthcare Life Scien…</t>
+        </is>
+      </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
+          <t>Icertis</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Ranjan Vitt</t>
+          <t>Rene Theriault</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>AI Compliance Governance Program…</t>
+          <t>IT Program Director</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>BRP INC</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Jose Voisin</t>
+          <t>Barbara Thrasher</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Global CIO</t>
+          <t>SR STAFF ARCHITECT</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Carmeuse</t>
+          <t>Tyson Foods, Inc.</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Christina Volk</t>
+          <t>Nissim Titan</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Head of Strate…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>SAP Deutschland SE &amp;Co.KG</t>
+          <t>4CAST SYSTEMS LTD</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Jessica Voyles</t>
+          <t>James Tiwari</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Account Executive, South</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Intellioz LLC</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Sandeep Vyas</t>
+          <t>Shuhei Toba</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Solutio…</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Incture Technologies Private Limited</t>
+          <t>Business Engineering Corporation</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Thomas von Alm</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>SVP Cross-Solution Services</t>
-        </is>
-      </c>
+          <t>John Tocci</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr"/>
       <c r="C256" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Cbs Corporate Business Solutions America In…</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Markus von Quast</t>
+          <t>Oliver Toloui</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Global Head Industry Ecosystem</t>
+          <t>Director - AI…</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Ibase Operations Corp Qualitest</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>TATSUO WATANABE</t>
+          <t>Ray Toma</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Principal Cons…</t>
+          <t>Senior Principal — Global Strategic Initia…</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>D I SQUARE CORPORATION.</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Masayuki Wada</t>
+          <t>Yuko Tominaga</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>SVP, Head of Corporate Digit…</t>
+          <t>Research Writer</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Fujitsu Limited</t>
+          <t>Freelance</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Stephen Wagenheim</t>
+          <t>Laura Tozzo</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Senior Sales Executive - Suppl…</t>
+          <t>AI Product Lead SAP IBP</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Dallas (Allen)</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Neha Wahi</t>
+          <t>Eero Traagel</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Global Alliance Lead</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>A.T. Kearney, Inc.</t>
+          <t>IBM Canada Limited</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Waka Wakabayashi</t>
+          <t>Adam Trahan</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Associate Partner</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>KPMG Consulting Co., Ltd.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Gustavo Waldfogiel</t>
+          <t>Evgeny Treskin</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>LAC HCM Head</t>
+          <t>SAP Alliances Director</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>SAP Argentina - Buenos Aires</t>
+          <t>Argano</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Shashikant Walimbe</t>
+          <t>Chetan Tripathi</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Vice President &amp; Global Head -…</t>
+          <t>oCFO Adoption expert</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>LTM LIMITED</t>
+          <t>SAP</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Julie Walker</t>
+          <t>Seshagiri Tripurana</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Sr. Director, Enterprise Applicatio…</t>
+          <t>Senior Director</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Armstrong</t>
+          <t>Johnson &amp; Johnson</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Rob Wallace</t>
+          <t>Masaru Tsukahira</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Senior Manager Digital &amp; In…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Jaguarlandrover</t>
+          <t>TOKYO ELECTRON LIMITED.</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Enzhou Wang</t>
+          <t>Lindsay Tucker</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Chief Technology Officer</t>
+          <t>Solution Consultant</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>City of Tacoma</t>
+          <t>Docusign</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>May Wang</t>
+          <t>Paul Turbes</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Direc…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
+          <t>KPMG LLP</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Adam Warner</t>
+          <t>Treaver Tyler</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Cost Analyst</t>
+          <t>Tech…</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Marathon Cheese Corporation</t>
+          <t>Meijer Great Lakes Limited Partnership</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Kosuke Watanabe</t>
+          <t>Kotaro Ueda</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Senior Account Executive</t>
+          <t>Chief Operating Officer</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>JSUG</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Takashi Watanabe</t>
+          <t>Rajkishore Una</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>執行役員</t>
+          <t>President/CEO</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>JFE Systems,Inc.</t>
+          <t>GyanSys, Inc.</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Robert Watson</t>
+          <t>Bala Parameswara Rao Upadhyay…</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Sr Account Executive</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Stefanini, Inc.</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Ashley Waxman</t>
+          <t>Oscar Uribe</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Strategic Sales Executive</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Aevitas IT LLC</t>
+          <t>EDUARDONO S A S</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Christy Weaver</t>
+          <t>SACHIN VAIDYA</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Global Demand Generation Man…</t>
+          <t>Director - Enterprise Commercial…</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Vertex, Inc.</t>
+          <t>Pfizer, Inc.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Mike Weaver</t>
+          <t>Jonathan VON RUEDEN</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Senior I…</t>
+          <t>Chief AI Officer</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>True Commerce Inc. TrueCommerce</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Chris Webster</t>
+          <t>Wagner Valentin</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>SVP IT Strategy &amp; Architecture</t>
+          <t>Director of Regulated Indust…</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Ahold Delhaize</t>
+          <t>SAP Brasil Ltda.</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Matt Webster</t>
+          <t>Jorge Valles Velásquez</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Director of…</t>
+          <t>KMMP…</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Gardner White Furniture Co., Inc.</t>
+          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Patrick Weil</t>
+          <t>Henri Vallet</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>VP Sales, Americas B2B</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Metrie Canada Ltd</t>
+          <t>Mirakl</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Sarah Weiler</t>
+          <t>Jeff Van Pelt</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Manager, Busine…</t>
+          <t>Founder / Managing Dire…</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ball Horticultural Company</t>
+          <t>Javelin Consulting</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Adam Werner</t>
+          <t>Meredith Van Wyk</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>VP, Corporate Technology</t>
+          <t>Americas Field Partner…</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Crocs, Inc.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Maddie Werner</t>
+          <t>Joris Van der Donck</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Director of Delivery Solutions</t>
+          <t>Sr Manag…</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Robra IT</t>
+          <t>Commscope Connectivity Belgium</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Katherine West</t>
+          <t>Vijay Varee</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>CX Account Executive</t>
+          <t>Senior Manager</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>Petsmart LLC</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Anja Wettling</t>
+          <t>Suman Varma</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>anuwo GmbH</t>
+          <t>Cintas Corporation</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Charleen Wetzstein</t>
+          <t>Chris Vassalotti</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>SAP Principal Architect</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>PROSPECTOR, LLC</t>
+          <t>Opentext</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Peter Wheatley</t>
+          <t>Raju Vedala</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Enterprise Architect…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>SAP America (Houston)</t>
+          <t>CES Business Technologies, LLC</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Robb White</t>
-        </is>
-      </c>
-      <c r="B286" t="inlineStr"/>
+          <t>Asier Vega Sanchez</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Implementation Consultant</t>
+        </is>
+      </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+          <t>Arkyn</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Peter Widmer</t>
+          <t>Jennifer Veillon</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Chief of Staff to the Global Head of S…</t>
+          <t>Dir Project Controls</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Chad Wiech</t>
+          <t>Ajay Reddy Velampudi</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Director of Solution…</t>
+          <t>Senior VP - Sa…</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>Miracle Software Systems Inc.</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Chamnida Wijetilleke</t>
+          <t>William Velastegui</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>JEFE DE TI Y PR…</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>The Ducats Group LLC</t>
+          <t>Plasticaucho Industrial S.A.</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Pete Wilkins</t>
-        </is>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>NA Partner Manager</t>
-        </is>
-      </c>
+          <t>Rajiv Vemula</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr"/>
       <c r="C290" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>Cognizant Technology Solutions U.S. Corporat…</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Mark Willey</t>
+          <t>Sundu Venkataramani</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Vice…</t>
+          <t>Industry Val…</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+          <t>SAP Industries (Washington DC)</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Ed Williamson</t>
+          <t>Venkat Venkataramani</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Client Services Lead</t>
+          <t>VP</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>XMATERIA LTD</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Monica Willis</t>
+          <t>Tom Venner-Crysell</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>HR Strategy and Value A…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Plano- Legacy West</t>
+          <t>ERPeople Solutions Ltd</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Charlotte Wilson</t>
+          <t>Eduardo Vergara</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Senior Manager Strategic Cha…</t>
+          <t>Manager/Head of Dept</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Direct Energy</t>
+          <t>Agrosuper S.A.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Emily Wisemiller</t>
+          <t>Amit Verma</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>RVP, Head of CFO Advisory…</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Julia Wolfe</t>
+          <t>Kumar Vidit</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Analyst Relations Manager</t>
+          <t>Product Marketing M…</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>SAP America(Bellevue)</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Jennifer Workman</t>
+          <t>Lakshmi Vidyashankar</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Techn…</t>
+          <t>VP of IT</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Universal Destinations &amp; Experiences</t>
+          <t>Marvin Engineering Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Steven Wright Wright</t>
+          <t>Jayant Vikram</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>VP Sales</t>
+          <t>Cloud Delivery Lead</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Acuiti Labs Limited</t>
+          <t>Accenture LLP</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Monty Wurth</t>
+          <t>Yeni Villanueva</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>VP of Operations</t>
+          <t>Supervisora…</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Optima Consulting L.L.C.</t>
+          <t>Compañia Minera Antamina S.A.</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Brad Wylie</t>
+          <t>Robert Vinyard</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Account Executive</t>
+          <t>VP and Senior Partner</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>IBM</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>KAORI YASHIKI</t>
+          <t>Thomas Vioux</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Business Resear…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services LLC</t>
+          <t>PwC</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>YOUNGHO YOO</t>
+          <t>Anil Visal</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Team Leader</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>LG CNS Co., Ltd.</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Mohamed YUSUF</t>
+          <t>Clara Viscido</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Head of Integrated Toolchain</t>
+          <t>Consulting Services Director</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>GEONOSIS</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Hikaru Yafuso</t>
-        </is>
-      </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>Senior Alliance Director</t>
-        </is>
-      </c>
+          <t>Paulo Vita Vita</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr"/>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Sonoko Yamamoto</t>
+          <t>Ranjan Vitt</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Partner Business Manager</t>
+          <t>AI Compliance Governance Program…</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Osamu Yamazaki</t>
+          <t>Jose Voisin</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Co…</t>
+          <t>Global CIO</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+          <t>Carmeuse</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Kenji Yanagi</t>
+          <t>Christina Volk</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Group Leader</t>
+          <t>Head of Strate…</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>ASAHI GROUP JAPAN, LTD.</t>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>EJ Yang</t>
+          <t>Jessica Voyles</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>IT Deputy Director</t>
+          <t>Account Executive, South</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>MediaTek Inc.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Kiran Yarlagadda Yarlagadda</t>
+          <t>Sandeep Vyas</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Managing…</t>
+          <t>Solutio…</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Adroix Corp DBA CodeForce 360</t>
+          <t>Incture Technologies Private Limited</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Takayuki Yasuda</t>
+          <t>Thomas von Alm</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>SVP Cross-Solution Services</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>JFE Systems, Inc.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Tomoki Yasuda</t>
+          <t>Markus von Quast</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>AssistantMana…</t>
+          <t>Global Head Industry Ecosystem</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>NTT DATA Japan Corporation</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Kazuhiro Yonekawa</t>
+          <t>TATSUO WATANABE</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Chief/Proj…</t>
+          <t>Principal Cons…</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>CANON MARKETING JAPAN INC.,</t>
+          <t>D I SQUARE CORPORATION.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Sungeui Yoon</t>
+          <t>Masayuki Wada</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Senior Specialist</t>
+          <t>SVP, Head of Corporate Digit…</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Fujitsu Limited</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Christopher Yope</t>
+          <t>Stephen Wagenheim</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>SAP Supply C…</t>
+          <t>Senior Sales Executive - Suppl…</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>DXC Technology Services LLC</t>
+          <t>Dallas (Allen)</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Kohei Yoshimatsu</t>
+          <t>Neha Wahi</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Global Alliance Lead</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>アズビル株式会社</t>
+          <t>A.T. Kearney, Inc.</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>taichi yoshida</t>
+          <t>Waka Wakabayashi</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Senior Ma…</t>
+          <t>Associate Partner</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>BENIC SOLUTION CORPORATION</t>
+          <t>KPMG Consulting Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>nakajima yuki</t>
+          <t>Gustavo Waldfogiel</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Member</t>
+          <t>LAC HCM Head</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Nitori Co., Ltd.</t>
+          <t>SAP Argentina - Buenos Aires</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Stefan Zach</t>
+          <t>Shashikant Walimbe</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>VP Global IT</t>
+          <t>Vice President &amp; Global Head -…</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Wieland Group</t>
+          <t>LTM LIMITED</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Beau Zaremski</t>
+          <t>Julie Walker</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>VP of Sales</t>
+          <t>Sr. Director, Enterprise Applicatio…</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Armstrong</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Yuan Zhang</t>
+          <t>Rob Wallace</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Senior Project Manager, SAP AI RIG</t>
+          <t>Senior Manager Digital &amp; In…</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Jaguarlandrover</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Cathy Zhou</t>
+          <t>Enzhou Wang</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>IT Director, EBS</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Ecolab Inc.</t>
+          <t>City of Tacoma</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Gustavo Zintak</t>
+          <t>May Wang</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>Direc…</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>SWISS MEDICAL S.A.</t>
+          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Alina Zuberi</t>
+          <t>Adam Warner</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Global Content Strategist</t>
+          <t>Cost Analyst</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>Marathon Cheese Corporation</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Yoshiaki Agata 縣</t>
+          <t>Kosuke Watanabe</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>consultant</t>
+          <t>Senior Account Executive</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>AJS株式会社</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>裕紀 阿保</t>
+          <t>Takashi Watanabe</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>執行役員</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>FORTIENCE CONSULTING INC.</t>
+          <t>JFE Systems,Inc.</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
+          <t>Robert Watson</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Sr Account Executive</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Ashley Waxman</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Strategic Sales Executive</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Aevitas IT LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Christy Weaver</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Global Demand Generation Man…</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Mike Weaver</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Senior I…</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>True Commerce Inc. TrueCommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Chris Webster</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>SVP IT Strategy &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Ahold Delhaize</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Matt Webster</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Director of…</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Gardner White Furniture Co., Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Patrick Weil</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>IT Director</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Metrie Canada Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Sarah Weiler</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Manager, Busine…</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Ball Horticultural Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Adam Werner</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>VP, Corporate Technology</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Crocs, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Maddie Werner</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Director of Delivery Solutions</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Robra IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Katherine West</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>CX Account Executive</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Anja Wettling</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>anuwo GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Charleen Wetzstein</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>SAP Principal Architect</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>PROSPECTOR, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Peter Wheatley</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Enterprise Architect…</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Robb White</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr"/>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Peter Widmer</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the Global Head of S…</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Chad Wiech</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Director of Solution…</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Chamnida Wijetilleke</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>The Ducats Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Pete Wilkins</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>NA Partner Manager</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>SAP America(Bellevue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Mark Willey</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Vice…</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Ed Williamson</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Client Services Lead</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>XMATERIA LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Monica Willis</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>HR Strategy and Value A…</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Plano- Legacy West</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Charlotte Wilson</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Senior Manager Strategic Cha…</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Direct Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Emily Wisemiller</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Sr. Data Analyst</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Molex</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Julia Wolfe</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Analyst Relations Manager</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Jennifer Workman</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Techn…</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Universal Destinations &amp; Experiences</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Steven Wright Wright</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>VP Sales</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Monty Wurth</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>VP of Operations</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Optima Consulting L.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Brad Wylie</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>KAORI YASHIKI</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Business Resear…</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Hitachi Digital Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>YOUNGHO YOO</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Team Leader</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>LG CNS Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Mohamed YUSUF</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Head of Integrated Toolchain</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Hikaru Yafuso</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Senior Alliance Director</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Sonoko Yamamoto</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Partner Business Manager</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Osamu Yamazaki</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Co…</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Kenji Yanagi</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Group Leader</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>ASAHI GROUP JAPAN, LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>EJ Yang</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>IT Deputy Director</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>MediaTek Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Kiran Yarlagadda Yarlagadda</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Managing…</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Adroix Corp DBA CodeForce 360</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Takayuki Yasuda</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>JFE Systems, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Tomoki Yasuda</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>AssistantMana…</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Kazuhiro Yonekawa</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Chief/Proj…</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>CANON MARKETING JAPAN INC.,</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Sungeui Yoon</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Senior Specialist</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Christopher Yope</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>SAP Supply C…</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>DXC Technology Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Kohei Yoshimatsu</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>アズビル株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>taichi yoshida</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Senior Ma…</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>nakajima yuki</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Nitori Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Stefan Zach</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>VP Global IT</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Wieland Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Beau Zaremski</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Yuan Zhang</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Senior Project Manager, SAP AI RIG</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Cathy Zhou</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>IT Director, EBS</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Gustavo Zintak</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>SWISS MEDICAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Alina Zuberi</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Global Content Strategist</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Yoshiaki Agata 縣</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>consultant</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>AJS株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>裕紀 阿保</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>FORTIENCE CONSULTING INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
           <t>謙介 青木</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
+      <c r="B380" t="inlineStr">
         <is>
           <t>Manager, Uvance Market Developme…</t>
         </is>
       </c>
-      <c r="C326" t="inlineStr">
+      <c r="C380" t="inlineStr">
         <is>
           <t>Fujitsu</t>
         </is>

</xml_diff>

<commit_message>
Add S section and 3 leading T section attendees
Inserts 46 entries (full S section plus MARCO TOMBOLINI, KAZUSHI
TOYOMASU, Stacey Taborelli) between Cugliari and Ahmed Taher.
Total now 425.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C380"/>
+  <dimension ref="A1:C426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4285,1343 +4285,1339 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Ahmed Taher</t>
+          <t>Sukhbir Singh</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>S…</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Al Daajan Trading</t>
+          <t>The School Board of Duval County Florida</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Chieko Takahata</t>
+          <t>Vikrant Sisodia</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Chief</t>
+          <t>Sr. Product Manager</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>BROTHER INDUSTRIES,LTD.</t>
+          <t>Autodesk, Inc.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Arai Takahiro</t>
+          <t>David Smith</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Services Delivery Manag…</t>
+          <t>VP, Chief Enterprise Ar…</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>SAP America (Reston)</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Eiji Takashina</t>
+          <t>Rachel Smith</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Associate Director</t>
+          <t>Partner Sales Manager</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Kyndryl Japan KK</t>
+          <t>Docusign Inc</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Tetsushi Takino</t>
+          <t>Mark Smysor</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Business Systems Analyst in Enterpri…</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>大和ハウス工業株式会社</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Makoto Tamura</t>
+          <t>Delaiah Snowden</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Alliance Group Director</t>
+          <t>IT Ana…</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>FUJITSU LIMITED</t>
+          <t>South Florida Water Management Dist</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Chiyuki Tanaka</t>
+          <t>Jairo Soares De Matos</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Team leader</t>
+          <t>Analyst - SAP Busi…</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Recruit Co., Ltd.</t>
+          <t>Canadian Blood Services</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Steve Tanaka</t>
+          <t>Michael Somerville</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Sr Vice Presid…</t>
+          <t>Sales Executive</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Blommer Chocolate Company</t>
+          <t>Checkout.com</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Yasuhiro Tanaka</t>
+          <t>YoonWon Song</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Recuruit Co.,Ltd.</t>
+          <t>i-SENS, Inc.</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Kristin Taner</t>
+          <t>Dag Terje Sorlie</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Chief Marke…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Vortex Software Consulting, LLC</t>
+          <t>Accenture</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Mitchell Tauer</t>
+          <t>Thiago Souza</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Services Account Execut…</t>
+          <t>IT CO…</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>MINERACAO SERRAS DO OESTE LTDA</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Roxanna Tavares</t>
+          <t>Meik Spanowsky</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Director, Gl…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>The Nielsen Company (US), LLC.</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Theo Tavrides</t>
+          <t>Thorsten Spihlmann</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Vice Presi…</t>
+          <t>Head of Business Development for T…</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>NTT Data Business Solutions, Inc.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Jamie Taylor</t>
+          <t>TD Srinivasan</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Global VP, Strategic Partnerships</t>
+          <t>Industry…</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>SAP Public Services, Inc. (Hudson Y</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Meghan Taylor</t>
+          <t>Mike Stafford</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Industry Account Ex…</t>
+          <t>Senior ABAP Developer</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>Titan Ventures LLC</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Samantha Taylor</t>
+          <t>Jennifer Stapleton</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Senior Solutions Account Exec…</t>
+          <t>VP of Accounting Strategy &amp;…</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>American Equity</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Sarah Taylor</t>
+          <t>John Stark</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Solution Advisor</t>
+          <t>Global Head of SAP Alliance</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Loftware</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Jorge Tercero</t>
-        </is>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>Manager/H…</t>
-        </is>
-      </c>
+          <t>Denis Staudt</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr"/>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Asociacion Mutual Sancor Salud</t>
+          <t>GLOBAL DISTRIBUIÇÃO DE BENS DE CONSU…</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Michael Teti</t>
+          <t>Maximilian Stein</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>SAP Product Owner - Treasury CPIT</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Carlisle Construction Materials</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Suji Thampi</t>
+          <t>Amanda Steiner</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Business Process Architect</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>MINDSPRINT PTE. LTD.</t>
+          <t>McKesson</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Le Thanh Phong</t>
-        </is>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>Managing Direc…</t>
-        </is>
-      </c>
+          <t>Dieter Steinmann</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr"/>
       <c r="C249" t="inlineStr">
         <is>
-          <t>FPT Japan Holdings Co., Ltd.</t>
+          <t>Fraport AG Frankfurt Airport Services Worldwi…</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Michael Theis</t>
+          <t>Jorrit Steinz</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Senior Director, Healthcare Life Scien…</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Icertis</t>
+          <t>ChannelEngine.com</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Rene Theriault</t>
+          <t>Robert Stemmler</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>IT Program Director</t>
+          <t>Global Alliances &amp; Ec…</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>BRP INC</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Barbara Thrasher</t>
+          <t>Yonathan Stephanos</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>SR STAFF ARCHITECT</t>
+          <t>SAP Data &amp; AI Business Group Le…</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Tyson Foods, Inc.</t>
+          <t>Accenture</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Nissim Titan</t>
+          <t>Patrick Stewart</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Account Executive</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>4CAST SYSTEMS LTD</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>James Tiwari</t>
+          <t>Jochen Stiebe</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Head of Sales Treas…</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Intellioz LLC</t>
+          <t>Target-Networks GmbH</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Shuhei Toba</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
+          <t>Leslie Stoffel</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr"/>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Business Engineering Corporation</t>
+          <t>CARMEUSE RESEARCH AND TECHNOLOGY S…</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>John Tocci</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr"/>
+          <t>Miodrag Stojanov</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Lead Engineer</t>
+        </is>
+      </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Cbs Corporate Business Solutions America In…</t>
+          <t>SEMOS SOFTWARE LLC</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Oliver Toloui</t>
+          <t>Bojana Stojanovich</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Director - AI…</t>
+          <t>VP, NA Strategic Partnerships</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Ibase Operations Corp Qualitest</t>
+          <t>Tricentis</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Ray Toma</t>
+          <t>Seda Strate</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Senior Principal — Global Strategic Initia…</t>
+          <t>Partner Innovation Lead</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Yuko Tominaga</t>
+          <t>Divya Struebing</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Research Writer</t>
+          <t>Supply Chain Customer…</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Freelance</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Laura Tozzo</t>
+          <t>Kevin Stupp</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>AI Product Lead SAP IBP</t>
+          <t>Director S4 Platform</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>The Hershey Company</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Eero Traagel</t>
+          <t>Harish Subramanian</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Principal Enterprise Arch…</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>IBM Canada Limited</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Adam Trahan</t>
+          <t>Marc Sudjian</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Enterprise Architect, SAP So…</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Bombardier Inc.</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Evgeny Treskin</t>
+          <t>Hirofumi Sugimoto</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>SAP Alliances Director</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Argano</t>
+          <t>ABeam Systems Ltd.</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Chetan Tripathi</t>
+          <t>Michael Sukachev</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>oCFO Adoption expert</t>
+          <t>Sr. EA</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Teranet Inc</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Seshagiri Tripurana</t>
+          <t>Som Suresh</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Senior Director</t>
+          <t>Man…</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Johnson &amp; Johnson</t>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Masaru Tsukahira</t>
+          <t>Jain Sushant</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Chief Revenue Officer, F&amp;S…</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>TOKYO ELECTRON LIMITED.</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Lindsay Tucker</t>
+          <t>Scott Sutker</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Solution Consultant</t>
+          <t>Vice President Customer Success…</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Docusign</t>
+          <t>Alpharetta</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Paul Turbes</t>
+          <t>Mergenthaler Sven</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Global Head of Strategic Central Ser…</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>KPMG LLP</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Treaver Tyler</t>
+          <t>Jereme Swoboda</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Tech…</t>
+          <t>Segment Director</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Meijer Great Lakes Limited Partnership</t>
+          <t>Avvale, Inc.</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Kotaro Ueda</t>
+          <t>Debra Syring</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Chief Operating Officer</t>
+          <t>Senior IT Manager</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>JSUG</t>
+          <t>Entegris, Inc.</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Rajkishore Una</t>
+          <t>Kai Szatkowski</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>President/CEO</t>
+          <t>Head of Product Sales</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>GyanSys, Inc.</t>
+          <t>Natuvion GmbH</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Bala Parameswara Rao Upadhyay…</t>
+          <t>MARCO TOMBOLINI</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Associate Director</t>
+          <t>Global He…</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Stefanini, Inc.</t>
+          <t>DOLCE &amp; GABBANA BEAUTY SRL</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Oscar Uribe</t>
+          <t>KAZUSHI TOYOMASU</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>Global Direct…</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>EDUARDONO S A S</t>
+          <t>MOL Chemical Tankers Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>SACHIN VAIDYA</t>
+          <t>Stacey Taborelli</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Director - Enterprise Commercial…</t>
+          <t>Executive Business Partn…</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Pfizer, Inc.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Jonathan VON RUEDEN</t>
+          <t>Ahmed Taher</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Chief AI Officer</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Al Daajan Trading</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Wagner Valentin</t>
+          <t>Chieko Takahata</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Director of Regulated Indust…</t>
+          <t>Chief</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>SAP Brasil Ltda.</t>
+          <t>BROTHER INDUSTRIES,LTD.</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Jorge Valles Velásquez</t>
+          <t>Arai Takahiro</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>KMMP…</t>
+          <t>Services Delivery Manag…</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Henri Vallet</t>
+          <t>Eiji Takashina</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>VP Sales, Americas B2B</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Mirakl</t>
+          <t>Kyndryl Japan KK</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Jeff Van Pelt</t>
+          <t>Tetsushi Takino</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Founder / Managing Dire…</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Javelin Consulting</t>
+          <t>大和ハウス工業株式会社</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Meredith Van Wyk</t>
+          <t>Makoto Tamura</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Americas Field Partner…</t>
+          <t>Alliance Group Director</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>FUJITSU LIMITED</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Joris Van der Donck</t>
+          <t>Chiyuki Tanaka</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Sr Manag…</t>
+          <t>Team leader</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Commscope Connectivity Belgium</t>
+          <t>Recruit Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Vijay Varee</t>
+          <t>Steve Tanaka</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Senior Manager</t>
+          <t>Sr Vice Presid…</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Petsmart LLC</t>
+          <t>Blommer Chocolate Company</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Suman Varma</t>
+          <t>Yasuhiro Tanaka</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Cintas Corporation</t>
+          <t>Recuruit Co.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Chris Vassalotti</t>
+          <t>Kristin Taner</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Chief Marke…</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Opentext</t>
+          <t>Vortex Software Consulting, LLC</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Raju Vedala</t>
+          <t>Mitchell Tauer</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Services Account Execut…</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>CES Business Technologies, LLC</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Asier Vega Sanchez</t>
+          <t>Roxanna Tavares</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Implementation Consultant</t>
+          <t>Director, Gl…</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Arkyn</t>
+          <t>The Nielsen Company (US), LLC.</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Jennifer Veillon</t>
+          <t>Theo Tavrides</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Dir Project Controls</t>
+          <t>Vice Presi…</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>NTT Data Business Solutions, Inc.</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Ajay Reddy Velampudi</t>
+          <t>Jamie Taylor</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Senior VP - Sa…</t>
+          <t>Global VP, Strategic Partnerships</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Miracle Software Systems Inc.</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>William Velastegui</t>
+          <t>Meghan Taylor</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>JEFE DE TI Y PR…</t>
+          <t>Industry Account Ex…</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Plasticaucho Industrial S.A.</t>
+          <t>Pittsburgh, SAP America</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Rajiv Vemula</t>
-        </is>
-      </c>
-      <c r="B290" t="inlineStr"/>
+          <t>Samantha Taylor</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Senior Solutions Account Exec…</t>
+        </is>
+      </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Cognizant Technology Solutions U.S. Corporat…</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Sundu Venkataramani</t>
+          <t>Sarah Taylor</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Industry Val…</t>
+          <t>Solution Advisor</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>SAP Industries (Washington DC)</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Venkat Venkataramani</t>
+          <t>Jorge Tercero</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>Manager/H…</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Asociacion Mutual Sancor Salud</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Tom Venner-Crysell</t>
+          <t>Michael Teti</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ERPeople Solutions Ltd</t>
+          <t>Carlisle Construction Materials</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Eduardo Vergara</t>
+          <t>Suji Thampi</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Agrosuper S.A.</t>
+          <t>MINDSPRINT PTE. LTD.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Amit Verma</t>
+          <t>Le Thanh Phong</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>RVP, Head of CFO Advisory…</t>
+          <t>Managing Direc…</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>SAP ASIA Pte Ltd</t>
+          <t>FPT Japan Holdings Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Kumar Vidit</t>
+          <t>Michael Theis</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Product Marketing M…</t>
+          <t>Senior Director, Healthcare Life Scien…</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>Icertis</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Lakshmi Vidyashankar</t>
+          <t>Rene Theriault</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>VP of IT</t>
+          <t>IT Program Director</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Marvin Engineering Co., Inc.</t>
+          <t>BRP INC</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Jayant Vikram</t>
+          <t>Barbara Thrasher</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Cloud Delivery Lead</t>
+          <t>SR STAFF ARCHITECT</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Accenture LLP</t>
+          <t>Tyson Foods, Inc.</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Yeni Villanueva</t>
+          <t>Nissim Titan</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Supervisora…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Compañia Minera Antamina S.A.</t>
+          <t>4CAST SYSTEMS LTD</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Robert Vinyard</t>
+          <t>James Tiwari</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>VP and Senior Partner</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Intellioz LLC</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Thomas Vioux</t>
+          <t>Shuhei Toba</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Business Engineering Corporation</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Anil Visal</t>
-        </is>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
+          <t>John Tocci</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr"/>
       <c r="C302" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers LLP</t>
+          <t>Cbs Corporate Business Solutions America In…</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Clara Viscido</t>
+          <t>Oliver Toloui</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Consulting Services Director</t>
+          <t>Director - AI…</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>GEONOSIS</t>
+          <t>Ibase Operations Corp Qualitest</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Paulo Vita Vita</t>
-        </is>
-      </c>
-      <c r="B304" t="inlineStr"/>
+          <t>Ray Toma</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Senior Principal — Global Strategic Initia…</t>
+        </is>
+      </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Ranjan Vitt</t>
+          <t>Yuko Tominaga</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>AI Compliance Governance Program…</t>
+          <t>Research Writer</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Freelance</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Jose Voisin</t>
+          <t>Laura Tozzo</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Global CIO</t>
+          <t>AI Product Lead SAP IBP</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Carmeuse</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Christina Volk</t>
+          <t>Eero Traagel</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Head of Strate…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>SAP Deutschland SE &amp;Co.KG</t>
+          <t>IBM Canada Limited</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Jessica Voyles</t>
+          <t>Adam Trahan</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Account Executive, South</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -5633,301 +5629,301 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Sandeep Vyas</t>
+          <t>Evgeny Treskin</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Solutio…</t>
+          <t>SAP Alliances Director</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Incture Technologies Private Limited</t>
+          <t>Argano</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Thomas von Alm</t>
+          <t>Chetan Tripathi</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>SVP Cross-Solution Services</t>
+          <t>oCFO Adoption expert</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>SAP</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Markus von Quast</t>
+          <t>Seshagiri Tripurana</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Global Head Industry Ecosystem</t>
+          <t>Senior Director</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Johnson &amp; Johnson</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>TATSUO WATANABE</t>
+          <t>Masaru Tsukahira</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Principal Cons…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>D I SQUARE CORPORATION.</t>
+          <t>TOKYO ELECTRON LIMITED.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Masayuki Wada</t>
+          <t>Lindsay Tucker</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>SVP, Head of Corporate Digit…</t>
+          <t>Solution Consultant</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Fujitsu Limited</t>
+          <t>Docusign</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Stephen Wagenheim</t>
+          <t>Paul Turbes</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Senior Sales Executive - Suppl…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Dallas (Allen)</t>
+          <t>KPMG LLP</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Neha Wahi</t>
+          <t>Treaver Tyler</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Global Alliance Lead</t>
+          <t>Tech…</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>A.T. Kearney, Inc.</t>
+          <t>Meijer Great Lakes Limited Partnership</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Waka Wakabayashi</t>
+          <t>Kotaro Ueda</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Associate Partner</t>
+          <t>Chief Operating Officer</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>KPMG Consulting Co., Ltd.</t>
+          <t>JSUG</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Gustavo Waldfogiel</t>
+          <t>Rajkishore Una</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>LAC HCM Head</t>
+          <t>President/CEO</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>SAP Argentina - Buenos Aires</t>
+          <t>GyanSys, Inc.</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Shashikant Walimbe</t>
+          <t>Bala Parameswara Rao Upadhyay…</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Vice President &amp; Global Head -…</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>LTM LIMITED</t>
+          <t>Stefanini, Inc.</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Julie Walker</t>
+          <t>Oscar Uribe</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Sr. Director, Enterprise Applicatio…</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Armstrong</t>
+          <t>EDUARDONO S A S</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Rob Wallace</t>
+          <t>SACHIN VAIDYA</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Senior Manager Digital &amp; In…</t>
+          <t>Director - Enterprise Commercial…</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Jaguarlandrover</t>
+          <t>Pfizer, Inc.</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Enzhou Wang</t>
+          <t>Jonathan VON RUEDEN</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Chief Technology Officer</t>
+          <t>Chief AI Officer</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>City of Tacoma</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>May Wang</t>
+          <t>Wagner Valentin</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Direc…</t>
+          <t>Director of Regulated Indust…</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
+          <t>SAP Brasil Ltda.</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Adam Warner</t>
+          <t>Jorge Valles Velásquez</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Cost Analyst</t>
+          <t>KMMP…</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Marathon Cheese Corporation</t>
+          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Kosuke Watanabe</t>
+          <t>Henri Vallet</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Senior Account Executive</t>
+          <t>VP Sales, Americas B2B</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>Mirakl</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Takashi Watanabe</t>
+          <t>Jeff Van Pelt</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>執行役員</t>
+          <t>Founder / Managing Dire…</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>JFE Systems,Inc.</t>
+          <t>Javelin Consulting</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Robert Watson</t>
+          <t>Meredith Van Wyk</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Sr Account Executive</t>
+          <t>Americas Field Partner…</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -5939,912 +5935,1686 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Ashley Waxman</t>
+          <t>Joris Van der Donck</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Strategic Sales Executive</t>
+          <t>Sr Manag…</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Aevitas IT LLC</t>
+          <t>Commscope Connectivity Belgium</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Christy Weaver</t>
+          <t>Vijay Varee</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Global Demand Generation Man…</t>
+          <t>Senior Manager</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Vertex, Inc.</t>
+          <t>Petsmart LLC</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Mike Weaver</t>
+          <t>Suman Varma</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Senior I…</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>True Commerce Inc. TrueCommerce</t>
+          <t>Cintas Corporation</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Chris Webster</t>
+          <t>Chris Vassalotti</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>SVP IT Strategy &amp; Architecture</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Ahold Delhaize</t>
+          <t>Opentext</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Matt Webster</t>
+          <t>Raju Vedala</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Director of…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Gardner White Furniture Co., Inc.</t>
+          <t>CES Business Technologies, LLC</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Patrick Weil</t>
+          <t>Asier Vega Sanchez</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Implementation Consultant</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Metrie Canada Ltd</t>
+          <t>Arkyn</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Sarah Weiler</t>
+          <t>Jennifer Veillon</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Manager, Busine…</t>
+          <t>Dir Project Controls</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Ball Horticultural Company</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Adam Werner</t>
+          <t>Ajay Reddy Velampudi</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>VP, Corporate Technology</t>
+          <t>Senior VP - Sa…</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Crocs, Inc.</t>
+          <t>Miracle Software Systems Inc.</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Maddie Werner</t>
+          <t>William Velastegui</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Director of Delivery Solutions</t>
+          <t>JEFE DE TI Y PR…</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Robra IT</t>
+          <t>Plasticaucho Industrial S.A.</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Katherine West</t>
-        </is>
-      </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>CX Account Executive</t>
-        </is>
-      </c>
+          <t>Rajiv Vemula</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr"/>
       <c r="C336" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>Cognizant Technology Solutions U.S. Corporat…</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Anja Wettling</t>
+          <t>Sundu Venkataramani</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Industry Val…</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>anuwo GmbH</t>
+          <t>SAP Industries (Washington DC)</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Charleen Wetzstein</t>
+          <t>Venkat Venkataramani</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>SAP Principal Architect</t>
+          <t>VP</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>PROSPECTOR, LLC</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Peter Wheatley</t>
+          <t>Tom Venner-Crysell</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Enterprise Architect…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>SAP America (Houston)</t>
+          <t>ERPeople Solutions Ltd</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Robb White</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr"/>
+          <t>Eduardo Vergara</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+          <t>Agrosuper S.A.</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Peter Widmer</t>
+          <t>Amit Verma</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Chief of Staff to the Global Head of S…</t>
+          <t>RVP, Head of CFO Advisory…</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Chad Wiech</t>
+          <t>Kumar Vidit</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Director of Solution…</t>
+          <t>Product Marketing M…</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>SAP America(Bellevue)</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Chamnida Wijetilleke</t>
+          <t>Lakshmi Vidyashankar</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>VP of IT</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>The Ducats Group LLC</t>
+          <t>Marvin Engineering Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Pete Wilkins</t>
+          <t>Jayant Vikram</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>NA Partner Manager</t>
+          <t>Cloud Delivery Lead</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>Accenture LLP</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Mark Willey</t>
+          <t>Yeni Villanueva</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Vice…</t>
+          <t>Supervisora…</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+          <t>Compañia Minera Antamina S.A.</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Ed Williamson</t>
+          <t>Robert Vinyard</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Client Services Lead</t>
+          <t>VP and Senior Partner</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>XMATERIA LTD</t>
+          <t>IBM</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Monica Willis</t>
+          <t>Thomas Vioux</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>HR Strategy and Value A…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Plano- Legacy West</t>
+          <t>PwC</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Charlotte Wilson</t>
+          <t>Anil Visal</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Senior Manager Strategic Cha…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Direct Energy</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Emily Wisemiller</t>
+          <t>Clara Viscido</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>Consulting Services Director</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>GEONOSIS</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Julia Wolfe</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>Analyst Relations Manager</t>
-        </is>
-      </c>
+          <t>Paulo Vita Vita</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr"/>
       <c r="C350" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Jennifer Workman</t>
+          <t>Ranjan Vitt</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Techn…</t>
+          <t>AI Compliance Governance Program…</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Universal Destinations &amp; Experiences</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Steven Wright Wright</t>
+          <t>Jose Voisin</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>VP Sales</t>
+          <t>Global CIO</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Acuiti Labs Limited</t>
+          <t>Carmeuse</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Monty Wurth</t>
+          <t>Christina Volk</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>VP of Operations</t>
+          <t>Head of Strate…</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Optima Consulting L.L.C.</t>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Brad Wylie</t>
+          <t>Jessica Voyles</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Account Executive</t>
+          <t>Account Executive, South</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>KAORI YASHIKI</t>
+          <t>Sandeep Vyas</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Business Resear…</t>
+          <t>Solutio…</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services LLC</t>
+          <t>Incture Technologies Private Limited</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>YOUNGHO YOO</t>
+          <t>Thomas von Alm</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Team Leader</t>
+          <t>SVP Cross-Solution Services</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>LG CNS Co., Ltd.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Mohamed YUSUF</t>
+          <t>Markus von Quast</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Head of Integrated Toolchain</t>
+          <t>Global Head Industry Ecosystem</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Hikaru Yafuso</t>
+          <t>TATSUO WATANABE</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Senior Alliance Director</t>
+          <t>Principal Cons…</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>D I SQUARE CORPORATION.</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Sonoko Yamamoto</t>
+          <t>Masayuki Wada</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Partner Business Manager</t>
+          <t>SVP, Head of Corporate Digit…</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>Fujitsu Limited</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Osamu Yamazaki</t>
+          <t>Stephen Wagenheim</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Co…</t>
+          <t>Senior Sales Executive - Suppl…</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+          <t>Dallas (Allen)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Kenji Yanagi</t>
+          <t>Neha Wahi</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Group Leader</t>
+          <t>Global Alliance Lead</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>ASAHI GROUP JAPAN, LTD.</t>
+          <t>A.T. Kearney, Inc.</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>EJ Yang</t>
+          <t>Waka Wakabayashi</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>IT Deputy Director</t>
+          <t>Associate Partner</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>MediaTek Inc.</t>
+          <t>KPMG Consulting Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Kiran Yarlagadda Yarlagadda</t>
+          <t>Gustavo Waldfogiel</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Managing…</t>
+          <t>LAC HCM Head</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Adroix Corp DBA CodeForce 360</t>
+          <t>SAP Argentina - Buenos Aires</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Takayuki Yasuda</t>
+          <t>Shashikant Walimbe</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>Vice President &amp; Global Head -…</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>JFE Systems, Inc.</t>
+          <t>LTM LIMITED</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Tomoki Yasuda</t>
+          <t>Julie Walker</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>AssistantMana…</t>
+          <t>Sr. Director, Enterprise Applicatio…</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>NTT DATA Japan Corporation</t>
+          <t>Armstrong</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Kazuhiro Yonekawa</t>
+          <t>Rob Wallace</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Chief/Proj…</t>
+          <t>Senior Manager Digital &amp; In…</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>CANON MARKETING JAPAN INC.,</t>
+          <t>Jaguarlandrover</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>Sungeui Yoon</t>
+          <t>Enzhou Wang</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Senior Specialist</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>City of Tacoma</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>Christopher Yope</t>
+          <t>May Wang</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>SAP Supply C…</t>
+          <t>Direc…</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>DXC Technology Services LLC</t>
+          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>Kohei Yoshimatsu</t>
+          <t>Adam Warner</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cost Analyst</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>アズビル株式会社</t>
+          <t>Marathon Cheese Corporation</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>taichi yoshida</t>
+          <t>Kosuke Watanabe</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Senior Ma…</t>
+          <t>Senior Account Executive</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>BENIC SOLUTION CORPORATION</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>nakajima yuki</t>
+          <t>Takashi Watanabe</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Member</t>
+          <t>執行役員</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Nitori Co., Ltd.</t>
+          <t>JFE Systems,Inc.</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>Stefan Zach</t>
+          <t>Robert Watson</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>VP Global IT</t>
+          <t>Sr Account Executive</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Wieland Group</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>Beau Zaremski</t>
+          <t>Ashley Waxman</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>VP of Sales</t>
+          <t>Strategic Sales Executive</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Aevitas IT LLC</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Yuan Zhang</t>
+          <t>Christy Weaver</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Senior Project Manager, SAP AI RIG</t>
+          <t>Global Demand Generation Man…</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Vertex, Inc.</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Cathy Zhou</t>
+          <t>Mike Weaver</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>IT Director, EBS</t>
+          <t>Senior I…</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Ecolab Inc.</t>
+          <t>True Commerce Inc. TrueCommerce</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Gustavo Zintak</t>
+          <t>Chris Webster</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>SVP IT Strategy &amp; Architecture</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>SWISS MEDICAL S.A.</t>
+          <t>Ahold Delhaize</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Alina Zuberi</t>
+          <t>Matt Webster</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Global Content Strategist</t>
+          <t>Director of…</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>Gardner White Furniture Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Yoshiaki Agata 縣</t>
+          <t>Patrick Weil</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>consultant</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>AJS株式会社</t>
+          <t>Metrie Canada Ltd</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>裕紀 阿保</t>
+          <t>Sarah Weiler</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Manager, Busine…</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>FORTIENCE CONSULTING INC.</t>
+          <t>Ball Horticultural Company</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
+          <t>Adam Werner</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>VP, Corporate Technology</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Crocs, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Maddie Werner</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Director of Delivery Solutions</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Robra IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Katherine West</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>CX Account Executive</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Anja Wettling</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>anuwo GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Charleen Wetzstein</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>SAP Principal Architect</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>PROSPECTOR, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Peter Wheatley</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Enterprise Architect…</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Robb White</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr"/>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Peter Widmer</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the Global Head of S…</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Chad Wiech</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Director of Solution…</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Chamnida Wijetilleke</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>The Ducats Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Pete Wilkins</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>NA Partner Manager</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>SAP America(Bellevue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Mark Willey</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Vice…</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Ed Williamson</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Client Services Lead</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>XMATERIA LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Monica Willis</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>HR Strategy and Value A…</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Plano- Legacy West</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Charlotte Wilson</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Senior Manager Strategic Cha…</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Direct Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Emily Wisemiller</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Sr. Data Analyst</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Molex</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Julia Wolfe</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Analyst Relations Manager</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Jennifer Workman</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Techn…</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Universal Destinations &amp; Experiences</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Steven Wright Wright</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>VP Sales</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Monty Wurth</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>VP of Operations</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Optima Consulting L.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Brad Wylie</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>KAORI YASHIKI</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Business Resear…</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Hitachi Digital Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>YOUNGHO YOO</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Team Leader</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>LG CNS Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Mohamed YUSUF</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Head of Integrated Toolchain</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Hikaru Yafuso</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Senior Alliance Director</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Sonoko Yamamoto</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Partner Business Manager</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Osamu Yamazaki</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Co…</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Kenji Yanagi</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Group Leader</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>ASAHI GROUP JAPAN, LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>EJ Yang</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>IT Deputy Director</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>MediaTek Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Kiran Yarlagadda Yarlagadda</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Managing…</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Adroix Corp DBA CodeForce 360</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Takayuki Yasuda</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>JFE Systems, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Tomoki Yasuda</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>AssistantMana…</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Kazuhiro Yonekawa</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Chief/Proj…</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>CANON MARKETING JAPAN INC.,</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Sungeui Yoon</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Senior Specialist</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Christopher Yope</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>SAP Supply C…</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>DXC Technology Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Kohei Yoshimatsu</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>アズビル株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>taichi yoshida</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Senior Ma…</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>nakajima yuki</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Nitori Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Stefan Zach</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>VP Global IT</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Wieland Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Beau Zaremski</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Yuan Zhang</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Senior Project Manager, SAP AI RIG</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Cathy Zhou</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>IT Director, EBS</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Gustavo Zintak</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>SWISS MEDICAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Alina Zuberi</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Global Content Strategist</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Yoshiaki Agata 縣</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>consultant</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>AJS株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>裕紀 阿保</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>FORTIENCE CONSULTING INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
           <t>謙介 青木</t>
         </is>
       </c>
-      <c r="B380" t="inlineStr">
+      <c r="B426" t="inlineStr">
         <is>
           <t>Manager, Uvance Market Developme…</t>
         </is>
       </c>
-      <c r="C380" t="inlineStr">
+      <c r="C426" t="inlineStr">
         <is>
           <t>Fujitsu</t>
         </is>

</xml_diff>

<commit_message>
Add earlier S section attendees (Sh-Si)
Inserts 11 entries (Olga Shumikhina through Natalie Singh) before
Sukhbir Singh. Total now 436. No duplicates.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C426"/>
+  <dimension ref="A1:C437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4285,493 +4285,497 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Sukhbir Singh</t>
+          <t>Olga Shumikhina</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>S…</t>
+          <t>Umoja HCM Team Lead</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>The School Board of Duval County Florida</t>
+          <t>The United Nations</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Vikrant Sisodia</t>
+          <t>Andrew Sigler</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Sr. Product Manager</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Autodesk, Inc.</t>
+          <t>Syntax Systems USA LP</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>David Smith</t>
+          <t>Mikolaj Sikorski</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>VP, Chief Enterprise Ar…</t>
+          <t>Strategic Partner Initiatives</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>SAP America (Reston)</t>
+          <t>SAP Ireland Ltd.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Rachel Smith</t>
+          <t>Jonathan Silva</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Partner Sales Manager</t>
+          <t>Instituição de Pagament…</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Docusign Inc</t>
+          <t>Nu Pagamentos S.A</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Mark Smysor</t>
+          <t>Renato Silva</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Business Systems Analyst in Enterpri…</t>
+          <t>Solutions Sa…</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Globant Brasil Consultoria Ltda</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Delaiah Snowden</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>IT Ana…</t>
-        </is>
-      </c>
+          <t>Sergei Silva</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr"/>
       <c r="C234" t="inlineStr">
         <is>
-          <t>South Florida Water Management Dist</t>
+          <t>Vistex</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Jairo Soares De Matos</t>
+          <t>Felix Silvagnoli</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Analyst - SAP Busi…</t>
+          <t>SAP Platform Owner</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Canadian Blood Services</t>
+          <t>BP International Limited</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Michael Somerville</t>
+          <t>Gianluca Simeone</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Sales Executive</t>
+          <t>Global SAP CTIO &amp; AI Leader</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Checkout.com</t>
+          <t>Capgemini</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>YoonWon Song</t>
+          <t>Cintia Simonelli</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Managing Part…</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>i-SENS, Inc.</t>
+          <t>SAP Argentina - Buenos Aires</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Dag Terje Sorlie</t>
+          <t>Eric Simonson</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Director - Product Marke…</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Thiago Souza</t>
+          <t>Natalie Singh</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>IT CO…</t>
+          <t>Global Strategic Scale L…</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>MINERACAO SERRAS DO OESTE LTDA</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Meik Spanowsky</t>
+          <t>Sukhbir Singh</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>S…</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers LLP</t>
+          <t>The School Board of Duval County Florida</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Thorsten Spihlmann</t>
+          <t>Vikrant Sisodia</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Head of Business Development for T…</t>
+          <t>Sr. Product Manager</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Autodesk, Inc.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>TD Srinivasan</t>
+          <t>David Smith</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Industry…</t>
+          <t>VP, Chief Enterprise Ar…</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>SAP Public Services, Inc. (Hudson Y</t>
+          <t>SAP America (Reston)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Mike Stafford</t>
+          <t>Rachel Smith</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Senior ABAP Developer</t>
+          <t>Partner Sales Manager</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Titan Ventures LLC</t>
+          <t>Docusign Inc</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Jennifer Stapleton</t>
+          <t>Mark Smysor</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>VP of Accounting Strategy &amp;…</t>
+          <t>Business Systems Analyst in Enterpri…</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>American Equity</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>John Stark</t>
+          <t>Delaiah Snowden</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Global Head of SAP Alliance</t>
+          <t>IT Ana…</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Loftware</t>
+          <t>South Florida Water Management Dist</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Denis Staudt</t>
-        </is>
-      </c>
-      <c r="B246" t="inlineStr"/>
+          <t>Jairo Soares De Matos</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Analyst - SAP Busi…</t>
+        </is>
+      </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>GLOBAL DISTRIBUIÇÃO DE BENS DE CONSU…</t>
+          <t>Canadian Blood Services</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Maximilian Stein</t>
+          <t>Michael Somerville</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>SAP Product Owner - Treasury CPIT</t>
+          <t>Sales Executive</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Checkout.com</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Amanda Steiner</t>
+          <t>YoonWon Song</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Business Process Architect</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>McKesson</t>
+          <t>i-SENS, Inc.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Dieter Steinmann</t>
-        </is>
-      </c>
-      <c r="B249" t="inlineStr"/>
+          <t>Dag Terje Sorlie</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Fraport AG Frankfurt Airport Services Worldwi…</t>
+          <t>Accenture</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Jorrit Steinz</t>
+          <t>Thiago Souza</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>IT CO…</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ChannelEngine.com</t>
+          <t>MINERACAO SERRAS DO OESTE LTDA</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Robert Stemmler</t>
+          <t>Meik Spanowsky</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Global Alliances &amp; Ec…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Yonathan Stephanos</t>
+          <t>Thorsten Spihlmann</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>SAP Data &amp; AI Business Group Le…</t>
+          <t>Head of Business Development for T…</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Patrick Stewart</t>
+          <t>TD Srinivasan</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Account Executive</t>
+          <t>Industry…</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>SAP Public Services, Inc. (Hudson Y</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Jochen Stiebe</t>
+          <t>Mike Stafford</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Head of Sales Treas…</t>
+          <t>Senior ABAP Developer</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Target-Networks GmbH</t>
+          <t>Titan Ventures LLC</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Leslie Stoffel</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr"/>
+          <t>Jennifer Stapleton</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>VP of Accounting Strategy &amp;…</t>
+        </is>
+      </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>CARMEUSE RESEARCH AND TECHNOLOGY S…</t>
+          <t>American Equity</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Miodrag Stojanov</t>
+          <t>John Stark</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Lead Engineer</t>
+          <t>Global Head of SAP Alliance</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>SEMOS SOFTWARE LLC</t>
+          <t>Loftware</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Bojana Stojanovich</t>
-        </is>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>VP, NA Strategic Partnerships</t>
-        </is>
-      </c>
+          <t>Denis Staudt</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr"/>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Tricentis</t>
+          <t>GLOBAL DISTRIBUIÇÃO DE BENS DE CONSU…</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Seda Strate</t>
+          <t>Maximilian Stein</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Partner Innovation Lead</t>
+          <t>SAP Product Owner - Treasury CPIT</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -4783,454 +4787,446 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Divya Struebing</t>
+          <t>Amanda Steiner</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Supply Chain Customer…</t>
+          <t>Business Process Architect</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>McKesson</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Kevin Stupp</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>Director S4 Platform</t>
-        </is>
-      </c>
+          <t>Dieter Steinmann</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr"/>
       <c r="C260" t="inlineStr">
         <is>
-          <t>The Hershey Company</t>
+          <t>Fraport AG Frankfurt Airport Services Worldwi…</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Harish Subramanian</t>
+          <t>Jorrit Steinz</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Principal Enterprise Arch…</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>ChannelEngine.com</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Marc Sudjian</t>
+          <t>Robert Stemmler</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Enterprise Architect, SAP So…</t>
+          <t>Global Alliances &amp; Ec…</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Bombardier Inc.</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Hirofumi Sugimoto</t>
+          <t>Yonathan Stephanos</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>SAP Data &amp; AI Business Group Le…</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ABeam Systems Ltd.</t>
+          <t>Accenture</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Michael Sukachev</t>
+          <t>Patrick Stewart</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Sr. EA</t>
+          <t>Account Executive</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Teranet Inc</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Som Suresh</t>
+          <t>Jochen Stiebe</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Man…</t>
+          <t>Head of Sales Treas…</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+          <t>Target-Networks GmbH</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Jain Sushant</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>Chief Revenue Officer, F&amp;S…</t>
-        </is>
-      </c>
+          <t>Leslie Stoffel</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr"/>
       <c r="C266" t="inlineStr">
         <is>
-          <t>SAP ASIA Pte Ltd</t>
+          <t>CARMEUSE RESEARCH AND TECHNOLOGY S…</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Scott Sutker</t>
+          <t>Miodrag Stojanov</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Vice President Customer Success…</t>
+          <t>Lead Engineer</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Alpharetta</t>
+          <t>SEMOS SOFTWARE LLC</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Mergenthaler Sven</t>
+          <t>Bojana Stojanovich</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Global Head of Strategic Central Ser…</t>
+          <t>VP, NA Strategic Partnerships</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Tricentis</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Jereme Swoboda</t>
+          <t>Seda Strate</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Segment Director</t>
+          <t>Partner Innovation Lead</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Avvale, Inc.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Debra Syring</t>
+          <t>Divya Struebing</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Senior IT Manager</t>
+          <t>Supply Chain Customer…</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Entegris, Inc.</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Kai Szatkowski</t>
+          <t>Kevin Stupp</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Head of Product Sales</t>
+          <t>Director S4 Platform</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Natuvion GmbH</t>
+          <t>The Hershey Company</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>MARCO TOMBOLINI</t>
+          <t>Harish Subramanian</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Global He…</t>
+          <t>Principal Enterprise Arch…</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>DOLCE &amp; GABBANA BEAUTY SRL</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>KAZUSHI TOYOMASU</t>
+          <t>Marc Sudjian</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Global Direct…</t>
+          <t>Enterprise Architect, SAP So…</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>MOL Chemical Tankers Pte Ltd</t>
+          <t>Bombardier Inc.</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Stacey Taborelli</t>
+          <t>Hirofumi Sugimoto</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Executive Business Partn…</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>ABeam Systems Ltd.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Ahmed Taher</t>
+          <t>Michael Sukachev</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Sr. EA</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Al Daajan Trading</t>
+          <t>Teranet Inc</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Chieko Takahata</t>
+          <t>Som Suresh</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Chief</t>
+          <t>Man…</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>BROTHER INDUSTRIES,LTD.</t>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Arai Takahiro</t>
+          <t>Jain Sushant</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Services Delivery Manag…</t>
+          <t>Chief Revenue Officer, F&amp;S…</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Eiji Takashina</t>
+          <t>Scott Sutker</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Associate Director</t>
+          <t>Vice President Customer Success…</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Kyndryl Japan KK</t>
+          <t>Alpharetta</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Tetsushi Takino</t>
+          <t>Mergenthaler Sven</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Global Head of Strategic Central Ser…</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>大和ハウス工業株式会社</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Makoto Tamura</t>
+          <t>Jereme Swoboda</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Alliance Group Director</t>
+          <t>Segment Director</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>FUJITSU LIMITED</t>
+          <t>Avvale, Inc.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Chiyuki Tanaka</t>
+          <t>Debra Syring</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Team leader</t>
+          <t>Senior IT Manager</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Recruit Co., Ltd.</t>
+          <t>Entegris, Inc.</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Steve Tanaka</t>
+          <t>Kai Szatkowski</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Sr Vice Presid…</t>
+          <t>Head of Product Sales</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Blommer Chocolate Company</t>
+          <t>Natuvion GmbH</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Yasuhiro Tanaka</t>
+          <t>MARCO TOMBOLINI</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Global He…</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Recuruit Co.,Ltd.</t>
+          <t>DOLCE &amp; GABBANA BEAUTY SRL</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Kristin Taner</t>
+          <t>KAZUSHI TOYOMASU</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Chief Marke…</t>
+          <t>Global Direct…</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Vortex Software Consulting, LLC</t>
+          <t>MOL Chemical Tankers Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Mitchell Tauer</t>
+          <t>Stacey Taborelli</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Services Account Execut…</t>
+          <t>Executive Business Partn…</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -5242,2379 +5238,2566 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Roxanna Tavares</t>
+          <t>Ahmed Taher</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Director, Gl…</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>The Nielsen Company (US), LLC.</t>
+          <t>Al Daajan Trading</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Theo Tavrides</t>
+          <t>Chieko Takahata</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Vice Presi…</t>
+          <t>Chief</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>NTT Data Business Solutions, Inc.</t>
+          <t>BROTHER INDUSTRIES,LTD.</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Jamie Taylor</t>
+          <t>Arai Takahiro</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Global VP, Strategic Partnerships</t>
+          <t>Services Delivery Manag…</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Meghan Taylor</t>
+          <t>Eiji Takashina</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Industry Account Ex…</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>Kyndryl Japan KK</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Samantha Taylor</t>
+          <t>Tetsushi Takino</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Senior Solutions Account Exec…</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>大和ハウス工業株式会社</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Sarah Taylor</t>
+          <t>Makoto Tamura</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Solution Advisor</t>
+          <t>Alliance Group Director</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>FUJITSU LIMITED</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Jorge Tercero</t>
+          <t>Chiyuki Tanaka</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Manager/H…</t>
+          <t>Team leader</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Asociacion Mutual Sancor Salud</t>
+          <t>Recruit Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Michael Teti</t>
+          <t>Steve Tanaka</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Sr Vice Presid…</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Carlisle Construction Materials</t>
+          <t>Blommer Chocolate Company</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Suji Thampi</t>
+          <t>Yasuhiro Tanaka</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>MINDSPRINT PTE. LTD.</t>
+          <t>Recuruit Co.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Le Thanh Phong</t>
+          <t>Kristin Taner</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Managing Direc…</t>
+          <t>Chief Marke…</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>FPT Japan Holdings Co., Ltd.</t>
+          <t>Vortex Software Consulting, LLC</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Michael Theis</t>
+          <t>Mitchell Tauer</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Senior Director, Healthcare Life Scien…</t>
+          <t>Services Account Execut…</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Icertis</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Rene Theriault</t>
+          <t>Roxanna Tavares</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>IT Program Director</t>
+          <t>Director, Gl…</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>BRP INC</t>
+          <t>The Nielsen Company (US), LLC.</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Barbara Thrasher</t>
+          <t>Theo Tavrides</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>SR STAFF ARCHITECT</t>
+          <t>Vice Presi…</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Tyson Foods, Inc.</t>
+          <t>NTT Data Business Solutions, Inc.</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Nissim Titan</t>
+          <t>Jamie Taylor</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Global VP, Strategic Partnerships</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>4CAST SYSTEMS LTD</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>James Tiwari</t>
+          <t>Meghan Taylor</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Industry Account Ex…</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Intellioz LLC</t>
+          <t>Pittsburgh, SAP America</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Shuhei Toba</t>
+          <t>Samantha Taylor</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Senior Solutions Account Exec…</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Business Engineering Corporation</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>John Tocci</t>
-        </is>
-      </c>
-      <c r="B302" t="inlineStr"/>
+          <t>Sarah Taylor</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Solution Advisor</t>
+        </is>
+      </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Cbs Corporate Business Solutions America In…</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Oliver Toloui</t>
+          <t>Jorge Tercero</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Director - AI…</t>
+          <t>Manager/H…</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Ibase Operations Corp Qualitest</t>
+          <t>Asociacion Mutual Sancor Salud</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Ray Toma</t>
+          <t>Michael Teti</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Senior Principal — Global Strategic Initia…</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>Carlisle Construction Materials</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Yuko Tominaga</t>
+          <t>Suji Thampi</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Research Writer</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Freelance</t>
+          <t>MINDSPRINT PTE. LTD.</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Laura Tozzo</t>
+          <t>Le Thanh Phong</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>AI Product Lead SAP IBP</t>
+          <t>Managing Direc…</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>FPT Japan Holdings Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Eero Traagel</t>
+          <t>Michael Theis</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Senior Director, Healthcare Life Scien…</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>IBM Canada Limited</t>
+          <t>Icertis</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Adam Trahan</t>
+          <t>Rene Theriault</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>IT Program Director</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>BRP INC</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Evgeny Treskin</t>
+          <t>Barbara Thrasher</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>SAP Alliances Director</t>
+          <t>SR STAFF ARCHITECT</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Argano</t>
+          <t>Tyson Foods, Inc.</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Chetan Tripathi</t>
+          <t>Nissim Titan</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>oCFO Adoption expert</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>4CAST SYSTEMS LTD</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Seshagiri Tripurana</t>
+          <t>James Tiwari</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Senior Director</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Johnson &amp; Johnson</t>
+          <t>Intellioz LLC</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Masaru Tsukahira</t>
+          <t>Shuhei Toba</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>TOKYO ELECTRON LIMITED.</t>
+          <t>Business Engineering Corporation</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Lindsay Tucker</t>
-        </is>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>Solution Consultant</t>
-        </is>
-      </c>
+          <t>John Tocci</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr"/>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Docusign</t>
+          <t>Cbs Corporate Business Solutions America In…</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Paul Turbes</t>
+          <t>Oliver Toloui</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Director - AI…</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>KPMG LLP</t>
+          <t>Ibase Operations Corp Qualitest</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Treaver Tyler</t>
+          <t>Ray Toma</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Tech…</t>
+          <t>Senior Principal — Global Strategic Initia…</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Meijer Great Lakes Limited Partnership</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Kotaro Ueda</t>
+          <t>Yuko Tominaga</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Chief Operating Officer</t>
+          <t>Research Writer</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>JSUG</t>
+          <t>Freelance</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Rajkishore Una</t>
+          <t>Laura Tozzo</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>President/CEO</t>
+          <t>AI Product Lead SAP IBP</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>GyanSys, Inc.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Bala Parameswara Rao Upadhyay…</t>
+          <t>Eero Traagel</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Associate Director</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Stefanini, Inc.</t>
+          <t>IBM Canada Limited</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Oscar Uribe</t>
+          <t>Adam Trahan</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>EDUARDONO S A S</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>SACHIN VAIDYA</t>
+          <t>Evgeny Treskin</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Director - Enterprise Commercial…</t>
+          <t>SAP Alliances Director</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Pfizer, Inc.</t>
+          <t>Argano</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Jonathan VON RUEDEN</t>
+          <t>Chetan Tripathi</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Chief AI Officer</t>
+          <t>oCFO Adoption expert</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>SAP</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Wagner Valentin</t>
+          <t>Seshagiri Tripurana</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Director of Regulated Indust…</t>
+          <t>Senior Director</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>SAP Brasil Ltda.</t>
+          <t>Johnson &amp; Johnson</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Jorge Valles Velásquez</t>
+          <t>Masaru Tsukahira</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>KMMP…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
+          <t>TOKYO ELECTRON LIMITED.</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Henri Vallet</t>
+          <t>Lindsay Tucker</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>VP Sales, Americas B2B</t>
+          <t>Solution Consultant</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Mirakl</t>
+          <t>Docusign</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Jeff Van Pelt</t>
+          <t>Paul Turbes</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Founder / Managing Dire…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Javelin Consulting</t>
+          <t>KPMG LLP</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Meredith Van Wyk</t>
+          <t>Treaver Tyler</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Americas Field Partner…</t>
+          <t>Tech…</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Meijer Great Lakes Limited Partnership</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Joris Van der Donck</t>
+          <t>Kotaro Ueda</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Sr Manag…</t>
+          <t>Chief Operating Officer</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Commscope Connectivity Belgium</t>
+          <t>JSUG</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Vijay Varee</t>
+          <t>Rajkishore Una</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Senior Manager</t>
+          <t>President/CEO</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Petsmart LLC</t>
+          <t>GyanSys, Inc.</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Suman Varma</t>
+          <t>Bala Parameswara Rao Upadhyay…</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Associate Director</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Cintas Corporation</t>
+          <t>Stefanini, Inc.</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Chris Vassalotti</t>
+          <t>Oscar Uribe</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Opentext</t>
+          <t>EDUARDONO S A S</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Raju Vedala</t>
+          <t>SACHIN VAIDYA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Director - Enterprise Commercial…</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>CES Business Technologies, LLC</t>
+          <t>Pfizer, Inc.</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Asier Vega Sanchez</t>
+          <t>Jonathan VON RUEDEN</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Implementation Consultant</t>
+          <t>Chief AI Officer</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Arkyn</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Jennifer Veillon</t>
+          <t>Wagner Valentin</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Dir Project Controls</t>
+          <t>Director of Regulated Indust…</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>SAP Brasil Ltda.</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Ajay Reddy Velampudi</t>
+          <t>Jorge Valles Velásquez</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Senior VP - Sa…</t>
+          <t>KMMP…</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Miracle Software Systems Inc.</t>
+          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>William Velastegui</t>
+          <t>Henri Vallet</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>JEFE DE TI Y PR…</t>
+          <t>VP Sales, Americas B2B</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Plasticaucho Industrial S.A.</t>
+          <t>Mirakl</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Rajiv Vemula</t>
-        </is>
-      </c>
-      <c r="B336" t="inlineStr"/>
+          <t>Jeff Van Pelt</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Founder / Managing Dire…</t>
+        </is>
+      </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Cognizant Technology Solutions U.S. Corporat…</t>
+          <t>Javelin Consulting</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Sundu Venkataramani</t>
+          <t>Meredith Van Wyk</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Industry Val…</t>
+          <t>Americas Field Partner…</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>SAP Industries (Washington DC)</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Venkat Venkataramani</t>
+          <t>Joris Van der Donck</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>Sr Manag…</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Commscope Connectivity Belgium</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Tom Venner-Crysell</t>
+          <t>Vijay Varee</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Senior Manager</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>ERPeople Solutions Ltd</t>
+          <t>Petsmart LLC</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Eduardo Vergara</t>
+          <t>Suman Varma</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Agrosuper S.A.</t>
+          <t>Cintas Corporation</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Amit Verma</t>
+          <t>Chris Vassalotti</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>RVP, Head of CFO Advisory…</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>SAP ASIA Pte Ltd</t>
+          <t>Opentext</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Kumar Vidit</t>
+          <t>Raju Vedala</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Product Marketing M…</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>CES Business Technologies, LLC</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Lakshmi Vidyashankar</t>
+          <t>Asier Vega Sanchez</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>VP of IT</t>
+          <t>Implementation Consultant</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Marvin Engineering Co., Inc.</t>
+          <t>Arkyn</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Jayant Vikram</t>
+          <t>Jennifer Veillon</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Cloud Delivery Lead</t>
+          <t>Dir Project Controls</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Accenture LLP</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Yeni Villanueva</t>
+          <t>Ajay Reddy Velampudi</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Supervisora…</t>
+          <t>Senior VP - Sa…</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Compañia Minera Antamina S.A.</t>
+          <t>Miracle Software Systems Inc.</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Robert Vinyard</t>
+          <t>William Velastegui</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>VP and Senior Partner</t>
+          <t>JEFE DE TI Y PR…</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Plasticaucho Industrial S.A.</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Thomas Vioux</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
+          <t>Rajiv Vemula</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr"/>
       <c r="C347" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Cognizant Technology Solutions U.S. Corporat…</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Anil Visal</t>
+          <t>Sundu Venkataramani</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Industry Val…</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers LLP</t>
+          <t>SAP Industries (Washington DC)</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Clara Viscido</t>
+          <t>Venkat Venkataramani</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Consulting Services Director</t>
+          <t>VP</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>GEONOSIS</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Paulo Vita Vita</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr"/>
+          <t>Tom Venner-Crysell</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
+          <t>ERPeople Solutions Ltd</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Ranjan Vitt</t>
+          <t>Eduardo Vergara</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>AI Compliance Governance Program…</t>
+          <t>Manager/Head of Dept</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Agrosuper S.A.</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Jose Voisin</t>
+          <t>Amit Verma</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Global CIO</t>
+          <t>RVP, Head of CFO Advisory…</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Carmeuse</t>
+          <t>SAP ASIA Pte Ltd</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Christina Volk</t>
+          <t>Kumar Vidit</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Head of Strate…</t>
+          <t>Product Marketing M…</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>SAP Deutschland SE &amp;Co.KG</t>
+          <t>SAP America(Bellevue)</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Jessica Voyles</t>
+          <t>Lakshmi Vidyashankar</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Account Executive, South</t>
+          <t>VP of IT</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>Marvin Engineering Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>Sandeep Vyas</t>
+          <t>Jayant Vikram</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Solutio…</t>
+          <t>Cloud Delivery Lead</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Incture Technologies Private Limited</t>
+          <t>Accenture LLP</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Thomas von Alm</t>
+          <t>Yeni Villanueva</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>SVP Cross-Solution Services</t>
+          <t>Supervisora…</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Compañia Minera Antamina S.A.</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Markus von Quast</t>
+          <t>Robert Vinyard</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Global Head Industry Ecosystem</t>
+          <t>VP and Senior Partner</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>IBM</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>TATSUO WATANABE</t>
+          <t>Thomas Vioux</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Principal Cons…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>D I SQUARE CORPORATION.</t>
+          <t>PwC</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Masayuki Wada</t>
+          <t>Anil Visal</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>SVP, Head of Corporate Digit…</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Fujitsu Limited</t>
+          <t>PricewaterhouseCoopers LLP</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Stephen Wagenheim</t>
+          <t>Clara Viscido</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Senior Sales Executive - Suppl…</t>
+          <t>Consulting Services Director</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Dallas (Allen)</t>
+          <t>GEONOSIS</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Neha Wahi</t>
-        </is>
-      </c>
-      <c r="B361" t="inlineStr">
-        <is>
-          <t>Global Alliance Lead</t>
-        </is>
-      </c>
+          <t>Paulo Vita Vita</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr"/>
       <c r="C361" t="inlineStr">
         <is>
-          <t>A.T. Kearney, Inc.</t>
+          <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Waka Wakabayashi</t>
+          <t>Ranjan Vitt</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Associate Partner</t>
+          <t>AI Compliance Governance Program…</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>KPMG Consulting Co., Ltd.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Gustavo Waldfogiel</t>
+          <t>Jose Voisin</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>LAC HCM Head</t>
+          <t>Global CIO</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>SAP Argentina - Buenos Aires</t>
+          <t>Carmeuse</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Shashikant Walimbe</t>
+          <t>Christina Volk</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Vice President &amp; Global Head -…</t>
+          <t>Head of Strate…</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>LTM LIMITED</t>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Julie Walker</t>
+          <t>Jessica Voyles</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Sr. Director, Enterprise Applicatio…</t>
+          <t>Account Executive, South</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Armstrong</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Rob Wallace</t>
+          <t>Sandeep Vyas</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Senior Manager Digital &amp; In…</t>
+          <t>Solutio…</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Jaguarlandrover</t>
+          <t>Incture Technologies Private Limited</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>Enzhou Wang</t>
+          <t>Thomas von Alm</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Chief Technology Officer</t>
+          <t>SVP Cross-Solution Services</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>City of Tacoma</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>May Wang</t>
+          <t>Markus von Quast</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Direc…</t>
+          <t>Global Head Industry Ecosystem</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>Adam Warner</t>
+          <t>TATSUO WATANABE</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Cost Analyst</t>
+          <t>Principal Cons…</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Marathon Cheese Corporation</t>
+          <t>D I SQUARE CORPORATION.</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>Kosuke Watanabe</t>
+          <t>Masayuki Wada</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Senior Account Executive</t>
+          <t>SVP, Head of Corporate Digit…</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>Fujitsu Limited</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>Takashi Watanabe</t>
+          <t>Stephen Wagenheim</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>執行役員</t>
+          <t>Senior Sales Executive - Suppl…</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>JFE Systems,Inc.</t>
+          <t>Dallas (Allen)</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>Robert Watson</t>
+          <t>Neha Wahi</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Sr Account Executive</t>
+          <t>Global Alliance Lead</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>A.T. Kearney, Inc.</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>Ashley Waxman</t>
+          <t>Waka Wakabayashi</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Strategic Sales Executive</t>
+          <t>Associate Partner</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Aevitas IT LLC</t>
+          <t>KPMG Consulting Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Christy Weaver</t>
+          <t>Gustavo Waldfogiel</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Global Demand Generation Man…</t>
+          <t>LAC HCM Head</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Vertex, Inc.</t>
+          <t>SAP Argentina - Buenos Aires</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Mike Weaver</t>
+          <t>Shashikant Walimbe</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Senior I…</t>
+          <t>Vice President &amp; Global Head -…</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>True Commerce Inc. TrueCommerce</t>
+          <t>LTM LIMITED</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Chris Webster</t>
+          <t>Julie Walker</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>SVP IT Strategy &amp; Architecture</t>
+          <t>Sr. Director, Enterprise Applicatio…</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Ahold Delhaize</t>
+          <t>Armstrong</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Matt Webster</t>
+          <t>Rob Wallace</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Director of…</t>
+          <t>Senior Manager Digital &amp; In…</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Gardner White Furniture Co., Inc.</t>
+          <t>Jaguarlandrover</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Patrick Weil</t>
+          <t>Enzhou Wang</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>IT Director</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Metrie Canada Ltd</t>
+          <t>City of Tacoma</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>Sarah Weiler</t>
+          <t>May Wang</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Manager, Busine…</t>
+          <t>Direc…</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Ball Horticultural Company</t>
+          <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>Adam Werner</t>
+          <t>Adam Warner</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>VP, Corporate Technology</t>
+          <t>Cost Analyst</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Crocs, Inc.</t>
+          <t>Marathon Cheese Corporation</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>Maddie Werner</t>
+          <t>Kosuke Watanabe</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Director of Delivery Solutions</t>
+          <t>Senior Account Executive</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Robra IT</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>Katherine West</t>
+          <t>Takashi Watanabe</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>CX Account Executive</t>
+          <t>執行役員</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>JFE Systems,Inc.</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>Anja Wettling</t>
+          <t>Robert Watson</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>Sr Account Executive</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>anuwo GmbH</t>
+          <t>SAP AMERICA, INC.</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>Charleen Wetzstein</t>
+          <t>Ashley Waxman</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>SAP Principal Architect</t>
+          <t>Strategic Sales Executive</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>PROSPECTOR, LLC</t>
+          <t>Aevitas IT LLC</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>Peter Wheatley</t>
+          <t>Christy Weaver</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Enterprise Architect…</t>
+          <t>Global Demand Generation Man…</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>SAP America (Houston)</t>
+          <t>Vertex, Inc.</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>Robb White</t>
-        </is>
-      </c>
-      <c r="B386" t="inlineStr"/>
+          <t>Mike Weaver</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Senior I…</t>
+        </is>
+      </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+          <t>True Commerce Inc. TrueCommerce</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>Peter Widmer</t>
+          <t>Chris Webster</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Chief of Staff to the Global Head of S…</t>
+          <t>SVP IT Strategy &amp; Architecture</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Ahold Delhaize</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>Chad Wiech</t>
+          <t>Matt Webster</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Director of Solution…</t>
+          <t>Director of…</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Pittsburgh, SAP America</t>
+          <t>Gardner White Furniture Co., Inc.</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>Chamnida Wijetilleke</t>
+          <t>Patrick Weil</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Managing Director</t>
+          <t>IT Director</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>The Ducats Group LLC</t>
+          <t>Metrie Canada Ltd</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Pete Wilkins</t>
+          <t>Sarah Weiler</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>NA Partner Manager</t>
+          <t>Manager, Busine…</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>SAP America(Bellevue)</t>
+          <t>Ball Horticultural Company</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>Mark Willey</t>
+          <t>Adam Werner</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Vice…</t>
+          <t>VP, Corporate Technology</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+          <t>Crocs, Inc.</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>Ed Williamson</t>
+          <t>Maddie Werner</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Client Services Lead</t>
+          <t>Director of Delivery Solutions</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>XMATERIA LTD</t>
+          <t>Robra IT</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>Monica Willis</t>
+          <t>Katherine West</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>HR Strategy and Value A…</t>
+          <t>CX Account Executive</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Plano- Legacy West</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>Charlotte Wilson</t>
+          <t>Anja Wettling</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Senior Manager Strategic Cha…</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Direct Energy</t>
+          <t>anuwo GmbH</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Emily Wisemiller</t>
+          <t>Charleen Wetzstein</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>SAP Principal Architect</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>PROSPECTOR, LLC</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>Julia Wolfe</t>
+          <t>Peter Wheatley</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Analyst Relations Manager</t>
+          <t>Enterprise Architect…</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>SAP America (Houston)</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>Jennifer Workman</t>
-        </is>
-      </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t>Techn…</t>
-        </is>
-      </c>
+          <t>Robb White</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr"/>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Universal Destinations &amp; Experiences</t>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>Steven Wright Wright</t>
+          <t>Peter Widmer</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>VP Sales</t>
+          <t>Chief of Staff to the Global Head of S…</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Acuiti Labs Limited</t>
+          <t>SAP SE</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>Monty Wurth</t>
+          <t>Chad Wiech</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>VP of Operations</t>
+          <t>Director of Solution…</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Optima Consulting L.L.C.</t>
+          <t>Pittsburgh, SAP America</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>Brad Wylie</t>
+          <t>Chamnida Wijetilleke</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Account Executive</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>SAP Canada</t>
+          <t>The Ducats Group LLC</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>KAORI YASHIKI</t>
+          <t>Pete Wilkins</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Business Resear…</t>
+          <t>NA Partner Manager</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services LLC</t>
+          <t>SAP America(Bellevue)</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>YOUNGHO YOO</t>
+          <t>Mark Willey</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Team Leader</t>
+          <t>Vice…</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>LG CNS Co., Ltd.</t>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>Mohamed YUSUF</t>
+          <t>Ed Williamson</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Head of Integrated Toolchain</t>
+          <t>Client Services Lead</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>XMATERIA LTD</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Hikaru Yafuso</t>
+          <t>Monica Willis</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Senior Alliance Director</t>
+          <t>HR Strategy and Value A…</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Plano- Legacy West</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>Sonoko Yamamoto</t>
+          <t>Charlotte Wilson</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Partner Business Manager</t>
+          <t>Senior Manager Strategic Cha…</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>SAP Japan Co., Ltd.</t>
+          <t>Direct Energy</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>Osamu Yamazaki</t>
+          <t>Emily Wisemiller</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Co…</t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
+          <t>Molex</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>Kenji Yanagi</t>
+          <t>Julia Wolfe</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Group Leader</t>
+          <t>Analyst Relations Manager</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>ASAHI GROUP JAPAN, LTD.</t>
+          <t>IBM</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>EJ Yang</t>
+          <t>Jennifer Workman</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>IT Deputy Director</t>
+          <t>Techn…</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>MediaTek Inc.</t>
+          <t>Universal Destinations &amp; Experiences</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>Kiran Yarlagadda Yarlagadda</t>
+          <t>Steven Wright Wright</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Managing…</t>
+          <t>VP Sales</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Adroix Corp DBA CodeForce 360</t>
+          <t>Acuiti Labs Limited</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Takayuki Yasuda</t>
+          <t>Monty Wurth</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>VP of Operations</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>JFE Systems, Inc.</t>
+          <t>Optima Consulting L.L.C.</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Tomoki Yasuda</t>
+          <t>Brad Wylie</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>AssistantMana…</t>
+          <t>Account Executive</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>NTT DATA Japan Corporation</t>
+          <t>SAP Canada</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Kazuhiro Yonekawa</t>
+          <t>KAORI YASHIKI</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Chief/Proj…</t>
+          <t>Business Resear…</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>CANON MARKETING JAPAN INC.,</t>
+          <t>Hitachi Digital Services LLC</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Sungeui Yoon</t>
+          <t>YOUNGHO YOO</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Senior Specialist</t>
+          <t>Team Leader</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>LG CNS Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Christopher Yope</t>
+          <t>Mohamed YUSUF</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>SAP Supply C…</t>
+          <t>Head of Integrated Toolchain</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>DXC Technology Services LLC</t>
+          <t>SAP MENA LLC</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Kohei Yoshimatsu</t>
+          <t>Hikaru Yafuso</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Senior Alliance Director</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>アズビル株式会社</t>
+          <t>Databricks</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>taichi yoshida</t>
+          <t>Sonoko Yamamoto</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Senior Ma…</t>
+          <t>Partner Business Manager</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>BENIC SOLUTION CORPORATION</t>
+          <t>SAP Japan Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>nakajima yuki</t>
+          <t>Osamu Yamazaki</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Member</t>
+          <t>Co…</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Nitori Co., Ltd.</t>
+          <t>Hitachi Industry &amp; Control Solutions, Ltd.</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Stefan Zach</t>
+          <t>Kenji Yanagi</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>VP Global IT</t>
+          <t>Group Leader</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Wieland Group</t>
+          <t>ASAHI GROUP JAPAN, LTD.</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>Beau Zaremski</t>
+          <t>EJ Yang</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>VP of Sales</t>
+          <t>IT Deputy Director</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>SAP AMERICA, INC.</t>
+          <t>MediaTek Inc.</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>Yuan Zhang</t>
+          <t>Kiran Yarlagadda Yarlagadda</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Senior Project Manager, SAP AI RIG</t>
+          <t>Managing…</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Adroix Corp DBA CodeForce 360</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Cathy Zhou</t>
+          <t>Takayuki Yasuda</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>IT Director, EBS</t>
+          <t>sales</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Ecolab Inc.</t>
+          <t>JFE Systems, Inc.</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>Gustavo Zintak</t>
+          <t>Tomoki Yasuda</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Manager/Head of Dept</t>
+          <t>AssistantMana…</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>SWISS MEDICAL S.A.</t>
+          <t>NTT DATA Japan Corporation</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>Alina Zuberi</t>
+          <t>Kazuhiro Yonekawa</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Global Content Strategist</t>
+          <t>Chief/Proj…</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>SAP MENA LLC</t>
+          <t>CANON MARKETING JAPAN INC.,</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Yoshiaki Agata 縣</t>
+          <t>Sungeui Yoon</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>consultant</t>
+          <t>Senior Specialist</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>AJS株式会社</t>
+          <t>Microsoft</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>裕紀 阿保</t>
+          <t>Christopher Yope</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>SAP Supply C…</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>FORTIENCE CONSULTING INC.</t>
+          <t>DXC Technology Services LLC</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
+          <t>Kohei Yoshimatsu</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>アズビル株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>taichi yoshida</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Senior Ma…</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>nakajima yuki</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Nitori Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Stefan Zach</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>VP Global IT</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Wieland Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Beau Zaremski</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Yuan Zhang</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Senior Project Manager, SAP AI RIG</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Cathy Zhou</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>IT Director, EBS</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Gustavo Zintak</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Manager/Head of Dept</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>SWISS MEDICAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Alina Zuberi</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Global Content Strategist</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Yoshiaki Agata 縣</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>consultant</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>AJS株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>裕紀 阿保</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>FORTIENCE CONSULTING INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
           <t>謙介 青木</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr">
+      <c r="B437" t="inlineStr">
         <is>
           <t>Manager, Uvance Market Developme…</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr">
+      <c r="C437" t="inlineStr">
         <is>
           <t>Fujitsu</t>
         </is>

</xml_diff>

<commit_message>
Append 56 new R/S section contacts to attendees.xlsx
Merge the contacts extracted from the latest screenshots into
attendees.xlsx (now 548 entries). Marco Sanna was already present and
was skipped. Removes the temporary contacts.xlsx and extract script.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C493"/>
+  <dimension ref="A1:C549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1307,7 +1307,6 @@
           <t>Andreas Axer</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>WIRTGEN GROUP Branch of John Deere Gmb…</t>
@@ -1796,7 +1795,6 @@
           <t>Dan Berard</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>International Business Machines Corporation…</t>
@@ -2370,7 +2368,6 @@
           <t>Adam Breiterman</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
           <t>Maryland &amp; Virginia Milk Producers Cooperati…</t>
@@ -2502,7 +2499,6 @@
           <t>Jay Brown</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
           <t>ConsultingNetwork Business Solutions, LLC</t>
@@ -2753,7 +2749,6 @@
           <t>Erin Buss</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
           <t>Globalsource Information Technology III, Inc.</t>
@@ -3480,7 +3475,6 @@
           <t>Taiseer Chirakkal</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr"/>
       <c r="C181" t="inlineStr">
         <is>
           <t>International Business Machines Corporation…</t>
@@ -3714,7 +3708,6 @@
           <t>Zach Clement</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr"/>
       <c r="C195" t="inlineStr">
         <is>
           <t>American Equity Investment Li fe Insurance C…</t>
@@ -4288,7 +4281,6 @@
           <t>Marco Sanna</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr"/>
       <c r="C229" t="inlineStr">
         <is>
           <t>cbs Corporate Business Solutions Unternehm…</t>
@@ -4318,7 +4310,6 @@
           <t>Subhayu Sarkar</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr"/>
       <c r="C231" t="inlineStr">
         <is>
           <t>Cognizant Technology Solutions U.S. Corporat…</t>
@@ -5016,7 +5007,6 @@
           <t>Vice President, Information Technol…</t>
         </is>
       </c>
-      <c r="C272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -5160,7 +5150,6 @@
           <t>Tomoya Shinozaki</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr"/>
       <c r="C281" t="inlineStr">
         <is>
           <t>フォーティエンスコンサルティング株式会社…</t>
@@ -5309,7 +5298,6 @@
           <t>Sergei Silva</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr"/>
       <c r="C290" t="inlineStr">
         <is>
           <t>Vistex</t>
@@ -5696,7 +5684,6 @@
           <t>Denis Staudt</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr"/>
       <c r="C313" t="inlineStr">
         <is>
           <t>GLOBAL DISTRIBUIÇÃO DE BENS DE CONSU…</t>
@@ -5743,7 +5730,6 @@
           <t>Dieter Steinmann</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr"/>
       <c r="C316" t="inlineStr">
         <is>
           <t>Fraport AG Frankfurt Airport Services Worldwi…</t>
@@ -5841,7 +5827,6 @@
           <t>Leslie Stoffel</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr"/>
       <c r="C322" t="inlineStr">
         <is>
           <t>CARMEUSE RESEARCH AND TECHNOLOGY S…</t>
@@ -6636,7 +6621,6 @@
           <t>John Tocci</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr"/>
       <c r="C369" t="inlineStr">
         <is>
           <t>Cbs Corporate Business Solutions America In…</t>
@@ -7210,7 +7194,6 @@
           <t>Rajiv Vemula</t>
         </is>
       </c>
-      <c r="B403" t="inlineStr"/>
       <c r="C403" t="inlineStr">
         <is>
           <t>Cognizant Technology Solutions U.S. Corporat…</t>
@@ -7444,7 +7427,6 @@
           <t>Paulo Vita Vita</t>
         </is>
       </c>
-      <c r="B417" t="inlineStr"/>
       <c r="C417" t="inlineStr">
         <is>
           <t>Get Servicos de Gestao, Tecnologia e Particip…</t>
@@ -8052,7 +8034,6 @@
           <t>Robb White</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr"/>
       <c r="C453" t="inlineStr">
         <is>
           <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
@@ -8736,6 +8717,938 @@
       <c r="C493" t="inlineStr">
         <is>
           <t>Fujitsu</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>James Rasque</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>IT Business Analyst Supervisor</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Kwik Trip Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Abhishek Rastogi</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Lead Specialist, Business Cont...</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>National Grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Jeannine Rau</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>SCSM</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Koushika Ravikumar</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>KATBOTZ LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Prachi Ray</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Marketing - SAP</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Vasee Rayan</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Senior Vic...</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>SAP Labs, LLC. (Newtown Square)</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Carlos Recio</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Vice President Testing Practice</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Innovise IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Araja Reddy</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Deloitte Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Sasi Reddy</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Sr. SAP Applicati...</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Sun Chemical Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Nico Reichen</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr"/>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Caitlin Reidy</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr"/>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Icertis Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Kristen Reinken</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Journey &amp; Change Management L...</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Efrain Reyes</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>SAP Function...</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Aecon Construction Group Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Luis Reyes</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Regional Sales Director SSLATAM</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Vistex Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Dan Rhoadhouse</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Process Ar...</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>The Scotts Miracle-Gro Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Fernando Riccardi</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Exed Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Devin Rich</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Chief Info. Off.</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Lansing Building Products, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Trey Riley</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Leprino Foods Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Lisa Rinaldi</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Finance Lead, ED...</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>General Electric Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Angela Rios</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Centro de Sistemas y Negocios S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Jerome Robertson</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Director, AI Driven Business Insights</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Pfizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Lauren Robinson</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr"/>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Sparks</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Devin Robnick</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Head of NA Field Market...</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Virginia Roda</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Chief Technology Off</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Southbay S.R.L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Alexander Rodde</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Head of Corporate Portfolio</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Sebastian Rode</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Global ERP Delivery Lead</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Hernan Rodriguez</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Practice Manager</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Nearshore Argentina S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Josiane Roger</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>CGI Information Systems and Management C...</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Laurie Rogosheske</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Director E...</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Wolters Kluwer United States Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Rachel Romanoski</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Director - SAP SCM...</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Diana Romaya</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>SAP...</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>John Rooney</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Regional Partner Director</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Stonebranch</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Susanne Ross</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Senior Partner Marketin...</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Coveo Solutions Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Cori Rothgery</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Data &amp; A...</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>DURACELL U.S. OPERATIONS, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Sylvain Roy</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>It Director</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Heroux-Devtek</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Renee Rubino</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Senior Manager of Alliance Partnershi...</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>SMC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Felix Rubio</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Industry Advisor Latin America</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>SAP Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Frank Ruetten</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Client Partner</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>IBM Deutschland GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Frank Ruland</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr"/>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Roxanne Ryan</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Director, Executive Progr...</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Scott Ryerson</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Partner Executive</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Capgemini America, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Royce Ryu</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Head of Services Deliver...</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Natalie Röthel</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Executive Assistant</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>mariano rivarola</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Gerente Industrial Regional</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>HZ GROUP S.R.L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Hanumantha Rao Sabbireddy</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Tech Mahindra</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Andrew Sackett</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Director of Partnerships</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Collibra Belgium BV</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Rinchen Sahni</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Digital Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>KATBOTZ LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>KG Saito</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>MACNICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Makoto Saito</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>IT Development Dept</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Tokyo Electron Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Tito Salazar</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Partner Growth Manager</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>OneRail</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Sarah Salzman</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Regional VP of Sales</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Basware, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Julissa Samuels</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Gerente de aplica...</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>American Sportswear, S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Brent Sandberg</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Project Manager, Business Transf...</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Carmeuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Sachin Sangle</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>ImpactQA</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>KATSUYUKI SHINZEKI</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Assistant Manager</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Marubeni Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>JASBIR SINGH</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Associate Partner, Global...</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>IBM India Pvt Ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 55 new P/Q/R section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Pa-Py, Q, and Ra-
Rascoe. attendees.xlsx now has 603 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C549"/>
+  <dimension ref="A1:C604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8879,7 +8879,6 @@
           <t>Nico Reichen</t>
         </is>
       </c>
-      <c r="B503" t="inlineStr"/>
       <c r="C503" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
@@ -8892,7 +8891,6 @@
           <t>Caitlin Reidy</t>
         </is>
       </c>
-      <c r="B504" t="inlineStr"/>
       <c r="C504" t="inlineStr">
         <is>
           <t>Icertis Inc.</t>
@@ -9075,7 +9073,6 @@
           <t>Lauren Robinson</t>
         </is>
       </c>
-      <c r="B515" t="inlineStr"/>
       <c r="C515" t="inlineStr">
         <is>
           <t>Sparks</t>
@@ -9173,7 +9170,6 @@
           <t>Josiane Roger</t>
         </is>
       </c>
-      <c r="B521" t="inlineStr"/>
       <c r="C521" t="inlineStr">
         <is>
           <t>CGI Information Systems and Management C...</t>
@@ -9356,7 +9352,6 @@
           <t>Frank Ruland</t>
         </is>
       </c>
-      <c r="B532" t="inlineStr"/>
       <c r="C532" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
@@ -9649,6 +9644,937 @@
       <c r="C549" t="inlineStr">
         <is>
           <t>IBM India Pvt Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Mayur Patel</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Director IT COE</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Axalta Coating Systems, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Subhajit Paul</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>IT Technical Lead - SAP CoE</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Jabil Circuit, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Dan Pavlick</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Director of Strategic Partnerships</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>OneRail</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Matt Pegoraro</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Field Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Paul Pelletier</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Logistics Operatio...</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Defense Logistics Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Leila Penteado</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Value Advisor Head Brazil</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Rogério Peres</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>JBS USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Eddie Perez</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Master Producti...</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Marvin Engineering Co., Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Fernanda Perez</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>General Manag...</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>SAP Argentina - Buenos Aires</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>April Perkins</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Sr. Mgr. SAP...</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>thyssenkrupp Materials NA, Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Ernie Perno</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>St Account...</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>The Hackett Group- Answerthink</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Teresa Perrius</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Director, Payroll Operations</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>American Airlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Catherine Perry-Robertson</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Partner, Natio...</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Hari S. Peruri</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>AGCO Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>George Peter</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Sr Mgmt Business Sys</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Pure Storage Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Mark Petersen</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Sr...</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Advanced Workforce Inc DBA TotalTek Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Sladjana Petrovic</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>IGM Financial</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Jim Phelan</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>EVP, US Country M...</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>msg global solutions, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Matt Phillips</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Sr. Director</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Woodward Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Alex Pierroutsakos</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Industry Exec Advisor -...</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>SAP America (Miami)</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Dave Pinet</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Finance AE</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>SAP Canada - Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>James Pinto</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr"/>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>International Business Machines Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Peter Pluim</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>President, Global Cloud Op...</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>SAP UK Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Tomas Pluma</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>SCM Solution Advisory LAC</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>SAP Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Chris Podeszwa</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Principal Accoun...</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Alokai (ex - Vue Storefront)</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Franck Poisson</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>PWC US Group LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Eric Pokriefka</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Manager, Customer IT</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>DTE Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Michael Polaha</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>SR VP Record to Report</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>BlackLine</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Paula Popity</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Celco -...</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Celulosa Arauco y Constitucion S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Simone Porcu</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Karin Porwoll</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Global Strategic Partner Marketing SAP</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Raja Pothapragada</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Customer/Partner Success Man...</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Panaya, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Joel Pousinho</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Maxfield Group Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Andrea Powers</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Global Account Director</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Mediafly</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Stacy Price</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>IT Manager</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>American Airlines, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Whitney Price</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Director Supply Chain C...</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Brenda Prinzing</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Senior Co...</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>SAP America Inc. (Hudson Yards)</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Pascal Proulx</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>STI Maintenance inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Mark Pryor</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>VP Digital, M&amp;A+ERP</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>bp</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Manoj Purohit</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>SVP and Head of APAC Cor...</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>SAP ASIA Pte Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Joyce Purtell</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Vice President, Tax Tech...</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Angie Pyles</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>HCM Account Executive</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Plano- Legacy West</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Ashley Quinn</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Solution Architect</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Gentex Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Huzefa Qutbuddin</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Executive Vice President</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Royal Cyber Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>MANOJ KUMAR RAMALINGAM</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Senior Manager</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>CSL BEHRING LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>AMIT RANJAN</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Sr. Director IT Enterprise Applicat...</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Saputo Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Budi Rachman</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Predictive...</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Hamilton Prime International LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Arun Rajakani</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Architect - SAP Cloud</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>A.O. Smith Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Vishal Rajpal</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>VP Client Inn...</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Sutherland Global Services Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Kannan Ramanathan</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Director of Sales</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>SoftServe, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Rajesh Ramegowda Shankarappa</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Honeywell International Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Claudia Ramos</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Sales representative</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>724 BC Consulting SAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Warren Rampersaud</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Enterprise Account E...</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Liam Ranik</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Industry Account Executi...</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Paul Rascoe</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Janitor</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Beam Therapeutics</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 56 new N/O/P section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Na-Nu, O, and Pa-Pa
(through Brian Partlow). attendees.xlsx now has 659 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C604"/>
+  <dimension ref="A1:C660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10010,7 +10010,6 @@
           <t>James Pinto</t>
         </is>
       </c>
-      <c r="B571" t="inlineStr"/>
       <c r="C571" t="inlineStr">
         <is>
           <t>International Business Machines Corporation</t>
@@ -10575,6 +10574,954 @@
       <c r="C604" t="inlineStr">
         <is>
           <t>Beam Therapeutics</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Kazuto Nakada</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Territory Ecosystem Man...</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Yoshihiro Nakamura</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Chief Info. Off.</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>MAFTEC Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>KiWoong Nam</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Blueward inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Balachander Nandagopal</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Icertis, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Travis Nault</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>AscendN, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>DEBS Nayak</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Director — SAP...</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>INNOVAPTE CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Madhur Nayak</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>AI Architect</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Miracle Software Systems Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Sunny Neely</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Industry Advisor, Consu...</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Daniel Nersveen</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>PFERD-W...</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>August Rüggeberg GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>MJ Nevarez</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Planner/Scheduler</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Pantexas Deterrence LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Pamela Newberry</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Manager S4 Systems</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Collins Aerospace</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Albert Nguyen</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>VP Strategic Growth</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Qualitest</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Tom Nierlich</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>VP, Strategic Alliances</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Sovos</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Youssef Nifaoui</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Customer Success Mana...</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Jim Nissen</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Senior Program Manager</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Caterpillar Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Steve Noffke</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>American National Insurance</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Dongjin Noh</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Senior Professional</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Samsung Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Pavel Nouel</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Vice President,...</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Colgate-Palmolive Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Carlos Nunez</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>MDR</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Vendelux</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>matthew nasta</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>IT OTC Manager</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>S.C. Johnson &amp; Son, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Liz O'Neill</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Director, Business Deve...</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>DIBELL GROUP, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Conor O'Rourke</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>SAP Account Manager</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>ALKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Atilola Odeyemi Odeyemi</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Associate VP</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Africa Finance Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Halil Oezcelik</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Customer Officer</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Masayoshi Okita</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Hitachi, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Testuo Okuma</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Executive Partner</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>BAYCURRENT, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Hiroshi Okura</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>SAP Japan CFO</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Yuta Okuyama</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>IT person</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>NTTデータグループ</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Matt Olive</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Vice President of Sales</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>T S P</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Aleksandro Oliveira</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Grupo Edson Queiroz</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Cristian Olsen</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Chief Info. Off.</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Grupo Herman Zupan</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Andre Ory</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>OTS ERP Director</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>State of Louisiana</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Rauf Osho</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Senior SAP System E...</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>MIT Lincoln Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Catherine Ouellet</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Team Leader SAP Busine...</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Foliot Furniture Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Tatsuya Owada</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr"/>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>NIPPON STEEL Hitachi Systems Solutions, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Chad Owen</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Principal, Customer Success</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>msg Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Christine Owens</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Sr PM/ S/4HANA lead</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>e.l.f. Cosmetics, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Megha Oza</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Strategi...</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Splisys IT Consulting Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>HyunMo PARK</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>BizTech i Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Carlos Mauricio Pacheco Campan...</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Regional BRM</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Softtek</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Sachin Pai</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>SVP &amp; Global Head —...</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Celebal Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Shieun Paik</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Director IT</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Cardinal Health 200, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Ganesh Palanievelu</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Tech Mahindra</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Augusto Palma</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Executive Manager CoE SAP</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>HYPERA S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Rodolfo Pampin</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>BAITCON S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Joyce Pan</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Finance Manager</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>SAP (China) Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Debasis Panda</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Delivery Director</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Defense Logistics Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Carolina Paolini</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Business Readiness...</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Jaguar Land Rover Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Ravikiran Papthimar Papthimar</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Sr. Dire...</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Incture Technologies Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Keshav Parameshwara</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Senior Customer...</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>SAP LABS INDIA PVT. LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Fernando Pariani</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Chief In...</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>CENTRO MEDICO AMENABAR S.R.L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Adarsh Parikh</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Silver Touch Technologies Canada Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Edward Park</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Agent 008</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>National Amusements, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Sang-Yull Park</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Team Leader</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Woongjin Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Anfernee Parker</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Senior Account Executive</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Brian Partlow</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Assis...</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Medical College of Virginia Foundation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 57 new M/N section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Mc-My and the start
of N (through Sahiba Nagpaul). attendees.xlsx now has 716 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C660"/>
+  <dimension ref="A1:C717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11161,7 +11161,6 @@
           <t>Tatsuya Owada</t>
         </is>
       </c>
-      <c r="B639" t="inlineStr"/>
       <c r="C639" t="inlineStr">
         <is>
           <t>NIPPON STEEL Hitachi Systems Solutions, Inc.</t>
@@ -11522,6 +11521,967 @@
       <c r="C660" t="inlineStr">
         <is>
           <t>Medical College of Virginia Foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Jenny McLean</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Partner, Retail Industry...</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Clarkston Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Kathryn McLean McLean</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>BONFIRE CONSULTING LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Tommy McMullen</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>SAP Practice Lead</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Fidelis Companies LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>John McNally</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Senior Account Executive</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Tom McSorley</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>General Ma...</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>The Gill Corporation --Maryland</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Mark Meanwell</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Senior Manager Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Sylvamo</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Michael Meany</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Enterprise Account Exec...</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Shane Meehan</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Sr. Director</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>BioMarin Pharmaceutical, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Thomas Mehlkopf</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Head of Treasury and Working Capit...</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Nilay Mehta</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Principal Solution Archit...</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Mariana Melbardis</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr"/>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Price Waterhouse &amp; Co Asesores de Empresa...</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Emily Meltzer</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Developme...</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Accenture Federal Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Ritesh Menon</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Senior Vice President &amp; Business...</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Incture LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Janet Mercado</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Power &amp; Cloud Client Leader</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Katherine Merrick</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Supv IT Program M...</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Puget Sound Energy, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Monica Alejandra Mesa</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Team Lead SAP Projec</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Cementos Argos S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Ryan Mezzanotte</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>SAP Account Manager</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Alku, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Maya Midmore</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Industry Account Executive</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Lynn Mikoshi</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Joe Miles</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Life Sciences Industry Director</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>UI Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Patrick Miller</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Director - Enterprise Applicat...</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Cerapedics Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Rebecca Miller</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Acc. Operations Mgr.</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Purdue University</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Piyush Mistry</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Rich Mitton</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>IT Director</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Mathis Home</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>S Mohanavelu Mohanavelu</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>ERP solu...</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Gulfstream Aerospace Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Sanjeev Monga</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Kraft Heinz Foods Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Matt Monroe</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Sr. Services Account...</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Hyunsook Moon</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>DIRECTOR</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>BSG partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Brian Moore</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>SVP &amp; General Manager, Servic...</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Stephine Morbach</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr"/>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>American Equity Investment Life Insurance C...</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Dodjie Morelos</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Carlisle Construction Materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Abby Morgan</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Customer Engagement Manag...</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Visionsoft Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Lori Morgan</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>VP, Sales</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Ritsuo Moriya</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>SAP AMO</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Kobelco Systems Corp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Alex Moronta</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Gerente Soluciones...</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Pasteurizadora Rica S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Meir Morozov</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Enterprise Account Specialist</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Panaya, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Craig Moskowitz</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>SAP Program Director</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Empower</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Michael Moukeiber</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Molex, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Basant Mudgal</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Consultant, Business...</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Celebal Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Krish Mujje</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>SVP, Digital &amp; AI S...</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Tachyon Technologies LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Maximilian Mundel</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>VP Platform Sales</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Adyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Hanane Murakami</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>IBM Japan, Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Kentaro Murata</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Empl...</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>パナソニックインダストリー株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Wataru Murayama</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Sales Manager(Retail /...)</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Kylie Murphy</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Mar...</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>SAP Global Marketing(Newtown Square)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Craig Murray</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Business Transformation...</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Piramanayagam Muthusamy</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Global Head, SAP Te...</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Kishore Muthyala</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Miracle Software Systems Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Jay Myers</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Value Advisor</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Ariba Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Suzi Myers</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Director, Application Dev</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Cardinal Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Florian Müller</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Head of Security Product Manageme...</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>PRAKASH NARAYANAN</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Enterprise Account Executive</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Bristlecone, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Suresh NG</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>SAP Sales Specialist</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Wanda NI LAIGHIN</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Vice President, Global Marketing...</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>SAP France</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Kota Nagashio</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Man...</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>パナソニック インダストリー株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Masaki Nagata</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Consulting Divisi...</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>DI SQUARE CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Sahiba Nagpaul</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>AVP, SolEx &amp; Partner Success at I...</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Icertis, Inc.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 55 new L/M section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Lo-Ly and Ma-Mc
(through Patricia McKinley). attendees.xlsx now has 771 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C717"/>
+  <dimension ref="A1:C772"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11700,7 +11700,6 @@
           <t>Mariana Melbardis</t>
         </is>
       </c>
-      <c r="B671" t="inlineStr"/>
       <c r="C671" t="inlineStr">
         <is>
           <t>Price Waterhouse &amp; Co Asesores de Empresa...</t>
@@ -12019,7 +12018,6 @@
           <t>Stephine Morbach</t>
         </is>
       </c>
-      <c r="B690" t="inlineStr"/>
       <c r="C690" t="inlineStr">
         <is>
           <t>American Equity Investment Life Insurance C...</t>
@@ -12482,6 +12480,933 @@
       <c r="C717" t="inlineStr">
         <is>
           <t>Icertis, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Anand Lokineni</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Jabil Circuit, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Sergio Lopez</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>WINES AND SPIRITS S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Diego Loria</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Gerente de sistemas</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>MAINCAL S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Nathalie Lotra</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr"/>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Eli Lilly and Company Lilly Technology Center...</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Tammy Louie</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Senior Financial Systems Analyst</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>AutoZone</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Wepoint Louis</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Vice-President</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>ONEPOINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Lydia Lousky</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Supply Ch...</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>SAP America Inc. (Hudson Yards)</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Diego Lozano</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Seidor Consulting SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Jeroen Luijrink</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>SAP Nederland BV</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Michael Lukac</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Enterprise AE</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Adam Benjamin Lustig</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>VP, Solution Advisory</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Basware</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Bill Lynch</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Sr Director IT</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Sharp</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Thomas Lynch</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>VP, Value Advisory</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Nicolas Löwe</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>BearingPoint GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Ravish M</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Expert, Advanced Success Pl...</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>SAP MENA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>YOSHIHIRO MISAWA</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Managing Director General...</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>JFE Systems,Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>TIZIANA MOROSINI</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Corporate Marketing Events</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>SAP Italia S.p.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Santipriya Madabushi</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Sapta Global Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Sanjay Madala</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>SAP Competency...</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>ShimentoX Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Janet Maddern</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>ERP Program Manager</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>UT-Battelle LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Aaron Maestas</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Sr Director, Health Systems Natio...</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>McKesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Sergo Maglakelidze</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Director, Privat...</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>Evan Magouirk</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Manager, Pricing &amp; A...</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Souvik Majumdar</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Naresh Makhijani Makhijani</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Glo...</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Bob Marchand</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Innovise-IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Melissa Marchetti</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>SAP...</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>John Marcine</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Industry Account Executive</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Alan Martin</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Senior Solutions Sales E...</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Lawrence Martin</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Chief Product Officer an...</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Sascha Martin</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>SVP, Global H...</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>SAP Deutschland SE &amp; Co.KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Martine Martine</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Portefeuille Soucy Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Raphael Martins</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Sol...</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Seidor - Tecnologia da Informação LTDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Fernando Martins Salles</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>I...</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>AMBAR SERVICOS DE INFORMATICA LTDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>Takahiro Marufuji</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Dire...</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>MITSUBISHI CHEMICAL CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Shiho Maruta</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Team leader</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>（株）リクルート</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Adriana Masson</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Chicken Farmers of Ontario</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Tsuyoshi Masuda</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>VP and Head of RISE Ja...</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>Monika Matel-Sousa</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Deputy Chief Technology Offi...</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>City of Toronto</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>Deepak Mathur</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Medline Industries, LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>Nikhil Mathur</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Celebal Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>Doug Maulbetsch</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Director SAP applications</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Lucid Motors</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>Jared Mayers</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Acquisition Suppo...</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Pantexas Deterrence LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>Lia Mazmanian</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Marketing Execution Specialist</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>Nelia Mazula</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Supply Chain Sales Exec...</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Gerard McCann</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Strategic Allianc...</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Opentext Ot Addison Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Kevin McCollom</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Global VP, General Mgr.</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Archlynk, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Gerry McCool</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Value Advisor</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Michaelene McCormick</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Senior Services Account...</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Lauren McCullin</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Senior Sales Executive-...</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>John McDonnell</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Industry Advisor, Wholes...</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>Teresa McGivern</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Global Workforce Tranf...</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>PROFINDA LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Ben McGrail</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Managing director</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>XMATERIA LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>Denise McGuigan</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Part...</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Patricia McKinley</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr"/>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>CARMEUSE RESEARCH AND TECHNOLOGY S...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 57 new K/L section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Kr-Ky and La-Lo
(through Kirk Logan). attendees.xlsx now has 828 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C772"/>
+  <dimension ref="A1:C829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12540,7 +12540,6 @@
           <t>Nathalie Lotra</t>
         </is>
       </c>
-      <c r="B721" t="inlineStr"/>
       <c r="C721" t="inlineStr">
         <is>
           <t>Eli Lilly and Company Lilly Technology Center...</t>
@@ -13403,10 +13402,974 @@
           <t>Patricia McKinley</t>
         </is>
       </c>
-      <c r="B772" t="inlineStr"/>
       <c r="C772" t="inlineStr">
         <is>
           <t>CARMEUSE RESEARCH AND TECHNOLOGY S...</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Jan Krueger</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Technical Account Director</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Intel Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>Mike Krug</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>SAP Technical...</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Pennsylvania State University</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>Siddhi Kshatriya</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Organizational Change Managem...</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>AutoZone</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>Greg Kull</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Leader, SAP Partner Sales</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>Amit Kumar</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>SAP Pro...</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Molex Electronic Technologies, LLC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>Sandeep Kumar</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Partner [Data, Analytics &amp; AI]</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>SCMXpert</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>Jazz Kundra</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Amgen Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Sabrina Kunze</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Consulting Sen...</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>SAP Deutschland SE &amp;Co.KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>Trent Kurbis</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Manager, IT Service M...</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>The Mosaic Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>Makoto Kurimoto</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr"/>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>キヤノンマーケティングジャパン株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>Dennis Kurlandski</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>Kohei Kuroda</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Senior Consultant</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Fortience Consulting Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>Amir Kviatkovsky Kviatkovsky</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Panaya Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>Changhyeok Kwon</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Senior Professional</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Samsung Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Christina Kyriasoglou</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Tech Reporter</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Bloomberg LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Martin Kögel</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>VOQUZ Labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Arvind LAKSHMAN</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>IT Director</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>BioMerieux Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>JUNG HYUN LIM</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Group leader</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Blueward INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>Kun-Yi LIM</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Principal Tax Product...</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Autodesk Asia Pte Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>ROBSON LUIS DA CUNHA</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Invent Software Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Jonathan La Blunda</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Gerente Comercial Interpac...</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>INTERPACK S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Marc Laberge</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>SCM Solution Director</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>DBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Rosemary Lafferty</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Business Excellence...</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Americas Styrenics LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Brian Laird</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Exec...</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>SAP America Public Sec.(Newtown Sq)</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Nick Lake</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Digital and Innovation Manager - Logistics</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>JLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Vijay Lakhanpal</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>AVP - CLOUD I...</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Celebal Technologies Pvt Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Jose Luis Lanchas</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Global Events</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Nicholas Landolfi</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Customer Success Partner</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Ariba Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Mark Landrosh</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Industry Executive Advis...</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Joanne Lang</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Natuvion Americas, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Marcus Lange</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Global Partner Manager for S...</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Dynatrace LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Juan Carlos Lara</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>KMMP...</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Komatsu-Mitsui Maquinarias Peru S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Joseph Lattanzi</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Logistics Business Analyst</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Lincoln Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Sean Laughlin</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Product Marketing Direct...</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>George Lawrie</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Senior Dir...</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>SAP Industries (Newtown Square)</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Julian Lebowitz</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Director SAP and Busines...</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Centerra Gold Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Austin Ledesma</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Account Director</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Solace</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>DaeWon Lee</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Blueward inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Hye Jin Lee</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Woongjin Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Jang Moo Lee</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>System Engineer</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>LG CNS America Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Juhong Lee</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>SAP Korea Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Steven Leighton</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Head Digital &amp; Inn...</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Dan Lemashov</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Sr. Finance SSE</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Bobbi Lemoshov</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>IMS Trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Dave Leong</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Principle - High Tech Strategic Ac...</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Bristlecone</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>David Leslie</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Software Engineer in Test</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>FlightSafety</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>Brent Lewis</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Sr. Mgr. Data...</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Armstrong World Industries, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>Kelly Lewis</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Director SAP Ap...</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Brown-Forman Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Verena Leymann</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Vice President and Head of Corporat...</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>Al Limaye</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>LSInextGen</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Mara Lincoln</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Sr Sponsorship Engagement Direct...</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Freeman</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Robert Lindberg</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Director of Ent. Sys</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>CHS Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Angela Lipscomb</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>IT Manager</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>DTE Electric Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Andrew Little</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Canadian Blood Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Noelia Llobera</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Sasami</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Gwyneth Lloyd-Jones</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Accenture Japan Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Kirk Logan</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>VP Supply Chain, C...</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Pittsburgh, SAP America</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 55 new K section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Ka-Kr (through Gopal
Krishnan). attendees.xlsx now has 883 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C829"/>
+  <dimension ref="A1:C884"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13567,7 +13567,6 @@
           <t>Makoto Kurimoto</t>
         </is>
       </c>
-      <c r="B782" t="inlineStr"/>
       <c r="C782" t="inlineStr">
         <is>
           <t>キヤノンマーケティングジャパン株式会社</t>
@@ -14370,6 +14369,933 @@
       <c r="C829" t="inlineStr">
         <is>
           <t>Pittsburgh, SAP America</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Maruti Kampli</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Director - API Digital Integrations</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Miraclesoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Hideaki Kanamori</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Principal Project Manager</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Masaya Kanatani</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Project M...</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>BENIC SOLUTION CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Sandeep Kandirelli</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Tachyon Technologies LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>Nadine Kanja</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Global Head Industry Business Unit...</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>Saumya Kapoor</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Global Head of Sales, Planni...</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>SAP UK Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>Kiran Kumar Karanam</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>IT SAP</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>FlightSafety International Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>Eswar Karnam</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>ERP Associate Director</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Stefanini</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>Srinivas Karnati</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Director, Digital Tr...</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Tachyon Technologies LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>Srinu Karuturi</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>SCSM-Procurement</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>New York - Hudson Yards</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>Mariusz Karwowski</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>SAP Architect</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>SLAVIA CONSULTING LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>Vivek Kasera</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Associate Vice President</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Birlasoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>Sean Kask</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Chief AI Strategy Officer</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>SAP (Schweiz) AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>Sasi Kathirasen Mani</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>SENIOR VICE PRESIDE...</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>SAP Australia Pty Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>Chaz Kattamuri</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Client Partner</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>TSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>Tony Kavadas</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Chief Sales Officer</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Mediafly</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>JR Kavanagh</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Sr Account Exec - SCM</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>Masayoshi Kawase</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>AssistantMana...</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>Kentaro Kazama</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>SectionManager</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>JSOL Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Cristina Kazda</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Director of IT, Commercial</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Ecolab Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>Steve Kelchen</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Sr Account Executive</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>TotalTek</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>BlackJet Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>Sarah Kennedy</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>VP, SAP Services</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>Aisling Keogh</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Coveo Solutions Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Shigeki Keumi</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>BU Head, General Manager</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Hitachi Asia</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>George Kezhakekuttiyil</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>SBU Leader</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Cognizant</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Darshana Khadke</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>SAP Business Analyst</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>KNPC Holdco, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Junghyun Kim</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Samsung Electronics Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Ron King</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>VP, Sales Executive</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Deloitte Consulting LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Kaede Kitabatake</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Kyndryl Japan KK</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Hiroshi Kitano</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>EY Strategy and Consulting Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Adam Kiwon</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>whitepaper.id GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>Jason Klimas</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Functional An...</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Hellermanntyton Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>Jonathon Kline</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>EBS Deputy Portfo...</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Defense Logistics Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>Edward Kloczkowski</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Director of Information Te...</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Paul's Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>Candice Knauss</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr"/>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>American Equity Investment Life Insurance C...</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>Motoki Kobashi</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Director, PFC sales3</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>Faith Koch</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>HR Coordi...</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Basin Electric Power Cooperative</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>Gerard Koelmeyer</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Customer References</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>Christian Koestler</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Global Director, Client...</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>Hiroki Komine</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>JFE Systems,Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>Hiroki Komiyama</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Gen...</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>NTT DATA Global Solutions Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>Srikanth Kondagunta</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Information Systems Offi...</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>The United Nations</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>Brian Kooistra</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Facilities Syste...</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Exact Sciences Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>Chris Kornely</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Aflac, Incorporated</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>Chris Kosrow</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Donna</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>Mykola Kosyak</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>SAP Techn...</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>System Design Analysis (SDA) inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>Kotani Kotani</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>BROTHER INDUSTRIES,LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>Matt Kramer</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>VP, Supply Chain Manag...</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>Filip Kransfeld</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Practice Director</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Avvale Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>Stephan Kreipl</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Head of Product Management SAP I...</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>Joel Kremke</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>SVP, WW Partner Alliances &amp; Progr...</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>OpenText</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>Jens Kreuter</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Executive Communic...</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>zeit:raum digital GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>Libby Krider</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Sales Executive</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>TrueCommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>Gopal Krishnan</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr"/>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>INK IT Solutions and Consulting Private Limite...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 22 new J/K section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Je-Jä and Ka-Kam.
The remaining K screenshots showed contacts already added in earlier
batches. attendees.xlsx now has 905 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C884"/>
+  <dimension ref="A1:C906"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14973,7 +14973,6 @@
           <t>Candice Knauss</t>
         </is>
       </c>
-      <c r="B865" t="inlineStr"/>
       <c r="C865" t="inlineStr">
         <is>
           <t>American Equity Investment Life Insurance C...</t>
@@ -15292,10 +15291,375 @@
           <t>Gopal Krishnan</t>
         </is>
       </c>
-      <c r="B884" t="inlineStr"/>
       <c r="C884" t="inlineStr">
         <is>
           <t>INK IT Solutions and Consulting Private Limite...</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>Pam Jeffries</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr"/>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Cognizant Technology Solutions U.S. Corporat...</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>Sergey Jermakov</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Senior Partner</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>SIA Clarity Labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>Jessica Jestis</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Technology Manager</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Southwest Airlines Co.</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>Rajat Jetly</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>VP - Sales and BD</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>INNOVISE IT LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>Mithlesh Jha</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Managing p...</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Noshtek Consulting Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>Jim Thomas Jim</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr"/>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Wietersdorfer Finanz und Beteiligungs GmbH...</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>Jurema Johnson</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>ReleaseOwl</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>Vijay Johnwesley</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Sr Mgr SAP Delivery</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Leprino Foods Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>Brian Jones</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Services Partner Manager</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>Darius Jones</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Senior Value Advisor</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Sony Jose</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>FlightSafety International Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Sunny Joshi</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Regional Sales Leader</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Aaron Joy Joy</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Business Consultant</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Travis County, TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Kenneth Juengling</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Manager...</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Pennsylvania Turnpike Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Christian Jäkel</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Schwarz Digits</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>GYOYEON KIM</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Team Manager</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Blueward INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Kimikazu Kabata</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Solution Advisor Expert</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Jeremy Kahl</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Procureme...</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Los Alamos National Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>Yogi Kalra</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>INNOVAPTE CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>Armin Kaltenmeier</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Partner, Global Chief...</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Ernst &amp; Young U.S. LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>Dishank Kamath</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Program Manager</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>Ravi Kishore Kamma</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Principal Produc...</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>ReleaseOwl Private Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append Susan Cunningham to attendees.xlsx
The other 55 C-section contacts in the latest screenshots were already
present. attendees.xlsx now has 906 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C906"/>
+  <dimension ref="A1:C907"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15303,7 +15303,6 @@
           <t>Pam Jeffries</t>
         </is>
       </c>
-      <c r="B885" t="inlineStr"/>
       <c r="C885" t="inlineStr">
         <is>
           <t>Cognizant Technology Solutions U.S. Corporat...</t>
@@ -15384,7 +15383,6 @@
           <t>Jim Thomas Jim</t>
         </is>
       </c>
-      <c r="B890" t="inlineStr"/>
       <c r="C890" t="inlineStr">
         <is>
           <t>Wietersdorfer Finanz und Beteiligungs GmbH...</t>
@@ -15660,6 +15658,23 @@
       <c r="C906" t="inlineStr">
         <is>
           <t>ReleaseOwl Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>Susan Cunningham</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Senior Programmer / An...</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Unisys Corporation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 51 new G section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Ga-Gu (Anindya Gaine
through Timothy Guizon). attendees.xlsx now has 957 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C907"/>
+  <dimension ref="A1:C958"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15678,6 +15678,869 @@
         </is>
       </c>
     </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>Anindya Gaine</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Program Director SAP Imp...</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Fluor Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>Suresh Gali</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>IT Solutions Architect</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>NRG Energy, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>Francisco Galindo</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Sr Director IT finance</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Colgate Palmolive</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>George Galindo</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Account Director</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>SAP Industries, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>Glenn Gammon</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Director of S...</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>TLP Management Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>Joanne Gammon</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Partner Delivery Manager</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Ariba US Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>Suman Gandhe</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>FICO Consultant</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Siemens Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>Gary Gang</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Client Engagement Manag...</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>Javier Garcia</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Commercial Dir...</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Smartshift Technologies, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>Jose Garcia</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Sr. Director, SAP Practice Lead</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Nsight, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>Amit Garussi</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>VP Product</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Panaya Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>Patti Gary</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Senior Enterprise Architect</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Tyson Foods, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>Dino Gattola</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Senior Account Executive, Sup...</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>SAP CANADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>Boris Gebhardt</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Manager...</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>STARTEAM Global Germany GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>Frank Genevieve</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>SAP Sales Executive</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>NTT DATA Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>Brent George</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>SAP Advisor</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Tricentis GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>Jacob George</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Raytheon</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>Mark George</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Program Direct...</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Delaware North America LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>Eliza Georgescu</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Senior Manager, Partner...</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Collibra Belgium BV</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>Kimberly Gershenzon</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Finance Account Executi...</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>Deana Gervais</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Strategic Sales Support Specialist</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Pferd Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>Stefanie Geßler</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>SAP EWM Expert</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>4flow SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>Keya Gholap</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>KATBOTZ LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>Benedikt Gieger</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Strategic Projects, SAP SCM</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>Richard Gilbert</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Head of B2B Partner...</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Worldpay (UK) Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>Stacey Gilbert</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Merck</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>Don Gillespie</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Senior Director Strategic Alliances</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>ADP, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>Joe Golemba</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Global Head, Strategic Alliances...</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Vistex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>Raul Gomez</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>VP of IT</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Hexagon AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>Santiago Julian Gomez</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Supply Chain Regional Man...</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>INTERPACK S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>Moises Gonzalez</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Client Engagement Manag...</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>Oziel Gonzalez</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>VA Head Mexico</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>SAP Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>Nelson González</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Subgerente e Operaciones...</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Grupo Kaufmann</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>Senthil Gopalan</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>D-1 (SVP)</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>The United Nations</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>Pooven Govender</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>APAC CLOUD ARCHITE...</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>SAP Australia Pty Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>Christine Graham</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Chief Information Officer</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Lakeview Farms, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>Geoff Gray</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Head of Product</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>The Config Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>Andrew Greaves</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Sen...</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>SAPOCOM Technologies Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>Samuel Grenade</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr"/>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Coveo Solutions Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>Betsy Griffin</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Senior Account Executive</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>Paula Griffin</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Seni...</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Medical College of Virginia Foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>Nicole Griffith</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Sr. Director, SAP Alliance</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Protera</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>Tim Grochowski</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Senior Cloud Executive</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>Anette Grossmueller</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Head of Cross Product Management,...</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>Scott Groth</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Directir, ERP Architect</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Pfizer, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>John Grzybek</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Senior SAP Projec...</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Fujitsu North America, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>Rodolfo Guerrero</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Account Manager</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>GBM Dominicana</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>Alex Guglielmetti</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>VP - IT Advisor</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Pantexan Deterrence</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>Patricia Guillermo</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>It Lead</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Kellanova/Mars</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>Dmitri Guinzbourg</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Team Lead/Supervisor</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Air Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>Timothy Guizon</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Finance Manager</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Henry Company LLC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append 54 new H/I section contacts to attendees.xlsx
Adds entries from the latest screenshots covering Ha-Hy and Ia-In
(through Tatsuya Inagaki). Skipped a clearly-bogus entry "Attendee
test InPersonTestThree". attendees.xlsx now has 1011 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C958"/>
+  <dimension ref="A1:C1012"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16330,7 +16330,6 @@
           <t>Samuel Grenade</t>
         </is>
       </c>
-      <c r="B946" t="inlineStr"/>
       <c r="C946" t="inlineStr">
         <is>
           <t>Coveo Solutions Inc</t>
@@ -16538,6 +16537,916 @@
       <c r="C958" t="inlineStr">
         <is>
           <t>Henry Company LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>Sriram Hariharasubramanian</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Partner, Tech Consult...</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>EY Global Services Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>Lori Harner</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Global Vice President, Pr...</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>Melissa Harris</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>IT Program Manager</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Masco Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>Paul Harris</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Senior Director, SAP Basi...</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Varsity Brands, LLC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>Joe Hartnett</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>OpenText</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>Richard Hatton</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>VP Platform Engin...</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>NBCUniversal Media, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>Kishie Hattori</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Chief Partner Officer</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>Chelsea Hebb</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Director, Cons...</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Collective Insights Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>Heiko Hecht</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>IBIS America Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>Tess Heiligers</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Business Advisor to SVP ERP Tranfo...</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>BP P.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>Christian Heinrich</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Chief Solutions Officer &amp; Membe...</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>sovanta AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>Isabel Heinz</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Sales Consultant</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>anuwo GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>David Heitz</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Account Director</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>Nicolas Helmstaetter</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Treasury Expert</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>Frauke Hering</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Sovereign Cloud Portfolio Manager</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>Adriana Hernandez</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Head Architecture</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Bachoco, S.A. de C.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>Sergio Hernandez</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Head of IT Solutions Ma...</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>Valarie Hernandez</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Travis County, TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>Juan Manuel Hernandez Bello</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>GERENTE SERVICI...</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Organizacion Terpel S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>Ralph Hess</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Executive...</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Navigator Business Solutions, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>Chris Hilko</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Industry Account Executi...</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>Scott Hillhouse</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Industry Account Executi...</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>Brandon Hilton</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Enterprise Syst...</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Eastman Chemical Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>Kent Hinkemeyer</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr"/>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Wolters Kluwer Global Business Services B.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>Gary Hinton</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Managing Partner - Shell</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>SAP Nederland BV</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>David Hoag</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Sr. Manager IT SAP</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Builders Firstsource, Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>Stefan Hoffmann</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Vice President Strategy &amp; Soluti...</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Argano LLC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>Robert Holland</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Chief Re...</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Wellesley Information Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>Michael Hom</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Global Head of Digit...</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Jpmorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>Ricardo Honda</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Head of BTM Brazil</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>Keith Hontz</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Global Head of SAP Alliance</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Zscaler, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>Stuart Hooker</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr"/>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Shell Information Technology International B.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>Norma Hopkins</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>SLED Field Marketin...</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>SAP Canada - Waterloo</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>Jeffrey Hornibrook</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Erin Houston Houston</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>IT Solution Manager</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>MSA the Safety Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>Aaron Hovick</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Asst. Director</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Hy-Vee, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>Mike Howard</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Thinklogicx</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>Hector Hoz</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>VP Solution Advisory Spend...</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>SAP Brasil Ltda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>Haibo Huang</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>Holina Huang</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Head of CE&amp;A of CS&amp;D...</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>SAP Taiwan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>Yvania Huertas Vargas</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Manager/Head o...</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>Josh Hulme</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>VP of Sales</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>INSPYR Solutions, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>Jens Hungershausen</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Chairman of the Board</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>DSAG eV</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>Ryan Hurney</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Sr. Manager</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>DXC Technology Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Farheen Hussain</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Solution - Customer Suc...</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>Omar Hussein Olmedo</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Poject Manager</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Bachoco, S.A. de C.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>Jared Hyde</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>VP / Assistant GM, Project Phoenix</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>CRH</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>KAZUSHI INA</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>JFE Systems,Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>Manabu Ichinogo</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Senior Principal</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Open Text K.K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>TOSHIKATSU Ikeuchi</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>General...</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>NEC Networks &amp; System Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>Masakazu Imanaga</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Head of Process Industr...</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>Vincent Immordino</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Director, Private Equity &amp; Canada Sales</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Esker</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>Akari Inada</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>ABeam Systems Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>Tatsuya Inagaki</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Sony Global Solutions Inc.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append 23 new I/J section contacts to attendees.xlsx
Adds entries from the latest screenshots covering the rest of I (Al
Ingallinera Jr through Ken Ito) and Ja-Je (Morgan Jacob through Suneth
Jayawardhane). attendees.xlsx now has 1034 contacts.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1012"/>
+  <dimension ref="A1:C1035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16937,7 +16937,6 @@
           <t>Kent Hinkemeyer</t>
         </is>
       </c>
-      <c r="B982" t="inlineStr"/>
       <c r="C982" t="inlineStr">
         <is>
           <t>Wolters Kluwer Global Business Services B.V.</t>
@@ -17069,7 +17068,6 @@
           <t>Stuart Hooker</t>
         </is>
       </c>
-      <c r="B990" t="inlineStr"/>
       <c r="C990" t="inlineStr">
         <is>
           <t>Shell Information Technology International B.V.</t>
@@ -17447,6 +17445,397 @@
       <c r="C1012" t="inlineStr">
         <is>
           <t>Sony Global Solutions Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>Al Ingallinera Jr</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>VP, Product Management...</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Baton Simulations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>Babu Inti</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>CommScope, Inc. of North Carolina</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>Rick Isom</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Enterprise Architect</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>Ken Ito</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Division Manager</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>TIS Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>Morgan Jacob</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Director Enterprise</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>L B Foster Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>Amith Kumar Jada</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>SAP Progr...</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>Mahi Jadhav</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>QTC Transformation Man...</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>Chung JaePhil</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>SAP Korea Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>Andrew Jaehnig</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>SAP Manager</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>ALKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>Alon Jaffe</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>VP Fe...</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>SAP America Public Sec.(Washington)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>Anand Jain Jain</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>MD - Enterprise Technolo...</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Eisner and Amper</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>Mehga Jain</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Enterprise Architect - M...</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>SAP INDIA PVT. LTD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>Naren Jain</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Managing Dire...</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>Prateek Jain</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Lead Consultant</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Celebal Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>Soumyaa Jain</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Content Specialist</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Cognitus Consulting LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>Raj Jakhete</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Vice President, I...</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Oliver Healthcare Packaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>William Jan</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Senior Value Advisor</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>Nathan Janardhana</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Information Systems Offi...</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>The United Nations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>Lars Janitz</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Senior Exe...</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>NTT DATA Business Solutions AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>Brian Janzen</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>SVP, Continuous Impr...</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Graham Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>Jose Antonio Jaramillo</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Pyramid Consulting SAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>Pawel Jaroszewicz</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Senior Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Onapsis Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>Suneth Jayawardhane</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Senior Principal, Valu...</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>SAP America (Reston)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 54 G and H section contacts from screenshots
Appends 32 G-surname and 22 H-surname attendees extracted from provided
screenshots. None were previously present in the list.
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C493"/>
+  <dimension ref="A1:C547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8739,6 +8739,908 @@
         </is>
       </c>
     </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Sriram Hariharasubramanian</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Partner, Tech Consult…</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>EY Global Services Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Lori Harner</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Global Vice President, Pr…</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Melissa Harris</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>IT Program Manager</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Masco Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Paul Harris</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Senior Director, SAP Basi…</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Varsity Brands, LLC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Joe Hartnett</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>OpenText</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Richard Hatton</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>VP Platform Engin…</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>NBCUniversal Media, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Kishie Hattori</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Chief Partner Officer</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>SAP Japan Co., Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Chelsea Hebb</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Director, Cons…</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Collective Insights Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Heiko Hecht</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>IBIS America Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Tess Heiligers</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Business Advisor to SVP ERP Tranfo…</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>BP P.L.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Christian Heinrich</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Chief Solutions Officer &amp; Membe…</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>sovanta AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>VALERIAN HARRIS</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>HCL America Solutions Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Angie Halderman</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Vice President, Sales</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Sarah Haley-Fuentes</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Director of Solution Engineering</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Vistex Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Callie Hall</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr"/>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>SAP Global Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Deborah Hamilton</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Head of Global Marketing</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Bristlecone, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Joe Hamilton</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Sr. Director AME Mfg. Technology</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Honeywell</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Sean Hamlin</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Value Advisor</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Youngshin Han</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>IT Team Manager</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>i-SENS. Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Rebecca Hanna</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Head of Services, ANZ</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>SAP AUSTRALIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Manoj Harbhajanka</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Acuiti Labs Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Hadi Hares</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Global Lead Product Manager</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Ajay Gupta</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Mana…</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Reliance Comfort Limited Partnership</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Anupam Gupta Gupta</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Celebal Technologies Americas, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Niladri Gupta</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Deloitte Consulting LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Piyush Gupta</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Global Head -…</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Celebal Technologies Pvt Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Raj Gupta</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Intellioz LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Varun Gupta</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>American Water Works Service Company, Inc.…</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Vishal Gupta</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Head of Finance &amp; Spe…</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>SAP Australia Pty Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>David Gust</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Nestor Guzman</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Dire…</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Aerovias Del Continente Americano S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Kalman Gyula</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr"/>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Karthik Gobi gobimayilsamygound…</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Service Owner (…</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Honeywell International Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Nicole Griffith</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Sr. Director, SAP Alliance</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Protera</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Tim Grochowski</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Senior Cloud Executive</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Anette Grossmueller</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Head of Cross Product Management,…</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Scott Groth</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Directir, ERP Architect</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Pfizer, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>John Grzybek</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Senior SAP Projec…</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Fujitsu North America, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Rodolfo Guerrero</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Account Manager</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>GBM Dominicana</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Alex Guglielmetti</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>VP - IT Advisor</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Pantexan Deterrence</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Patricia Guillermo</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>It Lead</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Kellanova/Mars</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Dmitri Guinzbourg</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Team Lead/Supervisor</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Air Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Timothy Guizon</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Finance Manager</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Henry Company LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Moises Gonzalez</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Client Engagement Manag…</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Oziel Gonzalez</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>VA Head Mexico</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>SAP Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Nelson González</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Subgerente e Operaciones…</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Grupo Kaufmann</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Senthil Gopalan</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>D-1 (SVP</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>The United Nations</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Pooven Govender</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>APAC CLOUD ARCHITE…</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>SAP Australia Pty Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Christine Graham</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Chief Information Officer</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Lakeview Farms, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Geoff Gray</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Head of Product</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>The Config Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Andrew Greaves</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Sen…</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>SAPOCOM Technologies Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Samuel Grenade</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr"/>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Coveo Solutions Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Betsy Griffin</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Senior Account Executive</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Paula Griffin</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Seni…</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Medical College of Virginia Foundation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 50 F and G section contacts from screenshots
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C547"/>
+  <dimension ref="A1:C597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9641,6 +9641,856 @@
         </is>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Gordon Folz</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Bristlecone, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Sandra Liliana Forero Cifuentes</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>SAP Product Manag…</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Softtek Renovation SAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Nina Forlenza</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Team Lead, Senior HRBP</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>ADP, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Chris Foti</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Director, ISV Alliances</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Basware Oyj</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Jeff Foy</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Vice President, Supply C…</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Luciana Franquet</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Galicia Seguros S.A.U.</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Andreas Franz</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>He…</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Heraeus Consulting &amp; IT Solutions GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Tom Frederick</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>GlobalSource IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Alan Freedman</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>VP Sales - Central…</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>The Addmore Group Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Jeremy Freeman</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Director, Technology</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Aritzia</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Brian Freymann</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Director, SAP Strategic Acco…</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Bristlecone, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Patrick Friday</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Alokai</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Lionel Fridman</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>VP SCM MCLAC</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>SAP Argentina - Buenos Aires</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Joakim Frisberg</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Oliver Froehlich</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>SAP Partner Manager Europe</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Vertex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Takeshi Fukushima</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>大和ハウス工業株式会社</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Sean Furukawa</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Deputy CEO</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>BearingPoint NA LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Anindya Gaine</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Program Director SAP Imp…</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Fluor Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Suresh Gali</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>IT Solutions Architect</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>NRG Energy, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Francisco Galindo</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Sr Director IT finance</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Colgate Palmolive</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>George Galindo</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Account Director</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>SAP Industries, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Glenn Gammon</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Director of S…</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>TLP Management Services LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Joanne Gammon</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Partner Delivery Manager</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Ariba US Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Suman Gandhe</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>FICO Consultant</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Siemens Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Gary Gang</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Client Engagement Manag…</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Veritas Prime, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Javier Garcia</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Commercial Dir…</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Smartshift Technologies, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Jose Garcia</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Sr. Director, SAP Practice Lead</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Nsight, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Amit Garussi</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>VP Product</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Panaya Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Patti Gary</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Senior Enterprise Architect</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Tyson Foods, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Satyanarayana Gade</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Enterprise Archi…</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Simpson Strong-Tie Co., Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>NISHANT GAUTAM</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>www.innovise-it.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Dino Gattola</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Senior Account Executive, Sup…</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>SAP CANADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Boris Gebhardt</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Manager…</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>STARTEAM Global Germany GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Frank Genevieve</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>SAP Sales Executive</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>NTT DATA Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Brent George</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>SAP Advisor</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Tricentis GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Jacob George</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Raytheon</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Mark George</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Program Direct…</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Delaware North America LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Eliza Georgescu</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Senior Manager, Partner…</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Collibra Belgium BV</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Kimberly Gershenzon</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Finance Account Executi…</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Deana Gervais</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Strategic Sales Support Specialist</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Pferd Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Stefanie Geßler</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>SAP EWM Expert</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>4flow SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Keya Gholap</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>KATBOTZ LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Benedikt Gieger</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Strategic Projects, SAP SCM</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Richard Gilbert</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Head of B2B Partner…</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Worldpay (UK) Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Stacey Gilbert</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Merck</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Don Gillespie</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Senior Director Strategic Alliances</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>ADP, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Joe Golemba</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Global Head, Strategic Alliances…</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Vistex, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Raul Gomez</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>VP of IT</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Hexagon AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Santiago Julian Gomez</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Supply Chain Regional Man…</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>INTERPACK S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>SANJAY KUMAR GUPTA</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>VICE PRESIDENT</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Limited</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 25 E and F section contacts from screenshots
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1077"/>
+  <dimension ref="A1:C1102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18579,6 +18579,431 @@
         </is>
       </c>
     </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>Jennifer Ertler</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>Jose Esparza</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Director…</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>BFS Ingenieria Aplicada S.A. de C.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>Jose Manuel Estevz Estevez</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Technology Consulta…</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>EY Global Services Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>Brandon Evans</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Managing Dire…</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>SHIGEHIRO FUJIKI</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Chief Info…</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Mitsubishi Corporation (Americas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>SATOSHI FUJITA</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>EY Global Services Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>Luciano Fanti Bianco</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>Kimberly Farino</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>IT Project Manager</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>MIT Lincoln Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>John Farr</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Value Advis…</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>SAP Industries (Washington DC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>Jonathan Farrell</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Enterprise Account Executive</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Panaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>Tim Faubert</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Executive Director,…</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>BeiGene (Beijing) Co., Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>Angelo Fazio</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Global Sales</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>IBM Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>Beth Feaster</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Sr Business Develop…</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>INSPYR Solutions, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>Craig Fee</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Sr. Business A…</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Purdue University Global, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>Richard Ferling</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Sourcing ma…</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>The Pittsburgh Paints Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>Alejandro Ferreira</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Bintech, S.A. de C.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>Jeff Fillegar</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Sr Director Solution Engineering</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Tricentis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>Rich Filler</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Sr. Mgr IT</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Exelon Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>Colin Finley</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Kearney &amp; Company, P.C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>JP Finnell</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Senior Director Strategic…</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>Jack Fiorini</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Senior Business Development…</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Onapsis Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>Kurt Fischbach</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Director of Data Governa…</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>ScottsMiracle-Gro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>Cedric Fiske</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Sales Development Representative</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Coveo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>Kieran Fitzgerald</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Software Sales Lead</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>The Config Team Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>Susana Flores Cabrera</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Contracts Coordinator</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Cheney Bros, Inc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 54 D and E section contacts from screenshots
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1102"/>
+  <dimension ref="A1:C1156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19004,6 +19004,920 @@
         </is>
       </c>
     </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>Bonnie Davies</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>VP Finance &amp; Spend</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>Wendy Davis</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Solution Customer S…</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>SAP America (Houston)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>Rebecca Day</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>IS ERP and Revenu…</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>The Health and Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>Andrea De Colle</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Enterprise Arc…</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>SAP Argentina - Buenos Aires</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>Jeff DeHulsters</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Business Consultant</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Travis County, TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>Adrian DeSantis</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Sales Engineer</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>TrueCommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>Sushil Debare</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>ECS Regional Delivery H…</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>Larry Deille</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Senior Manager Digital Transf…</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Lam Research</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>Drew Delaney</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Business P…</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>The Scotts Miracle-Gro Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>Amy Delise</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Walgreens</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>Meghan Demo</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Director of Marketing</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Cognitus Consulting LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>James Dender</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Account Director</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>Sven Denecken</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>SVP SAP Industries</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>Urnav Desai</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Prin…</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Deloitte Touche Tohmatsu Services, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>Alan Detlif</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Director Business Sys…</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>The Crosby Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>Holly Devine</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Industry Advisor</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>Andrea Devroy Devroy</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Senior Dire…</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>PT Intermediate Holdings III,  LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>Raman Dhooria</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Celebal Technologies Pvt Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>Aboubacar Diallo</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>AI Governance Program Co-Lead</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>SAP SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>Sofia Diaz</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>SR. Manager Inside Sales</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Globant</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>Kathrin Dorothea Diederich</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr"/>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>KPMG AG Wirtschaftsprüfungsgesellschaft -…</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>Linda Dietzel</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Director, IT Supply C…</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>The Hershey Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>Guillermina Digregorio</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Global Head of GCO Private Clo…</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>SAP Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>Ralf Dillmann</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Partner &amp; C…</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>BearingPoint North America LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>Michael Dillon</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Global Platform Leader</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>IBM Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>Haricharan Dingari</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Enterprise Arc…</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Bob's Discount Furniture, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>Everett Dittman</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Strategic Customer Advisor, A…</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Databricks Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>Pankaj Diwan</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>ArchLynk, LLC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>Ralph Dommes</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Dommes Consulting, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>Mari Doroud</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>HRIS Manager</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Nucor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>Amisha Doshi</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Industry Account Executi…</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>Rakesh Doshi</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Architecture Advisor</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>Chris Dougherty</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Pfizer, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>Ryan Doyle</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Principal Co…</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>SAP Industries (Washington DC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>Adam Drent</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>GlobalSource IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>Shannon Drost</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Vice President Technology Soluti…</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Horizontal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>Erasmo Duarte</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>IT Manager</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Ford Motor Company Brasil Ltda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>Nicolas Duchesneau</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Analyst TI</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Portefeuille Soucy Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>Leah Dudley</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Senior Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Onapsis Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>Barbara Duffey</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>VP, North America C…</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Lakeland Industries Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>Damodhar Dyava</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>SAP SD Manag…</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Bob's Discount Furniture, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>Willard Dyck</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Sr. Enterprise…</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>IGM Financial/Financière IGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>Jan de Leeuw</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Executive Director Central Fina…</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Ingram Micro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>Erin Earl</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Executive  Industry Advi…</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>SAP AMERICA, INC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>Norihiro Egawa</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>ABeam Aystems</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>Kenji Eguchi</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Basis Consulta…</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>NTT DATA Japan Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>Onyi Egunjobi</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Value Advisor Senior</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>SAP Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>Marci Ehrhart</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Global Practice Leader</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>ADP, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>Pauleen Elasio</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Field Finance, Asia Paci…</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>SAP Philippines, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>Mark Elkin</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>SVP, Global Head of Solution…</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>SAP CANADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>Stephen Elkins</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Manager Enterprise Business…</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Basin Electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>Barry Emptage</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Director, SAP E…</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>RHOMBI HOLDINGS LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>Martha Enriquez Carrola</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Customer Engagement and Ado…</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>SAP Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>Lander Errasti</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>BFS Ingenieria Aplicada S.A. de C.V.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 10 C and D section contacts from screenshots
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1156"/>
+  <dimension ref="A1:C1166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19918,6 +19918,176 @@
         </is>
       </c>
     </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>Matt Curtin</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>OneRail, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>Thomas Czichowsky</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Business Consulting Retail | S…</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Schwarz IT KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>Beth clarkin</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Director…</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>True Commerce Inc. TrueCommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>Nick DAVIS</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Global Process Owner Order…</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Elanco US Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>Abdelhalim Dadouche</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>SAP Product Specialist</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Databricks Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>Chung DaeYoung</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Head of Enterprise 2</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>SAP Korea Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>Gerardo Dall'Orso</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>ADECO AGROPECUARIA S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>Madhu Raju Dandu</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Director, Dig…</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>RELEASEOWL PRIVATE LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>Nicolas Daniels</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Global Account Director</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Mediafly</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>Sushovan Datta</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Tech Mahindra (americas) Inc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Highlight rows by industry category
Adds row fill colors based on company name keywords:
- Retail & CPG: pastel yellow (#FFF9C4)
- Big 4 (Deloitte/EY/KPMG/PwC): pastel red (#FFCDD2)
- Deal advisor firms (McKinsey/Bain/BCG/BearingPoint/Grant Thornton/JPMorgan/etc.): pastel blue (#BBDEFB)
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+        <bgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,11 +74,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,17 +507,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Katrina Acebedo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Data Architect</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>The Hershey Company</t>
         </is>
@@ -605,17 +626,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Saritha Aguru</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Service Delivery &amp; Product M…</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Ernst &amp; Young</t>
         </is>
@@ -690,17 +711,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Ebenezer Aladeojebi</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Product Manager</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>J.P Morgan Chase &amp; Co.</t>
         </is>
@@ -826,17 +847,17 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Salazar del Rio Alma Aurora</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Functional leader</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -894,17 +915,17 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>David Amiot</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Deloitte</t>
         </is>
@@ -1383,17 +1404,17 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Jin Seon Baek</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>ERP Manager</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>H Mart Companies, Inc.</t>
         </is>
@@ -1434,17 +1455,17 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Staci Baker</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -1536,17 +1557,17 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Paul Baraniuk</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Global Solution…</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Florida Crystals Corporation</t>
         </is>
@@ -1757,17 +1778,17 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Marissa Bennett</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>Director, Global People Solutio…</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>PepsiCo, Inc</t>
         </is>
@@ -1872,17 +1893,17 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>Kerry Jo Berger</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>JPMorgan Chase Bank, NA</t>
         </is>
@@ -2127,17 +2148,17 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="3" t="inlineStr">
         <is>
           <t>Beverley Den Boestert</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="3" t="inlineStr">
         <is>
           <t>Director - Technology…</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="3" t="inlineStr">
         <is>
           <t>EY Global Services Ltd</t>
         </is>
@@ -2195,17 +2216,17 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>Patrick Boruta</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>Partner - Business Consultin…</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>Grant Thornton</t>
         </is>
@@ -2365,13 +2386,13 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>Adam Breiterman</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr">
+      <c r="B115" s="2" t="inlineStr"/>
+      <c r="C115" s="2" t="inlineStr">
         <is>
           <t>Maryland &amp; Virginia Milk Producers Cooperati…</t>
         </is>
@@ -2829,17 +2850,17 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
+      <c r="A143" s="3" t="inlineStr">
         <is>
           <t>Lisa Cabarcos</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
+      <c r="B143" s="3" t="inlineStr">
         <is>
           <t>America's SAP Allianc…</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C143" s="3" t="inlineStr">
         <is>
           <t>Ernst &amp; Young U.S. LLP</t>
         </is>
@@ -2965,34 +2986,34 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t>Pat Carmody</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>Senior Manag…</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
         <is>
           <t>Sharp Electronics Corporation</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="A152" s="4" t="inlineStr">
         <is>
           <t>Tyler Carr</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B152" s="4" t="inlineStr">
         <is>
           <t>Sr. Capabilities Manag…</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C152" s="4" t="inlineStr">
         <is>
           <t>McKinsey &amp; Company</t>
         </is>
@@ -3254,17 +3275,17 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
+      <c r="A168" s="2" t="inlineStr">
         <is>
           <t>Greg Chamberland</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>IT, Enterprise…</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
+      <c r="C168" s="2" t="inlineStr">
         <is>
           <t>Ocean Spray Cranberries, Inc.</t>
         </is>
@@ -3288,17 +3309,17 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
+      <c r="A170" s="2" t="inlineStr">
         <is>
           <t>Prasanna Chand</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>Director - Enterprise Tech</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C170" s="2" t="inlineStr">
         <is>
           <t>Wayfair</t>
         </is>
@@ -3322,17 +3343,17 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
+      <c r="A172" s="2" t="inlineStr">
         <is>
           <t>Matt Charleston</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Sr Manager Fi…</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
+      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>Performance Food Group, Inc.</t>
         </is>
@@ -3407,34 +3428,34 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
+      <c r="A177" s="2" t="inlineStr">
         <is>
           <t>Abraham Cherian</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Director Security Govern…</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>Kontoor Brands Inc</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Venu Cherupillil</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Systems Engineer Sr Princi…</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>The Home Depot</t>
         </is>
@@ -3556,34 +3577,34 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>Parinda Choksi</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>CIO - Enablement</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>Ball Horticultural Co.</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>Sanjay Choubey</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Global Chief Digital an…</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>Sylvamo Corporation</t>
         </is>
@@ -3807,17 +3828,17 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
+      <c r="A201" s="2" t="inlineStr">
         <is>
           <t>Colin Cole</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
+      <c r="B201" s="2" t="inlineStr">
         <is>
           <t>IT Director</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>JBS USA Food Company Holdings</t>
         </is>
@@ -3875,17 +3896,17 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr">
+      <c r="A205" s="3" t="inlineStr">
         <is>
           <t>Oisin Collins</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B205" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="3" t="inlineStr">
         <is>
           <t>Deloitte</t>
         </is>
@@ -4045,17 +4066,17 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
         <is>
           <t>Juan Correa</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
+      <c r="B215" s="2" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="C215" s="2" t="inlineStr">
         <is>
           <t>Sharp Corporation</t>
         </is>
@@ -4096,17 +4117,17 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr">
+      <c r="A218" s="3" t="inlineStr">
         <is>
           <t>Maryanne Coughlin</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
+      <c r="B218" s="3" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr">
+      <c r="C218" s="3" t="inlineStr">
         <is>
           <t>PwC</t>
         </is>
@@ -4343,17 +4364,17 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" t="inlineStr">
+      <c r="A233" s="3" t="inlineStr">
         <is>
           <t>Yuki Sato</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
+      <c r="B233" s="3" t="inlineStr">
         <is>
           <t>Business Consulting…</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr">
+      <c r="C233" s="3" t="inlineStr">
         <is>
           <t>EY Global Services Ltd</t>
         </is>
@@ -4479,17 +4500,17 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" t="inlineStr">
+      <c r="A241" s="3" t="inlineStr">
         <is>
           <t>Kathrin Schmalzing</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr">
+      <c r="B241" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr">
+      <c r="C241" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -4836,17 +4857,17 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" t="inlineStr">
+      <c r="A262" s="2" t="inlineStr">
         <is>
           <t>Dawn Shakeshaft</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr">
+      <c r="B262" s="2" t="inlineStr">
         <is>
           <t>Controller</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr">
+      <c r="C262" s="2" t="inlineStr">
         <is>
           <t>Associated Feed &amp; Supply Co.</t>
         </is>
@@ -5589,17 +5610,17 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" t="inlineStr">
+      <c r="A307" s="3" t="inlineStr">
         <is>
           <t>Meik Spanowsky</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
+      <c r="B307" s="3" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr">
+      <c r="C307" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -5768,17 +5789,17 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" t="inlineStr">
+      <c r="A318" s="4" t="inlineStr">
         <is>
           <t>Robert Stemmler</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
+      <c r="B318" s="4" t="inlineStr">
         <is>
           <t>Global Alliances &amp; Ec…</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr">
+      <c r="C318" s="4" t="inlineStr">
         <is>
           <t>McKinsey &amp; Company</t>
         </is>
@@ -5917,17 +5938,17 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" t="inlineStr">
+      <c r="A327" s="2" t="inlineStr">
         <is>
           <t>Kevin Stupp</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
+      <c r="B327" s="2" t="inlineStr">
         <is>
           <t>Director S4 Platform</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr">
+      <c r="C327" s="2" t="inlineStr">
         <is>
           <t>The Hershey Company</t>
         </is>
@@ -6002,17 +6023,17 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="inlineStr">
+      <c r="A332" s="3" t="inlineStr">
         <is>
           <t>Som Suresh</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
+      <c r="B332" s="3" t="inlineStr">
         <is>
           <t>Man…</t>
         </is>
       </c>
-      <c r="C332" t="inlineStr">
+      <c r="C332" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -6291,17 +6312,17 @@
       </c>
     </row>
     <row r="349">
-      <c r="A349" t="inlineStr">
+      <c r="A349" s="2" t="inlineStr">
         <is>
           <t>Steve Tanaka</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
+      <c r="B349" s="2" t="inlineStr">
         <is>
           <t>Sr Vice Presid…</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C349" s="2" t="inlineStr">
         <is>
           <t>Blommer Chocolate Company</t>
         </is>
@@ -6563,17 +6584,17 @@
       </c>
     </row>
     <row r="365">
-      <c r="A365" t="inlineStr">
+      <c r="A365" s="2" t="inlineStr">
         <is>
           <t>Barbara Thrasher</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr">
+      <c r="B365" s="2" t="inlineStr">
         <is>
           <t>SR STAFF ARCHITECT</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="2" t="inlineStr">
         <is>
           <t>Tyson Foods, Inc.</t>
         </is>
@@ -6831,17 +6852,17 @@
       </c>
     </row>
     <row r="381">
-      <c r="A381" t="inlineStr">
+      <c r="A381" s="3" t="inlineStr">
         <is>
           <t>Paul Turbes</t>
         </is>
       </c>
-      <c r="B381" t="inlineStr">
+      <c r="B381" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="C381" t="inlineStr">
+      <c r="C381" s="3" t="inlineStr">
         <is>
           <t>KPMG LLP</t>
         </is>
@@ -7069,17 +7090,17 @@
       </c>
     </row>
     <row r="395">
-      <c r="A395" t="inlineStr">
+      <c r="A395" s="2" t="inlineStr">
         <is>
           <t>Vijay Varee</t>
         </is>
       </c>
-      <c r="B395" t="inlineStr">
+      <c r="B395" s="2" t="inlineStr">
         <is>
           <t>Senior Manager</t>
         </is>
       </c>
-      <c r="C395" t="inlineStr">
+      <c r="C395" s="2" t="inlineStr">
         <is>
           <t>Petsmart LLC</t>
         </is>
@@ -7388,34 +7409,34 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="inlineStr">
+      <c r="A414" s="3" t="inlineStr">
         <is>
           <t>Thomas Vioux</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B414" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C414" s="3" t="inlineStr">
         <is>
           <t>PwC</t>
         </is>
       </c>
     </row>
     <row r="415">
-      <c r="A415" t="inlineStr">
+      <c r="A415" s="3" t="inlineStr">
         <is>
           <t>Anil Visal</t>
         </is>
       </c>
-      <c r="B415" t="inlineStr">
+      <c r="B415" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C415" t="inlineStr">
+      <c r="C415" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -7639,17 +7660,17 @@
       </c>
     </row>
     <row r="429">
-      <c r="A429" t="inlineStr">
+      <c r="A429" s="3" t="inlineStr">
         <is>
           <t>Waka Wakabayashi</t>
         </is>
       </c>
-      <c r="B429" t="inlineStr">
+      <c r="B429" s="3" t="inlineStr">
         <is>
           <t>Associate Partner</t>
         </is>
       </c>
-      <c r="C429" t="inlineStr">
+      <c r="C429" s="3" t="inlineStr">
         <is>
           <t>KPMG Consulting Co., Ltd.</t>
         </is>
@@ -7741,34 +7762,34 @@
       </c>
     </row>
     <row r="435">
-      <c r="A435" t="inlineStr">
+      <c r="A435" s="3" t="inlineStr">
         <is>
           <t>May Wang</t>
         </is>
       </c>
-      <c r="B435" t="inlineStr">
+      <c r="B435" s="3" t="inlineStr">
         <is>
           <t>Direc…</t>
         </is>
       </c>
-      <c r="C435" t="inlineStr">
+      <c r="C435" s="3" t="inlineStr">
         <is>
           <t>Deloitte Consulting (Shanghai) Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="436">
-      <c r="A436" t="inlineStr">
+      <c r="A436" s="2" t="inlineStr">
         <is>
           <t>Adam Warner</t>
         </is>
       </c>
-      <c r="B436" t="inlineStr">
+      <c r="B436" s="2" t="inlineStr">
         <is>
           <t>Cost Analyst</t>
         </is>
       </c>
-      <c r="C436" t="inlineStr">
+      <c r="C436" s="2" t="inlineStr">
         <is>
           <t>Marathon Cheese Corporation</t>
         </is>
@@ -7877,34 +7898,34 @@
       </c>
     </row>
     <row r="443">
-      <c r="A443" t="inlineStr">
+      <c r="A443" s="2" t="inlineStr">
         <is>
           <t>Chris Webster</t>
         </is>
       </c>
-      <c r="B443" t="inlineStr">
+      <c r="B443" s="2" t="inlineStr">
         <is>
           <t>SVP IT Strategy &amp; Architecture</t>
         </is>
       </c>
-      <c r="C443" t="inlineStr">
+      <c r="C443" s="2" t="inlineStr">
         <is>
           <t>Ahold Delhaize</t>
         </is>
       </c>
     </row>
     <row r="444">
-      <c r="A444" t="inlineStr">
+      <c r="A444" s="2" t="inlineStr">
         <is>
           <t>Matt Webster</t>
         </is>
       </c>
-      <c r="B444" t="inlineStr">
+      <c r="B444" s="2" t="inlineStr">
         <is>
           <t>Director of…</t>
         </is>
       </c>
-      <c r="C444" t="inlineStr">
+      <c r="C444" s="2" t="inlineStr">
         <is>
           <t>Gardner White Furniture Co., Inc.</t>
         </is>
@@ -7928,34 +7949,34 @@
       </c>
     </row>
     <row r="446">
-      <c r="A446" t="inlineStr">
+      <c r="A446" s="2" t="inlineStr">
         <is>
           <t>Sarah Weiler</t>
         </is>
       </c>
-      <c r="B446" t="inlineStr">
+      <c r="B446" s="2" t="inlineStr">
         <is>
           <t>Manager, Busine…</t>
         </is>
       </c>
-      <c r="C446" t="inlineStr">
+      <c r="C446" s="2" t="inlineStr">
         <is>
           <t>Ball Horticultural Company</t>
         </is>
       </c>
     </row>
     <row r="447">
-      <c r="A447" t="inlineStr">
+      <c r="A447" s="2" t="inlineStr">
         <is>
           <t>Adam Werner</t>
         </is>
       </c>
-      <c r="B447" t="inlineStr">
+      <c r="B447" s="2" t="inlineStr">
         <is>
           <t>VP, Corporate Technology</t>
         </is>
       </c>
-      <c r="C447" t="inlineStr">
+      <c r="C447" s="2" t="inlineStr">
         <is>
           <t>Crocs, Inc.</t>
         </is>
@@ -8047,13 +8068,13 @@
       </c>
     </row>
     <row r="453">
-      <c r="A453" t="inlineStr">
+      <c r="A453" s="2" t="inlineStr">
         <is>
           <t>Robb White</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr"/>
-      <c r="C453" t="inlineStr">
+      <c r="B453" s="2" t="inlineStr"/>
+      <c r="C453" s="2" t="inlineStr">
         <is>
           <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
         </is>
@@ -8128,17 +8149,17 @@
       </c>
     </row>
     <row r="458">
-      <c r="A458" t="inlineStr">
+      <c r="A458" s="3" t="inlineStr">
         <is>
           <t>Mark Willey</t>
         </is>
       </c>
-      <c r="B458" t="inlineStr">
+      <c r="B458" s="3" t="inlineStr">
         <is>
           <t>Vice…</t>
         </is>
       </c>
-      <c r="C458" t="inlineStr">
+      <c r="C458" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -8859,17 +8880,17 @@
       </c>
     </row>
     <row r="501">
-      <c r="A501" t="inlineStr">
+      <c r="A501" s="3" t="inlineStr">
         <is>
           <t>Araja Reddy</t>
         </is>
       </c>
-      <c r="B501" t="inlineStr">
+      <c r="B501" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="C501" t="inlineStr">
+      <c r="C501" s="3" t="inlineStr">
         <is>
           <t>Deloitte Consulting</t>
         </is>
@@ -8893,13 +8914,13 @@
       </c>
     </row>
     <row r="503">
-      <c r="A503" t="inlineStr">
+      <c r="A503" s="3" t="inlineStr">
         <is>
           <t>Nico Reichen</t>
         </is>
       </c>
-      <c r="B503" t="inlineStr"/>
-      <c r="C503" t="inlineStr">
+      <c r="B503" s="3" t="inlineStr"/>
+      <c r="C503" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
         </is>
@@ -9234,17 +9255,17 @@
       </c>
     </row>
     <row r="524">
-      <c r="A524" t="inlineStr">
+      <c r="A524" s="3" t="inlineStr">
         <is>
           <t>Diana Romaya</t>
         </is>
       </c>
-      <c r="B524" t="inlineStr">
+      <c r="B524" s="3" t="inlineStr">
         <is>
           <t>SAP...</t>
         </is>
       </c>
-      <c r="C524" t="inlineStr">
+      <c r="C524" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -9370,13 +9391,13 @@
       </c>
     </row>
     <row r="532">
-      <c r="A532" t="inlineStr">
+      <c r="A532" s="3" t="inlineStr">
         <is>
           <t>Frank Ruland</t>
         </is>
       </c>
-      <c r="B532" t="inlineStr"/>
-      <c r="C532" t="inlineStr">
+      <c r="B532" s="3" t="inlineStr"/>
+      <c r="C532" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers GmbH Wirtschaftsp...</t>
         </is>
@@ -9434,17 +9455,17 @@
       </c>
     </row>
     <row r="536">
-      <c r="A536" t="inlineStr">
+      <c r="A536" s="4" t="inlineStr">
         <is>
           <t>Natalie Röthel</t>
         </is>
       </c>
-      <c r="B536" t="inlineStr">
+      <c r="B536" s="4" t="inlineStr">
         <is>
           <t>Executive Assistant</t>
         </is>
       </c>
-      <c r="C536" t="inlineStr">
+      <c r="C536" s="4" t="inlineStr">
         <is>
           <t>McKinsey &amp; Company</t>
         </is>
@@ -9774,17 +9795,17 @@
       </c>
     </row>
     <row r="556">
-      <c r="A556" t="inlineStr">
+      <c r="A556" s="2" t="inlineStr">
         <is>
           <t>Rogério Peres</t>
         </is>
       </c>
-      <c r="B556" t="inlineStr">
+      <c r="B556" s="2" t="inlineStr">
         <is>
           <t>CIO</t>
         </is>
       </c>
-      <c r="C556" t="inlineStr">
+      <c r="C556" s="2" t="inlineStr">
         <is>
           <t>JBS USA</t>
         </is>
@@ -9876,17 +9897,17 @@
       </c>
     </row>
     <row r="562">
-      <c r="A562" t="inlineStr">
+      <c r="A562" s="3" t="inlineStr">
         <is>
           <t>Catherine Perry-Robertson</t>
         </is>
       </c>
-      <c r="B562" t="inlineStr">
+      <c r="B562" s="3" t="inlineStr">
         <is>
           <t>Partner, Natio...</t>
         </is>
       </c>
-      <c r="C562" t="inlineStr">
+      <c r="C562" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -10093,17 +10114,17 @@
       </c>
     </row>
     <row r="575">
-      <c r="A575" t="inlineStr">
+      <c r="A575" s="3" t="inlineStr">
         <is>
           <t>Franck Poisson</t>
         </is>
       </c>
-      <c r="B575" t="inlineStr">
+      <c r="B575" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C575" t="inlineStr">
+      <c r="C575" s="3" t="inlineStr">
         <is>
           <t>PWC US Group LLP</t>
         </is>
@@ -10892,17 +10913,17 @@
       </c>
     </row>
     <row r="622">
-      <c r="A622" t="inlineStr">
+      <c r="A622" s="2" t="inlineStr">
         <is>
           <t>Pavel Nouel</t>
         </is>
       </c>
-      <c r="B622" t="inlineStr">
+      <c r="B622" s="2" t="inlineStr">
         <is>
           <t>Vice President,...</t>
         </is>
       </c>
-      <c r="C622" t="inlineStr">
+      <c r="C622" s="2" t="inlineStr">
         <is>
           <t>Colgate-Palmolive Company</t>
         </is>
@@ -11636,17 +11657,17 @@
       </c>
     </row>
     <row r="666">
-      <c r="A666" t="inlineStr">
+      <c r="A666" s="2" t="inlineStr">
         <is>
           <t>Mark Meanwell</t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
+      <c r="B666" s="2" t="inlineStr">
         <is>
           <t>Senior Manager Data &amp; Analytics</t>
         </is>
       </c>
-      <c r="C666" t="inlineStr">
+      <c r="C666" s="2" t="inlineStr">
         <is>
           <t>Sylvamo</t>
         </is>
@@ -11921,17 +11942,17 @@
       </c>
     </row>
     <row r="683">
-      <c r="A683" t="inlineStr">
+      <c r="A683" s="3" t="inlineStr">
         <is>
           <t>Piyush Mistry</t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B683" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C683" t="inlineStr">
+      <c r="C683" s="3" t="inlineStr">
         <is>
           <t>Deloitte</t>
         </is>
@@ -12576,17 +12597,17 @@
       </c>
     </row>
     <row r="722">
-      <c r="A722" t="inlineStr">
+      <c r="A722" s="2" t="inlineStr">
         <is>
           <t>Tammy Louie</t>
         </is>
       </c>
-      <c r="B722" t="inlineStr">
+      <c r="B722" s="2" t="inlineStr">
         <is>
           <t>Senior Financial Systems Analyst</t>
         </is>
       </c>
-      <c r="C722" t="inlineStr">
+      <c r="C722" s="2" t="inlineStr">
         <is>
           <t>AutoZone</t>
         </is>
@@ -12729,17 +12750,17 @@
       </c>
     </row>
     <row r="731">
-      <c r="A731" t="inlineStr">
+      <c r="A731" s="4" t="inlineStr">
         <is>
           <t>Nicolas Löwe</t>
         </is>
       </c>
-      <c r="B731" t="inlineStr">
+      <c r="B731" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C731" t="inlineStr">
+      <c r="C731" s="4" t="inlineStr">
         <is>
           <t>BearingPoint GmbH</t>
         </is>
@@ -12916,17 +12937,17 @@
       </c>
     </row>
     <row r="742">
-      <c r="A742" t="inlineStr">
+      <c r="A742" s="3" t="inlineStr">
         <is>
           <t>Naresh Makhijani Makhijani</t>
         </is>
       </c>
-      <c r="B742" t="inlineStr">
+      <c r="B742" s="3" t="inlineStr">
         <is>
           <t>Glo...</t>
         </is>
       </c>
-      <c r="C742" t="inlineStr">
+      <c r="C742" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -12950,17 +12971,17 @@
       </c>
     </row>
     <row r="744">
-      <c r="A744" t="inlineStr">
+      <c r="A744" s="3" t="inlineStr">
         <is>
           <t>Melissa Marchetti</t>
         </is>
       </c>
-      <c r="B744" t="inlineStr">
+      <c r="B744" s="3" t="inlineStr">
         <is>
           <t>SAP...</t>
         </is>
       </c>
-      <c r="C744" t="inlineStr">
+      <c r="C744" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -13409,17 +13430,17 @@
       </c>
     </row>
     <row r="771">
-      <c r="A771" t="inlineStr">
+      <c r="A771" s="3" t="inlineStr">
         <is>
           <t>Denise McGuigan</t>
         </is>
       </c>
-      <c r="B771" t="inlineStr">
+      <c r="B771" s="3" t="inlineStr">
         <is>
           <t>Part...</t>
         </is>
       </c>
-      <c r="C771" t="inlineStr">
+      <c r="C771" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -13473,17 +13494,17 @@
       </c>
     </row>
     <row r="775">
-      <c r="A775" t="inlineStr">
+      <c r="A775" s="2" t="inlineStr">
         <is>
           <t>Siddhi Kshatriya</t>
         </is>
       </c>
-      <c r="B775" t="inlineStr">
+      <c r="B775" s="2" t="inlineStr">
         <is>
           <t>Organizational Change Managem...</t>
         </is>
       </c>
-      <c r="C775" t="inlineStr">
+      <c r="C775" s="2" t="inlineStr">
         <is>
           <t>AutoZone</t>
         </is>
@@ -13605,17 +13626,17 @@
       </c>
     </row>
     <row r="783">
-      <c r="A783" t="inlineStr">
+      <c r="A783" s="3" t="inlineStr">
         <is>
           <t>Dennis Kurlandski</t>
         </is>
       </c>
-      <c r="B783" t="inlineStr">
+      <c r="B783" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="C783" t="inlineStr">
+      <c r="C783" s="3" t="inlineStr">
         <is>
           <t>KPMG</t>
         </is>
@@ -14880,17 +14901,17 @@
       </c>
     </row>
     <row r="858">
-      <c r="A858" t="inlineStr">
+      <c r="A858" s="3" t="inlineStr">
         <is>
           <t>Ron King</t>
         </is>
       </c>
-      <c r="B858" t="inlineStr">
+      <c r="B858" s="3" t="inlineStr">
         <is>
           <t>VP, Sales Executive</t>
         </is>
       </c>
-      <c r="C858" t="inlineStr">
+      <c r="C858" s="3" t="inlineStr">
         <is>
           <t>Deloitte Consulting LLP</t>
         </is>
@@ -14914,17 +14935,17 @@
       </c>
     </row>
     <row r="860">
-      <c r="A860" t="inlineStr">
+      <c r="A860" s="3" t="inlineStr">
         <is>
           <t>Hiroshi Kitano</t>
         </is>
       </c>
-      <c r="B860" t="inlineStr">
+      <c r="B860" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C860" t="inlineStr">
+      <c r="C860" s="3" t="inlineStr">
         <is>
           <t>EY Strategy and Consulting Co., Ltd.</t>
         </is>
@@ -15063,17 +15084,17 @@
       </c>
     </row>
     <row r="869">
-      <c r="A869" t="inlineStr">
+      <c r="A869" s="4" t="inlineStr">
         <is>
           <t>Christian Koestler</t>
         </is>
       </c>
-      <c r="B869" t="inlineStr">
+      <c r="B869" s="4" t="inlineStr">
         <is>
           <t>Global Director, Client...</t>
         </is>
       </c>
-      <c r="C869" t="inlineStr">
+      <c r="C869" s="4" t="inlineStr">
         <is>
           <t>McKinsey &amp; Company</t>
         </is>
@@ -15646,17 +15667,17 @@
       </c>
     </row>
     <row r="904">
-      <c r="A904" t="inlineStr">
+      <c r="A904" s="3" t="inlineStr">
         <is>
           <t>Armin Kaltenmeier</t>
         </is>
       </c>
-      <c r="B904" t="inlineStr">
+      <c r="B904" s="3" t="inlineStr">
         <is>
           <t>Partner, Global Chief...</t>
         </is>
       </c>
-      <c r="C904" t="inlineStr">
+      <c r="C904" s="3" t="inlineStr">
         <is>
           <t>Ernst &amp; Young U.S. LLP</t>
         </is>
@@ -15748,17 +15769,17 @@
       </c>
     </row>
     <row r="910">
-      <c r="A910" t="inlineStr">
+      <c r="A910" s="2" t="inlineStr">
         <is>
           <t>Francisco Galindo</t>
         </is>
       </c>
-      <c r="B910" t="inlineStr">
+      <c r="B910" s="2" t="inlineStr">
         <is>
           <t>Sr Director IT finance</t>
         </is>
       </c>
-      <c r="C910" t="inlineStr">
+      <c r="C910" s="2" t="inlineStr">
         <is>
           <t>Colgate Palmolive</t>
         </is>
@@ -15901,17 +15922,17 @@
       </c>
     </row>
     <row r="919">
-      <c r="A919" t="inlineStr">
+      <c r="A919" s="2" t="inlineStr">
         <is>
           <t>Patti Gary</t>
         </is>
       </c>
-      <c r="B919" t="inlineStr">
+      <c r="B919" s="2" t="inlineStr">
         <is>
           <t>Senior Enterprise Architect</t>
         </is>
       </c>
-      <c r="C919" t="inlineStr">
+      <c r="C919" s="2" t="inlineStr">
         <is>
           <t>Tyson Foods, Inc.</t>
         </is>
@@ -16309,17 +16330,17 @@
       </c>
     </row>
     <row r="943">
-      <c r="A943" t="inlineStr">
+      <c r="A943" s="2" t="inlineStr">
         <is>
           <t>Christine Graham</t>
         </is>
       </c>
-      <c r="B943" t="inlineStr">
+      <c r="B943" s="2" t="inlineStr">
         <is>
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="C943" t="inlineStr">
+      <c r="C943" s="2" t="inlineStr">
         <is>
           <t>Lakeview Farms, LLC</t>
         </is>
@@ -16526,17 +16547,17 @@
       </c>
     </row>
     <row r="956">
-      <c r="A956" t="inlineStr">
+      <c r="A956" s="2" t="inlineStr">
         <is>
           <t>Patricia Guillermo</t>
         </is>
       </c>
-      <c r="B956" t="inlineStr">
+      <c r="B956" s="2" t="inlineStr">
         <is>
           <t>It Lead</t>
         </is>
       </c>
-      <c r="C956" t="inlineStr">
+      <c r="C956" s="2" t="inlineStr">
         <is>
           <t>Kellanova/Mars</t>
         </is>
@@ -16577,17 +16598,17 @@
       </c>
     </row>
     <row r="959">
-      <c r="A959" t="inlineStr">
+      <c r="A959" s="3" t="inlineStr">
         <is>
           <t>Sriram Hariharasubramanian</t>
         </is>
       </c>
-      <c r="B959" t="inlineStr">
+      <c r="B959" s="3" t="inlineStr">
         <is>
           <t>Partner, Tech Consult...</t>
         </is>
       </c>
-      <c r="C959" t="inlineStr">
+      <c r="C959" s="3" t="inlineStr">
         <is>
           <t>EY Global Services Ltd</t>
         </is>
@@ -16628,17 +16649,17 @@
       </c>
     </row>
     <row r="962">
-      <c r="A962" t="inlineStr">
+      <c r="A962" s="2" t="inlineStr">
         <is>
           <t>Paul Harris</t>
         </is>
       </c>
-      <c r="B962" t="inlineStr">
+      <c r="B962" s="2" t="inlineStr">
         <is>
           <t>Senior Director, SAP Basi...</t>
         </is>
       </c>
-      <c r="C962" t="inlineStr">
+      <c r="C962" s="2" t="inlineStr">
         <is>
           <t>Varsity Brands, LLC.</t>
         </is>
@@ -16832,17 +16853,17 @@
       </c>
     </row>
     <row r="974">
-      <c r="A974" t="inlineStr">
+      <c r="A974" s="2" t="inlineStr">
         <is>
           <t>Adriana Hernandez</t>
         </is>
       </c>
-      <c r="B974" t="inlineStr">
+      <c r="B974" s="2" t="inlineStr">
         <is>
           <t>Head Architecture</t>
         </is>
       </c>
-      <c r="C974" t="inlineStr">
+      <c r="C974" s="2" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -17049,17 +17070,17 @@
       </c>
     </row>
     <row r="987">
-      <c r="A987" t="inlineStr">
+      <c r="A987" s="4" t="inlineStr">
         <is>
           <t>Michael Hom</t>
         </is>
       </c>
-      <c r="B987" t="inlineStr">
+      <c r="B987" s="4" t="inlineStr">
         <is>
           <t>Global Head of Digit...</t>
         </is>
       </c>
-      <c r="C987" t="inlineStr">
+      <c r="C987" s="4" t="inlineStr">
         <is>
           <t>Jpmorgan Chase &amp; Co.</t>
         </is>
@@ -17334,17 +17355,17 @@
       </c>
     </row>
     <row r="1004">
-      <c r="A1004" t="inlineStr">
+      <c r="A1004" s="2" t="inlineStr">
         <is>
           <t>Omar Hussein Olmedo</t>
         </is>
       </c>
-      <c r="B1004" t="inlineStr">
+      <c r="B1004" s="2" t="inlineStr">
         <is>
           <t>Poject Manager</t>
         </is>
       </c>
-      <c r="C1004" t="inlineStr">
+      <c r="C1004" s="2" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -17691,17 +17712,17 @@
       </c>
     </row>
     <row r="1025">
-      <c r="A1025" t="inlineStr">
+      <c r="A1025" s="3" t="inlineStr">
         <is>
           <t>Naren Jain</t>
         </is>
       </c>
-      <c r="B1025" t="inlineStr">
+      <c r="B1025" s="3" t="inlineStr">
         <is>
           <t>Managing Dire...</t>
         </is>
       </c>
-      <c r="C1025" t="inlineStr">
+      <c r="C1025" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -17895,17 +17916,17 @@
       </c>
     </row>
     <row r="1037">
-      <c r="A1037" t="inlineStr">
+      <c r="A1037" s="3" t="inlineStr">
         <is>
           <t>Angie Halderman</t>
         </is>
       </c>
-      <c r="B1037" t="inlineStr">
+      <c r="B1037" s="3" t="inlineStr">
         <is>
           <t>Vice President, Sales</t>
         </is>
       </c>
-      <c r="C1037" t="inlineStr">
+      <c r="C1037" s="3" t="inlineStr">
         <is>
           <t>Deloitte</t>
         </is>
@@ -18095,17 +18116,17 @@
       </c>
     </row>
     <row r="1049">
-      <c r="A1049" t="inlineStr">
+      <c r="A1049" s="3" t="inlineStr">
         <is>
           <t>Niladri Gupta</t>
         </is>
       </c>
-      <c r="B1049" t="inlineStr">
+      <c r="B1049" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="C1049" t="inlineStr">
+      <c r="C1049" s="3" t="inlineStr">
         <is>
           <t>Deloitte Consulting LLP</t>
         </is>
@@ -18210,13 +18231,13 @@
       </c>
     </row>
     <row r="1056">
-      <c r="A1056" t="inlineStr">
+      <c r="A1056" s="2" t="inlineStr">
         <is>
           <t>Kalman Gyula</t>
         </is>
       </c>
-      <c r="B1056" t="inlineStr"/>
-      <c r="C1056" t="inlineStr">
+      <c r="B1056" s="2" t="inlineStr"/>
+      <c r="C1056" s="2" t="inlineStr">
         <is>
           <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
         </is>
@@ -18393,17 +18414,17 @@
       </c>
     </row>
     <row r="1067">
-      <c r="A1067" t="inlineStr">
+      <c r="A1067" s="2" t="inlineStr">
         <is>
           <t>Jeremy Freeman</t>
         </is>
       </c>
-      <c r="B1067" t="inlineStr">
+      <c r="B1067" s="2" t="inlineStr">
         <is>
           <t>Director, Technology</t>
         </is>
       </c>
-      <c r="C1067" t="inlineStr">
+      <c r="C1067" s="2" t="inlineStr">
         <is>
           <t>Aritzia</t>
         </is>
@@ -18512,17 +18533,17 @@
       </c>
     </row>
     <row r="1074">
-      <c r="A1074" t="inlineStr">
+      <c r="A1074" s="4" t="inlineStr">
         <is>
           <t>Sean Furukawa</t>
         </is>
       </c>
-      <c r="B1074" t="inlineStr">
+      <c r="B1074" s="4" t="inlineStr">
         <is>
           <t>Deputy CEO</t>
         </is>
       </c>
-      <c r="C1074" t="inlineStr">
+      <c r="C1074" s="4" t="inlineStr">
         <is>
           <t>BearingPoint NA LLC</t>
         </is>
@@ -18580,17 +18601,17 @@
       </c>
     </row>
     <row r="1078">
-      <c r="A1078" t="inlineStr">
+      <c r="A1078" s="3" t="inlineStr">
         <is>
           <t>Jennifer Ertler</t>
         </is>
       </c>
-      <c r="B1078" t="inlineStr">
+      <c r="B1078" s="3" t="inlineStr">
         <is>
           <t>Principal</t>
         </is>
       </c>
-      <c r="C1078" t="inlineStr">
+      <c r="C1078" s="3" t="inlineStr">
         <is>
           <t>Deloitte</t>
         </is>
@@ -18614,34 +18635,34 @@
       </c>
     </row>
     <row r="1080">
-      <c r="A1080" t="inlineStr">
+      <c r="A1080" s="3" t="inlineStr">
         <is>
           <t>Jose Manuel Estevz Estevez</t>
         </is>
       </c>
-      <c r="B1080" t="inlineStr">
+      <c r="B1080" s="3" t="inlineStr">
         <is>
           <t>Technology Consulta…</t>
         </is>
       </c>
-      <c r="C1080" t="inlineStr">
+      <c r="C1080" s="3" t="inlineStr">
         <is>
           <t>EY Global Services Ltd</t>
         </is>
       </c>
     </row>
     <row r="1081">
-      <c r="A1081" t="inlineStr">
+      <c r="A1081" s="3" t="inlineStr">
         <is>
           <t>Brandon Evans</t>
         </is>
       </c>
-      <c r="B1081" t="inlineStr">
+      <c r="B1081" s="3" t="inlineStr">
         <is>
           <t>Managing Dire…</t>
         </is>
       </c>
-      <c r="C1081" t="inlineStr">
+      <c r="C1081" s="3" t="inlineStr">
         <is>
           <t>PricewaterhouseCoopers LLP</t>
         </is>
@@ -18665,17 +18686,17 @@
       </c>
     </row>
     <row r="1083">
-      <c r="A1083" t="inlineStr">
+      <c r="A1083" s="3" t="inlineStr">
         <is>
           <t>SATOSHI FUJITA</t>
         </is>
       </c>
-      <c r="B1083" t="inlineStr">
+      <c r="B1083" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C1083" t="inlineStr">
+      <c r="C1083" s="3" t="inlineStr">
         <is>
           <t>EY Global Services Ltd</t>
         </is>
@@ -18988,17 +19009,17 @@
       </c>
     </row>
     <row r="1102">
-      <c r="A1102" t="inlineStr">
+      <c r="A1102" s="2" t="inlineStr">
         <is>
           <t>Susana Flores Cabrera</t>
         </is>
       </c>
-      <c r="B1102" t="inlineStr">
+      <c r="B1102" s="2" t="inlineStr">
         <is>
           <t>Contracts Coordinator</t>
         </is>
       </c>
-      <c r="C1102" t="inlineStr">
+      <c r="C1102" s="2" t="inlineStr">
         <is>
           <t>Cheney Bros, Inc.</t>
         </is>
@@ -19158,17 +19179,17 @@
       </c>
     </row>
     <row r="1112">
-      <c r="A1112" t="inlineStr">
+      <c r="A1112" s="2" t="inlineStr">
         <is>
           <t>Amy Delise</t>
         </is>
       </c>
-      <c r="B1112" t="inlineStr">
+      <c r="B1112" s="2" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="C1112" t="inlineStr">
+      <c r="C1112" s="2" t="inlineStr">
         <is>
           <t>Walgreens</t>
         </is>
@@ -19226,17 +19247,17 @@
       </c>
     </row>
     <row r="1116">
-      <c r="A1116" t="inlineStr">
+      <c r="A1116" s="3" t="inlineStr">
         <is>
           <t>Urnav Desai</t>
         </is>
       </c>
-      <c r="B1116" t="inlineStr">
+      <c r="B1116" s="3" t="inlineStr">
         <is>
           <t>Prin…</t>
         </is>
       </c>
-      <c r="C1116" t="inlineStr">
+      <c r="C1116" s="3" t="inlineStr">
         <is>
           <t>Deloitte Touche Tohmatsu Services, LLC</t>
         </is>
@@ -19345,30 +19366,30 @@
       </c>
     </row>
     <row r="1123">
-      <c r="A1123" t="inlineStr">
+      <c r="A1123" s="3" t="inlineStr">
         <is>
           <t>Kathrin Dorothea Diederich</t>
         </is>
       </c>
-      <c r="B1123" t="inlineStr"/>
-      <c r="C1123" t="inlineStr">
+      <c r="B1123" s="3" t="inlineStr"/>
+      <c r="C1123" s="3" t="inlineStr">
         <is>
           <t>KPMG AG Wirtschaftsprüfungsgesellschaft -…</t>
         </is>
       </c>
     </row>
     <row r="1124">
-      <c r="A1124" t="inlineStr">
+      <c r="A1124" s="2" t="inlineStr">
         <is>
           <t>Linda Dietzel</t>
         </is>
       </c>
-      <c r="B1124" t="inlineStr">
+      <c r="B1124" s="2" t="inlineStr">
         <is>
           <t>Director, IT Supply C…</t>
         </is>
       </c>
-      <c r="C1124" t="inlineStr">
+      <c r="C1124" s="2" t="inlineStr">
         <is>
           <t>The Hershey Company</t>
         </is>
@@ -19392,17 +19413,17 @@
       </c>
     </row>
     <row r="1126">
-      <c r="A1126" t="inlineStr">
+      <c r="A1126" s="4" t="inlineStr">
         <is>
           <t>Ralf Dillmann</t>
         </is>
       </c>
-      <c r="B1126" t="inlineStr">
+      <c r="B1126" s="4" t="inlineStr">
         <is>
           <t>Partner &amp; C…</t>
         </is>
       </c>
-      <c r="C1126" t="inlineStr">
+      <c r="C1126" s="4" t="inlineStr">
         <is>
           <t>BearingPoint North America LLC</t>
         </is>
@@ -19426,17 +19447,17 @@
       </c>
     </row>
     <row r="1128">
-      <c r="A1128" t="inlineStr">
+      <c r="A1128" s="2" t="inlineStr">
         <is>
           <t>Haricharan Dingari</t>
         </is>
       </c>
-      <c r="B1128" t="inlineStr">
+      <c r="B1128" s="2" t="inlineStr">
         <is>
           <t>Enterprise Arc…</t>
         </is>
       </c>
-      <c r="C1128" t="inlineStr">
+      <c r="C1128" s="2" t="inlineStr">
         <is>
           <t>Bob's Discount Furniture, LLC</t>
         </is>
@@ -19681,17 +19702,17 @@
       </c>
     </row>
     <row r="1143">
-      <c r="A1143" t="inlineStr">
+      <c r="A1143" s="2" t="inlineStr">
         <is>
           <t>Damodhar Dyava</t>
         </is>
       </c>
-      <c r="B1143" t="inlineStr">
+      <c r="B1143" s="2" t="inlineStr">
         <is>
           <t>SAP SD Manag…</t>
         </is>
       </c>
-      <c r="C1143" t="inlineStr">
+      <c r="C1143" s="2" t="inlineStr">
         <is>
           <t>Bob's Discount Furniture, LLC</t>
         </is>

</xml_diff>

<commit_message>
Highlight >$5B Retail/CPG companies in pastel green
</commit_message>
<xml_diff>
--- a/attendees.xlsx
+++ b/attendees.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -45,8 +45,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-        <bgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00BBDEFB"/>
         <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -82,6 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -847,17 +854,17 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Salazar del Rio Alma Aurora</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Functional leader</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -1404,17 +1411,17 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Jin Seon Baek</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>ERP Manager</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>H Mart Companies, Inc.</t>
         </is>
@@ -1557,17 +1564,17 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>Paul Baraniuk</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>Global Solution…</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>Florida Crystals Corporation</t>
         </is>
@@ -2386,13 +2393,13 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t>Adam Breiterman</t>
         </is>
       </c>
-      <c r="B115" s="2" t="inlineStr"/>
-      <c r="C115" s="2" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr"/>
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>Maryland &amp; Virginia Milk Producers Cooperati…</t>
         </is>
@@ -3275,17 +3282,17 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="inlineStr">
+      <c r="A168" s="5" t="inlineStr">
         <is>
           <t>Greg Chamberland</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
+      <c r="B168" s="5" t="inlineStr">
         <is>
           <t>IT, Enterprise…</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
+      <c r="C168" s="5" t="inlineStr">
         <is>
           <t>Ocean Spray Cranberries, Inc.</t>
         </is>
@@ -3428,17 +3435,17 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+      <c r="A177" s="5" t="inlineStr">
         <is>
           <t>Abraham Cherian</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B177" s="5" t="inlineStr">
         <is>
           <t>Director Security Govern…</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C177" s="5" t="inlineStr">
         <is>
           <t>Kontoor Brands Inc</t>
         </is>
@@ -3577,34 +3584,34 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+      <c r="A186" s="5" t="inlineStr">
         <is>
           <t>Parinda Choksi</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B186" s="5" t="inlineStr">
         <is>
           <t>CIO - Enablement</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C186" s="5" t="inlineStr">
         <is>
           <t>Ball Horticultural Co.</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+      <c r="A187" s="5" t="inlineStr">
         <is>
           <t>Sanjay Choubey</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B187" s="5" t="inlineStr">
         <is>
           <t>Global Chief Digital an…</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C187" s="5" t="inlineStr">
         <is>
           <t>Sylvamo Corporation</t>
         </is>
@@ -4857,17 +4864,17 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="inlineStr">
+      <c r="A262" s="5" t="inlineStr">
         <is>
           <t>Dawn Shakeshaft</t>
         </is>
       </c>
-      <c r="B262" s="2" t="inlineStr">
+      <c r="B262" s="5" t="inlineStr">
         <is>
           <t>Controller</t>
         </is>
       </c>
-      <c r="C262" s="2" t="inlineStr">
+      <c r="C262" s="5" t="inlineStr">
         <is>
           <t>Associated Feed &amp; Supply Co.</t>
         </is>
@@ -6312,17 +6319,17 @@
       </c>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="inlineStr">
+      <c r="A349" s="5" t="inlineStr">
         <is>
           <t>Steve Tanaka</t>
         </is>
       </c>
-      <c r="B349" s="2" t="inlineStr">
+      <c r="B349" s="5" t="inlineStr">
         <is>
           <t>Sr Vice Presid…</t>
         </is>
       </c>
-      <c r="C349" s="2" t="inlineStr">
+      <c r="C349" s="5" t="inlineStr">
         <is>
           <t>Blommer Chocolate Company</t>
         </is>
@@ -7779,17 +7786,17 @@
       </c>
     </row>
     <row r="436">
-      <c r="A436" s="2" t="inlineStr">
+      <c r="A436" s="5" t="inlineStr">
         <is>
           <t>Adam Warner</t>
         </is>
       </c>
-      <c r="B436" s="2" t="inlineStr">
+      <c r="B436" s="5" t="inlineStr">
         <is>
           <t>Cost Analyst</t>
         </is>
       </c>
-      <c r="C436" s="2" t="inlineStr">
+      <c r="C436" s="5" t="inlineStr">
         <is>
           <t>Marathon Cheese Corporation</t>
         </is>
@@ -7915,17 +7922,17 @@
       </c>
     </row>
     <row r="444">
-      <c r="A444" s="2" t="inlineStr">
+      <c r="A444" s="5" t="inlineStr">
         <is>
           <t>Matt Webster</t>
         </is>
       </c>
-      <c r="B444" s="2" t="inlineStr">
+      <c r="B444" s="5" t="inlineStr">
         <is>
           <t>Director of…</t>
         </is>
       </c>
-      <c r="C444" s="2" t="inlineStr">
+      <c r="C444" s="5" t="inlineStr">
         <is>
           <t>Gardner White Furniture Co., Inc.</t>
         </is>
@@ -7949,34 +7956,34 @@
       </c>
     </row>
     <row r="446">
-      <c r="A446" s="2" t="inlineStr">
+      <c r="A446" s="5" t="inlineStr">
         <is>
           <t>Sarah Weiler</t>
         </is>
       </c>
-      <c r="B446" s="2" t="inlineStr">
+      <c r="B446" s="5" t="inlineStr">
         <is>
           <t>Manager, Busine…</t>
         </is>
       </c>
-      <c r="C446" s="2" t="inlineStr">
+      <c r="C446" s="5" t="inlineStr">
         <is>
           <t>Ball Horticultural Company</t>
         </is>
       </c>
     </row>
     <row r="447">
-      <c r="A447" s="2" t="inlineStr">
+      <c r="A447" s="5" t="inlineStr">
         <is>
           <t>Adam Werner</t>
         </is>
       </c>
-      <c r="B447" s="2" t="inlineStr">
+      <c r="B447" s="5" t="inlineStr">
         <is>
           <t>VP, Corporate Technology</t>
         </is>
       </c>
-      <c r="C447" s="2" t="inlineStr">
+      <c r="C447" s="5" t="inlineStr">
         <is>
           <t>Crocs, Inc.</t>
         </is>
@@ -8068,13 +8075,13 @@
       </c>
     </row>
     <row r="453">
-      <c r="A453" s="2" t="inlineStr">
+      <c r="A453" s="5" t="inlineStr">
         <is>
           <t>Robb White</t>
         </is>
       </c>
-      <c r="B453" s="2" t="inlineStr"/>
-      <c r="C453" s="2" t="inlineStr">
+      <c r="B453" s="5" t="inlineStr"/>
+      <c r="C453" s="5" t="inlineStr">
         <is>
           <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
         </is>
@@ -11657,17 +11664,17 @@
       </c>
     </row>
     <row r="666">
-      <c r="A666" s="2" t="inlineStr">
+      <c r="A666" s="5" t="inlineStr">
         <is>
           <t>Mark Meanwell</t>
         </is>
       </c>
-      <c r="B666" s="2" t="inlineStr">
+      <c r="B666" s="5" t="inlineStr">
         <is>
           <t>Senior Manager Data &amp; Analytics</t>
         </is>
       </c>
-      <c r="C666" s="2" t="inlineStr">
+      <c r="C666" s="5" t="inlineStr">
         <is>
           <t>Sylvamo</t>
         </is>
@@ -16330,17 +16337,17 @@
       </c>
     </row>
     <row r="943">
-      <c r="A943" s="2" t="inlineStr">
+      <c r="A943" s="5" t="inlineStr">
         <is>
           <t>Christine Graham</t>
         </is>
       </c>
-      <c r="B943" s="2" t="inlineStr">
+      <c r="B943" s="5" t="inlineStr">
         <is>
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="C943" s="2" t="inlineStr">
+      <c r="C943" s="5" t="inlineStr">
         <is>
           <t>Lakeview Farms, LLC</t>
         </is>
@@ -16649,17 +16656,17 @@
       </c>
     </row>
     <row r="962">
-      <c r="A962" s="2" t="inlineStr">
+      <c r="A962" s="5" t="inlineStr">
         <is>
           <t>Paul Harris</t>
         </is>
       </c>
-      <c r="B962" s="2" t="inlineStr">
+      <c r="B962" s="5" t="inlineStr">
         <is>
           <t>Senior Director, SAP Basi...</t>
         </is>
       </c>
-      <c r="C962" s="2" t="inlineStr">
+      <c r="C962" s="5" t="inlineStr">
         <is>
           <t>Varsity Brands, LLC.</t>
         </is>
@@ -16853,17 +16860,17 @@
       </c>
     </row>
     <row r="974">
-      <c r="A974" s="2" t="inlineStr">
+      <c r="A974" s="5" t="inlineStr">
         <is>
           <t>Adriana Hernandez</t>
         </is>
       </c>
-      <c r="B974" s="2" t="inlineStr">
+      <c r="B974" s="5" t="inlineStr">
         <is>
           <t>Head Architecture</t>
         </is>
       </c>
-      <c r="C974" s="2" t="inlineStr">
+      <c r="C974" s="5" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -17355,17 +17362,17 @@
       </c>
     </row>
     <row r="1004">
-      <c r="A1004" s="2" t="inlineStr">
+      <c r="A1004" s="5" t="inlineStr">
         <is>
           <t>Omar Hussein Olmedo</t>
         </is>
       </c>
-      <c r="B1004" s="2" t="inlineStr">
+      <c r="B1004" s="5" t="inlineStr">
         <is>
           <t>Poject Manager</t>
         </is>
       </c>
-      <c r="C1004" s="2" t="inlineStr">
+      <c r="C1004" s="5" t="inlineStr">
         <is>
           <t>Bachoco, S.A. de C.V.</t>
         </is>
@@ -18231,13 +18238,13 @@
       </c>
     </row>
     <row r="1056">
-      <c r="A1056" s="2" t="inlineStr">
+      <c r="A1056" s="5" t="inlineStr">
         <is>
           <t>Kalman Gyula</t>
         </is>
       </c>
-      <c r="B1056" s="2" t="inlineStr"/>
-      <c r="C1056" s="2" t="inlineStr">
+      <c r="B1056" s="5" t="inlineStr"/>
+      <c r="C1056" s="5" t="inlineStr">
         <is>
           <t>BSN SPORTS, LLC f/k/n Sports Supply Group,…</t>
         </is>
@@ -18414,17 +18421,17 @@
       </c>
     </row>
     <row r="1067">
-      <c r="A1067" s="2" t="inlineStr">
+      <c r="A1067" s="5" t="inlineStr">
         <is>
           <t>Jeremy Freeman</t>
         </is>
       </c>
-      <c r="B1067" s="2" t="inlineStr">
+      <c r="B1067" s="5" t="inlineStr">
         <is>
           <t>Director, Technology</t>
         </is>
       </c>
-      <c r="C1067" s="2" t="inlineStr">
+      <c r="C1067" s="5" t="inlineStr">
         <is>
           <t>Aritzia</t>
         </is>
@@ -19009,17 +19016,17 @@
       </c>
     </row>
     <row r="1102">
-      <c r="A1102" s="2" t="inlineStr">
+      <c r="A1102" s="5" t="inlineStr">
         <is>
           <t>Susana Flores Cabrera</t>
         </is>
       </c>
-      <c r="B1102" s="2" t="inlineStr">
+      <c r="B1102" s="5" t="inlineStr">
         <is>
           <t>Contracts Coordinator</t>
         </is>
       </c>
-      <c r="C1102" s="2" t="inlineStr">
+      <c r="C1102" s="5" t="inlineStr">
         <is>
           <t>Cheney Bros, Inc.</t>
         </is>
@@ -19447,17 +19454,17 @@
       </c>
     </row>
     <row r="1128">
-      <c r="A1128" s="2" t="inlineStr">
+      <c r="A1128" s="5" t="inlineStr">
         <is>
           <t>Haricharan Dingari</t>
         </is>
       </c>
-      <c r="B1128" s="2" t="inlineStr">
+      <c r="B1128" s="5" t="inlineStr">
         <is>
           <t>Enterprise Arc…</t>
         </is>
       </c>
-      <c r="C1128" s="2" t="inlineStr">
+      <c r="C1128" s="5" t="inlineStr">
         <is>
           <t>Bob's Discount Furniture, LLC</t>
         </is>
@@ -19702,17 +19709,17 @@
       </c>
     </row>
     <row r="1143">
-      <c r="A1143" s="2" t="inlineStr">
+      <c r="A1143" s="5" t="inlineStr">
         <is>
           <t>Damodhar Dyava</t>
         </is>
       </c>
-      <c r="B1143" s="2" t="inlineStr">
+      <c r="B1143" s="5" t="inlineStr">
         <is>
           <t>SAP SD Manag…</t>
         </is>
       </c>
-      <c r="C1143" s="2" t="inlineStr">
+      <c r="C1143" s="5" t="inlineStr">
         <is>
           <t>Bob's Discount Furniture, LLC</t>
         </is>

</xml_diff>